<commit_message>
added all updated files
</commit_message>
<xml_diff>
--- a/SUMMARY.xlsx
+++ b/SUMMARY.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amartyn/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amartyn/MPIPZ/amartyn/CSSP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F367EF8-400C-5B45-9102-0FA297C4E562}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{970F8E47-2383-484E-AE29-A96041933F9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" xr2:uid="{3CB25A69-F844-9241-B587-A0F2F035342F}"/>
+    <workbookView xWindow="5380" yWindow="6460" windowWidth="27420" windowHeight="19640" xr2:uid="{3CB25A69-F844-9241-B587-A0F2F035342F}"/>
   </bookViews>
   <sheets>
     <sheet name="summary" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="74">
   <si>
     <t>A</t>
   </si>
@@ -139,9 +139,6 @@
     <t>Nodule ASVs</t>
   </si>
   <si>
-    <t>WT V2</t>
-  </si>
-  <si>
     <t>CSSP</t>
   </si>
   <si>
@@ -208,9 +205,6 @@
     <t>ROOT EXUDATES</t>
   </si>
   <si>
-    <t>(Simona's suggestion)</t>
-  </si>
-  <si>
     <t>pca</t>
   </si>
   <si>
@@ -260,6 +254,9 @@
   </si>
   <si>
     <t>(incl. taxonomy, v5v7 sequences, grouping)</t>
+  </si>
+  <si>
+    <t>X</t>
   </si>
 </sst>
 </file>
@@ -298,7 +295,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -341,6 +338,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="11">
     <border>
@@ -460,7 +463,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -473,7 +476,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
@@ -481,10 +483,13 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -799,7 +804,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71DAC3A5-AA30-0140-ACA0-23B73C5BF466}">
-  <dimension ref="A1:K66"/>
+  <dimension ref="A1:L58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.6640625" customWidth="1"/>
@@ -810,27 +815,27 @@
     <col min="11" max="11" width="82.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="21" customFormat="1" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="19" t="s">
+    <row r="1" spans="1:12" s="19" customFormat="1" ht="21" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="19"/>
+      <c r="B1" s="18"/>
       <c r="C1" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D1" s="20"/>
       <c r="E1" s="20"/>
-      <c r="F1" s="19"/>
+      <c r="F1" s="18"/>
       <c r="G1" s="20" t="s">
         <v>15</v>
       </c>
       <c r="H1" s="20"/>
       <c r="J1" s="20" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="K1" s="20"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
@@ -843,64 +848,85 @@
       <c r="E3" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="J3" s="17">
+      <c r="F3" t="s">
+        <v>73</v>
+      </c>
+      <c r="J3" s="16">
         <v>1</v>
       </c>
-      <c r="K3" s="18" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K3" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="L3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
       <c r="C4" s="11"/>
-      <c r="D4" s="12" t="s">
+      <c r="D4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" s="12" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="F4" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="2"/>
       <c r="C5" s="11"/>
-      <c r="D5" s="12" t="s">
+      <c r="D5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="E5" s="12" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="F5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
       <c r="C6" s="11"/>
-      <c r="D6" s="12" t="s">
+      <c r="D6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="21" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="F6" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="2"/>
       <c r="C7" s="11"/>
-      <c r="D7" s="12" t="s">
+      <c r="D7" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="E7" s="12" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="F7" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="2"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="15" t="s">
+      <c r="C8" s="13"/>
+      <c r="D8" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="16" t="s">
+      <c r="E8" s="15" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="F8" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>26</v>
       </c>
@@ -913,525 +939,493 @@
       <c r="E10" s="10" t="s">
         <v>1</v>
       </c>
+      <c r="F10" t="s">
+        <v>73</v>
+      </c>
       <c r="G10" s="8">
         <v>1</v>
       </c>
       <c r="H10" s="10" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="I10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" s="3"/>
       <c r="C11" s="11"/>
-      <c r="D11" s="12" t="s">
+      <c r="D11" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="E11" s="12" t="s">
         <v>27</v>
       </c>
+      <c r="F11" t="s">
+        <v>73</v>
+      </c>
       <c r="G11" s="11"/>
-      <c r="H11" s="13" t="s">
+      <c r="H11" s="12" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="I11" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" s="3"/>
       <c r="C12" s="11"/>
-      <c r="D12" s="12" t="s">
+      <c r="D12" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E12" s="13" t="s">
+      <c r="E12" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="G12" s="14"/>
-      <c r="H12" s="16" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="F12" t="s">
+        <v>73</v>
+      </c>
+      <c r="G12" s="11"/>
+      <c r="H12" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="I12" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" s="3"/>
       <c r="C13" s="11"/>
-      <c r="D13" s="12" t="s">
+      <c r="D13" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E13" s="13" t="s">
+      <c r="E13" s="12" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="F13" t="s">
+        <v>73</v>
+      </c>
+      <c r="G13" s="13"/>
+      <c r="H13" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="I13" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="3"/>
-      <c r="C14" s="11"/>
-      <c r="D14" s="12" t="s">
+      <c r="C14" s="13"/>
+      <c r="D14" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="E14" s="13" t="s">
+      <c r="E14" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="F14" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="D15" s="1"/>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A16" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" s="8">
+        <v>3</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="F16" t="s">
+        <v>73</v>
+      </c>
+      <c r="G16" s="8">
+        <v>2</v>
+      </c>
+      <c r="H16" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="I16" t="s">
+        <v>73</v>
+      </c>
+      <c r="J16" s="16">
+        <v>2</v>
+      </c>
+      <c r="K16" s="17" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A17" s="4"/>
+      <c r="C17" s="11"/>
+      <c r="D17" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E17" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="F17" t="s">
+        <v>73</v>
+      </c>
+      <c r="G17" s="13"/>
+      <c r="H17" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="I17" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A18" s="4"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E18" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="F18" t="s">
+        <v>73</v>
+      </c>
+      <c r="G18" s="1"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A19" s="4"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="E19" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="G19" s="8">
+        <v>3</v>
+      </c>
+      <c r="H19" s="22" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A15" s="3"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="E15" s="16" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A18" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="C18" s="8">
+      <c r="I19" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A20" s="4"/>
+      <c r="D20" s="1"/>
+      <c r="G20" s="13"/>
+      <c r="H20" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="I20" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A22" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C22" s="8">
+        <v>4</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="E22" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="J22" s="16">
+        <v>3</v>
+      </c>
+      <c r="K22" s="17" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A23" s="6"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D18" s="9" t="s">
+      <c r="E23" s="12" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A24" s="6"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E24" s="12" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A25" s="6"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="E25" s="23" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A27" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C27" s="8">
+        <v>5</v>
+      </c>
+      <c r="D27" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="E18" s="10" t="s">
+      <c r="E27" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="G18" s="8">
-        <v>1</v>
-      </c>
-      <c r="H18" s="10" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A19" s="3" t="s">
+      <c r="G27" s="8">
+        <v>4</v>
+      </c>
+      <c r="H27" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="J27" s="16">
+        <v>4</v>
+      </c>
+      <c r="K27" s="17" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A28" s="5"/>
+      <c r="C28" s="11"/>
+      <c r="D28" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E28" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="G28" s="11"/>
+      <c r="H28" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="J28" s="1"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A29" s="5"/>
+      <c r="C29" s="11"/>
+      <c r="D29" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E29" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="G29" s="11"/>
+      <c r="H29" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="J29" s="16">
+        <v>5</v>
+      </c>
+      <c r="K29" s="17" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A30" s="5"/>
+      <c r="C30" s="11"/>
+      <c r="D30" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E30" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="G30" s="11"/>
+      <c r="H30" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="J30" s="1"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A31" s="5"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="E31" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="G31" s="13"/>
+      <c r="H31" s="15" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A33" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="C33" s="8">
+        <v>6</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="E33" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="G33" s="16">
+        <v>5</v>
+      </c>
+      <c r="H33" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="J33" s="16">
+        <v>6</v>
+      </c>
+      <c r="K33" s="17" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A34" s="7"/>
+      <c r="C34" s="11"/>
+      <c r="D34" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E34" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="C19" s="11"/>
-      <c r="D19" s="12" t="s">
-        <v>2</v>
-      </c>
-      <c r="E19" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="G19" s="11"/>
-      <c r="H19" s="13" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A20" s="3"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="12" t="s">
+      <c r="J34" s="1"/>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A35" s="7"/>
+      <c r="C35" s="11"/>
+      <c r="D35" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E20" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="G20" s="11"/>
-      <c r="H20" s="13" t="s">
+      <c r="E35" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="J35" s="16">
         <v>7</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A21" s="3"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="12" t="s">
+      <c r="K35" s="17" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A36" s="7"/>
+      <c r="C36" s="13"/>
+      <c r="D36" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="E21" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="G21" s="14"/>
-      <c r="H21" s="16" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A22" s="3"/>
-      <c r="C22" s="14"/>
-      <c r="D22" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="E22" s="16" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="D23" s="1"/>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A24" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C24" s="8">
-        <v>3</v>
-      </c>
-      <c r="D24" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="E24" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="G24" s="8">
-        <v>2</v>
-      </c>
-      <c r="H24" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="J24" s="17">
-        <v>2</v>
-      </c>
-      <c r="K24" s="18" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A25" s="4"/>
-      <c r="C25" s="11"/>
-      <c r="D25" s="12" t="s">
-        <v>2</v>
-      </c>
-      <c r="E25" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="G25" s="14"/>
-      <c r="H25" s="16" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A26" s="4"/>
-      <c r="C26" s="11"/>
-      <c r="D26" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="E26" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="G26" s="1"/>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A27" s="4"/>
-      <c r="C27" s="14"/>
-      <c r="D27" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E27" s="16" t="s">
-        <v>39</v>
-      </c>
-      <c r="G27" s="8">
-        <v>3</v>
-      </c>
-      <c r="H27" s="10" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A28" s="4"/>
-      <c r="D28" s="1"/>
-      <c r="G28" s="14"/>
-      <c r="H28" s="16" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A30" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C30" s="8">
-        <v>4</v>
-      </c>
-      <c r="D30" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="E30" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="J30" s="17">
-        <v>3</v>
-      </c>
-      <c r="K30" s="18" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A31" s="6"/>
-      <c r="C31" s="11"/>
-      <c r="D31" s="12" t="s">
-        <v>2</v>
-      </c>
-      <c r="E31" s="13" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A32" s="6"/>
-      <c r="C32" s="11"/>
-      <c r="D32" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="E32" s="13" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A33" s="6"/>
-      <c r="C33" s="14"/>
-      <c r="D33" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E33" s="16" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A35" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="C35" s="8">
-        <v>5</v>
-      </c>
-      <c r="D35" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="E35" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="G35" s="8">
-        <v>4</v>
-      </c>
-      <c r="H35" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="J35" s="17">
-        <v>4</v>
-      </c>
-      <c r="K35" s="18" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A36" s="5"/>
-      <c r="C36" s="11"/>
-      <c r="D36" s="12" t="s">
-        <v>2</v>
-      </c>
-      <c r="E36" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="G36" s="11"/>
-      <c r="H36" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="J36" s="1"/>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A37" s="5"/>
-      <c r="C37" s="11"/>
-      <c r="D37" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="E37" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="G37" s="11"/>
-      <c r="H37" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="J37" s="17">
-        <v>5</v>
-      </c>
-      <c r="K37" s="18" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A38" s="5"/>
-      <c r="C38" s="11"/>
-      <c r="D38" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="E38" s="13" t="s">
-        <v>9</v>
-      </c>
-      <c r="G38" s="11"/>
-      <c r="H38" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="J38" s="1"/>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A39" s="5"/>
-      <c r="C39" s="14"/>
-      <c r="D39" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="E39" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="G39" s="14"/>
-      <c r="H39" s="16" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A41" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="C41" s="8">
-        <v>6</v>
-      </c>
-      <c r="D41" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="E41" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="G41" s="17">
-        <v>5</v>
-      </c>
-      <c r="H41" s="18" t="s">
-        <v>62</v>
-      </c>
-      <c r="J41" s="17">
-        <v>6</v>
-      </c>
-      <c r="K41" s="18" t="s">
+      <c r="E36" s="15" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="21" x14ac:dyDescent="0.25">
+      <c r="A40" s="18" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A42" s="7"/>
-      <c r="C42" s="11"/>
-      <c r="D42" s="12" t="s">
-        <v>2</v>
-      </c>
-      <c r="E42" s="13" t="s">
-        <v>59</v>
-      </c>
-      <c r="J42" s="1"/>
+      <c r="A42" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A43" s="7"/>
-      <c r="C43" s="11"/>
-      <c r="D43" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="E43" s="13" t="s">
-        <v>60</v>
-      </c>
-      <c r="J43" s="17">
-        <v>7</v>
-      </c>
-      <c r="K43" s="18" t="s">
+      <c r="B43" t="s">
+        <v>17</v>
+      </c>
+      <c r="F43" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A44" s="7"/>
-      <c r="C44" s="14"/>
-      <c r="D44" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E44" s="16" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" ht="21" x14ac:dyDescent="0.25">
-      <c r="A48" s="19" t="s">
+      <c r="B44" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B45" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B46" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B47" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A48" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F48" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A50" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="G48" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A49" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="F49" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A50" s="1"/>
+      <c r="B50" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B51" t="s">
-        <v>17</v>
-      </c>
-      <c r="F51" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B52" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B53" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B54" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B55" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A56" s="1" t="s">
-        <v>22</v>
+        <v>69</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A55" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B56" t="s">
+        <v>24</v>
       </c>
       <c r="F56" t="s">
-        <v>67</v>
-      </c>
-      <c r="G56" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A57" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="F57" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A58" s="1"/>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B57" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="B58" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B59" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B60" t="s">
         <v>72</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B61" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A63" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B64" t="s">
-        <v>24</v>
-      </c>
-      <c r="F64" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="65" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B65" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="66" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B66" t="s">
-        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added new to do list
</commit_message>
<xml_diff>
--- a/SUMMARY.xlsx
+++ b/SUMMARY.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amartyn/MPIPZ/amartyn/CSSP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{970F8E47-2383-484E-AE29-A96041933F9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71204097-CDDC-7B49-93E1-80A2CC7265CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5380" yWindow="6460" windowWidth="27420" windowHeight="19640" xr2:uid="{3CB25A69-F844-9241-B587-A0F2F035342F}"/>
+    <workbookView xWindow="5380" yWindow="600" windowWidth="29120" windowHeight="19640" xr2:uid="{3CB25A69-F844-9241-B587-A0F2F035342F}"/>
   </bookViews>
   <sheets>
     <sheet name="summary" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="80">
   <si>
     <t>A</t>
   </si>
@@ -257,6 +257,24 @@
   </si>
   <si>
     <t>X</t>
+  </si>
+  <si>
+    <t>soil - bulk</t>
+  </si>
+  <si>
+    <t>soil - WT</t>
+  </si>
+  <si>
+    <t>soil - CSSP</t>
+  </si>
+  <si>
+    <t>soil - prediction</t>
+  </si>
+  <si>
+    <t>syncoms</t>
+  </si>
+  <si>
+    <t>root exudates</t>
   </si>
 </sst>
 </file>
@@ -484,12 +502,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -804,635 +822,655 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71DAC3A5-AA30-0140-ACA0-23B73C5BF466}">
-  <dimension ref="A1:L58"/>
+  <dimension ref="A1:M58"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.6640625" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.1640625" customWidth="1"/>
-    <col min="8" max="8" width="44.83203125" customWidth="1"/>
-    <col min="10" max="10" width="10.83203125" customWidth="1"/>
-    <col min="11" max="11" width="82.5" customWidth="1"/>
+    <col min="3" max="3" width="14.5" customWidth="1"/>
+    <col min="6" max="6" width="22.1640625" customWidth="1"/>
+    <col min="9" max="9" width="44.83203125" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" customWidth="1"/>
+    <col min="12" max="12" width="82.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="19" customFormat="1" ht="21" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" s="19" customFormat="1" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="18" t="s">
         <v>13</v>
       </c>
       <c r="B1" s="18"/>
-      <c r="C1" s="20" t="s">
+      <c r="C1" s="18"/>
+      <c r="D1" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="20" t="s">
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="H1" s="20"/>
-      <c r="J1" s="20" t="s">
+      <c r="I1" s="23"/>
+      <c r="K1" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="K1" s="20"/>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="L1" s="23"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" t="s">
+        <v>74</v>
+      </c>
+      <c r="D3" s="8">
         <v>1</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="E3" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="F3" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="F3" t="s">
-        <v>73</v>
-      </c>
-      <c r="J3" s="16">
+      <c r="G3" t="s">
+        <v>73</v>
+      </c>
+      <c r="K3" s="16">
         <v>1</v>
       </c>
-      <c r="K3" s="17" t="s">
+      <c r="L3" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="L3" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
-      <c r="C4" s="11"/>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="11"/>
+      <c r="E4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="12" t="s">
+      <c r="F4" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="F4" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="G4" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="2"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="11"/>
+      <c r="E5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="12" t="s">
+      <c r="F5" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="F5" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="G5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="11"/>
+      <c r="E6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="21" t="s">
+      <c r="F6" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="F6" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="G6" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="2"/>
-      <c r="C7" s="11"/>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="11"/>
+      <c r="E7" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="12" t="s">
+      <c r="F7" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="F7" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="G7" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="2"/>
-      <c r="C8" s="13"/>
-      <c r="D8" s="14" t="s">
+      <c r="D8" s="13"/>
+      <c r="E8" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="E8" s="15" t="s">
+      <c r="F8" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="F8" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="G8" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C10" t="s">
+        <v>75</v>
+      </c>
+      <c r="D10" s="8">
         <v>2</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="E10" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="F10" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="F10" t="s">
-        <v>73</v>
-      </c>
-      <c r="G10" s="8">
+      <c r="G10" t="s">
+        <v>73</v>
+      </c>
+      <c r="H10" s="8">
         <v>1</v>
       </c>
-      <c r="H10" s="10" t="s">
+      <c r="I10" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="I10" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="J10" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="3"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="1" t="s">
+      <c r="D11" s="11"/>
+      <c r="E11" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E11" s="12" t="s">
+      <c r="F11" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="F11" t="s">
-        <v>73</v>
-      </c>
-      <c r="G11" s="11"/>
-      <c r="H11" s="12" t="s">
+      <c r="G11" t="s">
+        <v>73</v>
+      </c>
+      <c r="H11" s="11"/>
+      <c r="I11" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="I11" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="J11" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="3"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="1" t="s">
+      <c r="D12" s="11"/>
+      <c r="E12" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E12" s="12" t="s">
+      <c r="F12" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="F12" t="s">
-        <v>73</v>
-      </c>
-      <c r="G12" s="11"/>
-      <c r="H12" s="21" t="s">
+      <c r="G12" t="s">
+        <v>73</v>
+      </c>
+      <c r="H12" s="11"/>
+      <c r="I12" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="I12" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="J12" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="3"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="1" t="s">
+      <c r="D13" s="11"/>
+      <c r="E13" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E13" s="12" t="s">
+      <c r="F13" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="F13" t="s">
-        <v>73</v>
-      </c>
-      <c r="G13" s="13"/>
-      <c r="H13" s="15" t="s">
+      <c r="G13" t="s">
+        <v>73</v>
+      </c>
+      <c r="H13" s="13"/>
+      <c r="I13" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="I13" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="J13" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="3"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="14" t="s">
+      <c r="D14" s="13"/>
+      <c r="E14" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="E14" s="15" t="s">
+      <c r="F14" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="F14" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="D15" s="1"/>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="G14" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="E15" s="1"/>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C16" s="8">
+      <c r="C16" t="s">
+        <v>76</v>
+      </c>
+      <c r="D16" s="8">
         <v>3</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="E16" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="E16" s="10" t="s">
+      <c r="F16" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="F16" t="s">
-        <v>73</v>
-      </c>
-      <c r="G16" s="8">
+      <c r="G16" t="s">
+        <v>73</v>
+      </c>
+      <c r="H16" s="8">
         <v>2</v>
       </c>
-      <c r="H16" s="10" t="s">
+      <c r="I16" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="I16" t="s">
-        <v>73</v>
-      </c>
-      <c r="J16" s="16">
+      <c r="J16" t="s">
+        <v>73</v>
+      </c>
+      <c r="K16" s="16">
         <v>2</v>
       </c>
-      <c r="K16" s="17" t="s">
+      <c r="L16" s="17" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" s="4"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="1" t="s">
+      <c r="D17" s="11"/>
+      <c r="E17" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E17" s="12" t="s">
+      <c r="F17" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="F17" t="s">
-        <v>73</v>
-      </c>
-      <c r="G17" s="13"/>
-      <c r="H17" s="15" t="s">
+      <c r="G17" t="s">
+        <v>73</v>
+      </c>
+      <c r="H17" s="13"/>
+      <c r="I17" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="I17" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J17" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" s="4"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="1" t="s">
+      <c r="D18" s="11"/>
+      <c r="E18" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E18" s="12" t="s">
+      <c r="F18" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="F18" t="s">
-        <v>73</v>
-      </c>
-      <c r="G18" s="1"/>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="G18" t="s">
+        <v>73</v>
+      </c>
+      <c r="H18" s="1"/>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" s="4"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="14" t="s">
+      <c r="D19" s="13"/>
+      <c r="E19" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="E19" s="15" t="s">
+      <c r="F19" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="G19" s="8">
+      <c r="H19" s="8">
         <v>3</v>
       </c>
-      <c r="H19" s="22" t="s">
+      <c r="I19" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="I19" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J19" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" s="4"/>
-      <c r="D20" s="1"/>
-      <c r="G20" s="13"/>
-      <c r="H20" s="15" t="s">
+      <c r="E20" s="1"/>
+      <c r="H20" s="13"/>
+      <c r="I20" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="I20" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="J20" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A22" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C22" s="8">
+      <c r="C22" t="s">
+        <v>77</v>
+      </c>
+      <c r="D22" s="8">
         <v>4</v>
       </c>
-      <c r="D22" s="9" t="s">
+      <c r="E22" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="E22" s="10" t="s">
+      <c r="F22" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="J22" s="16">
+      <c r="K22" s="16">
         <v>3</v>
       </c>
-      <c r="K22" s="17" t="s">
+      <c r="L22" s="17" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" s="6"/>
-      <c r="C23" s="11"/>
-      <c r="D23" s="1" t="s">
+      <c r="D23" s="11"/>
+      <c r="E23" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E23" s="12" t="s">
+      <c r="F23" s="12" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A24" s="6"/>
-      <c r="C24" s="11"/>
-      <c r="D24" s="1" t="s">
+      <c r="D24" s="11"/>
+      <c r="E24" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E24" s="12" t="s">
+      <c r="F24" s="12" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="6"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="14" t="s">
+      <c r="D25" s="13"/>
+      <c r="E25" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="E25" s="23" t="s">
+      <c r="F25" s="22" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A27" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C27" s="8">
+      <c r="C27" t="s">
+        <v>78</v>
+      </c>
+      <c r="D27" s="8">
         <v>5</v>
       </c>
-      <c r="D27" s="9" t="s">
+      <c r="E27" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="E27" s="10" t="s">
+      <c r="F27" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="G27" s="8">
+      <c r="H27" s="8">
         <v>4</v>
       </c>
-      <c r="H27" s="10" t="s">
+      <c r="I27" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="J27" s="16">
+      <c r="K27" s="16">
         <v>4</v>
       </c>
-      <c r="K27" s="17" t="s">
+      <c r="L27" s="17" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A28" s="5"/>
-      <c r="C28" s="11"/>
-      <c r="D28" s="1" t="s">
+      <c r="D28" s="11"/>
+      <c r="E28" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E28" s="12" t="s">
+      <c r="F28" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="G28" s="11"/>
-      <c r="H28" s="12" t="s">
+      <c r="H28" s="11"/>
+      <c r="I28" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="J28" s="1"/>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K28" s="1"/>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A29" s="5"/>
-      <c r="C29" s="11"/>
-      <c r="D29" s="1" t="s">
+      <c r="D29" s="11"/>
+      <c r="E29" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E29" s="12" t="s">
+      <c r="F29" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="G29" s="11"/>
-      <c r="H29" s="21" t="s">
+      <c r="H29" s="11"/>
+      <c r="I29" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="J29" s="16">
+      <c r="K29" s="16">
         <v>5</v>
       </c>
-      <c r="K29" s="17" t="s">
+      <c r="L29" s="17" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A30" s="5"/>
-      <c r="C30" s="11"/>
-      <c r="D30" s="1" t="s">
+      <c r="D30" s="11"/>
+      <c r="E30" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E30" s="12" t="s">
+      <c r="F30" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="G30" s="11"/>
-      <c r="H30" s="12" t="s">
+      <c r="H30" s="11"/>
+      <c r="I30" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="J30" s="1"/>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K30" s="1"/>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A31" s="5"/>
-      <c r="C31" s="13"/>
-      <c r="D31" s="14" t="s">
+      <c r="D31" s="13"/>
+      <c r="E31" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="E31" s="15" t="s">
+      <c r="F31" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="G31" s="13"/>
-      <c r="H31" s="15" t="s">
+      <c r="H31" s="13"/>
+      <c r="I31" s="15" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A33" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="C33" s="8">
+      <c r="C33" t="s">
+        <v>79</v>
+      </c>
+      <c r="D33" s="8">
         <v>6</v>
       </c>
-      <c r="D33" s="9" t="s">
+      <c r="E33" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="E33" s="10" t="s">
+      <c r="F33" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="G33" s="16">
+      <c r="H33" s="16">
         <v>5</v>
       </c>
-      <c r="H33" s="17" t="s">
+      <c r="I33" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="J33" s="16">
+      <c r="K33" s="16">
         <v>6</v>
       </c>
-      <c r="K33" s="17" t="s">
+      <c r="L33" s="17" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A34" s="7"/>
-      <c r="C34" s="11"/>
-      <c r="D34" s="1" t="s">
+      <c r="D34" s="11"/>
+      <c r="E34" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E34" s="12" t="s">
+      <c r="F34" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="J34" s="1"/>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="K34" s="1"/>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A35" s="7"/>
-      <c r="C35" s="11"/>
-      <c r="D35" s="1" t="s">
+      <c r="D35" s="11"/>
+      <c r="E35" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E35" s="12" t="s">
+      <c r="F35" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="J35" s="16">
+      <c r="K35" s="16">
         <v>7</v>
       </c>
-      <c r="K35" s="17" t="s">
+      <c r="L35" s="17" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A36" s="7"/>
-      <c r="C36" s="13"/>
-      <c r="D36" s="14" t="s">
+      <c r="D36" s="13"/>
+      <c r="E36" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="E36" s="15" t="s">
+      <c r="F36" s="15" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="40" spans="1:11" ht="21" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:12" ht="21" x14ac:dyDescent="0.25">
       <c r="A40" s="18" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B43" t="s">
         <v>17</v>
       </c>
-      <c r="F43" t="s">
+      <c r="G43" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B44" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B45" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B46" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B47" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="F48" t="s">
+      <c r="G48" t="s">
         <v>65</v>
       </c>
-      <c r="G48" t="s">
+      <c r="H48" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="F49" t="s">
+      <c r="G49" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A50" s="1"/>
       <c r="B50" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B51" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B52" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B53" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B56" t="s">
         <v>24</v>
       </c>
-      <c r="F56" t="s">
+      <c r="G56" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B57" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B58" t="s">
         <v>72</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="J1:K1"/>
+    <mergeCell ref="D1:F1"/>
+    <mergeCell ref="H1:I1"/>
+    <mergeCell ref="K1:L1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
added all new files and new draft
</commit_message>
<xml_diff>
--- a/SUMMARY.xlsx
+++ b/SUMMARY.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amartyn/MPIPZ/amartyn/CSSP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71204097-CDDC-7B49-93E1-80A2CC7265CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FD7BD64-17A7-4545-8927-9EA87AE74B80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5380" yWindow="600" windowWidth="29120" windowHeight="19640" xr2:uid="{3CB25A69-F844-9241-B587-A0F2F035342F}"/>
+    <workbookView xWindow="4060" yWindow="500" windowWidth="30840" windowHeight="19640" xr2:uid="{3CB25A69-F844-9241-B587-A0F2F035342F}"/>
   </bookViews>
   <sheets>
     <sheet name="summary" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="84">
   <si>
     <t>A</t>
   </si>
@@ -79,12 +79,6 @@
     <t>Section</t>
   </si>
   <si>
-    <t>Main Figure</t>
-  </si>
-  <si>
-    <t>Supplementary Figure</t>
-  </si>
-  <si>
     <t>Raw data</t>
   </si>
   <si>
@@ -275,6 +269,24 @@
   </si>
   <si>
     <t>root exudates</t>
+  </si>
+  <si>
+    <t>nodule cts WT vs mutants</t>
+  </si>
+  <si>
+    <t>shoot fw axenic conditions (ctrls)</t>
+  </si>
+  <si>
+    <t>stacked bp detected features and pw info</t>
+  </si>
+  <si>
+    <t>XX</t>
+  </si>
+  <si>
+    <t>Main Figures</t>
+  </si>
+  <si>
+    <t>Supplementary Figures</t>
   </si>
 </sst>
 </file>
@@ -481,7 +493,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -508,6 +520,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -822,12 +835,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71DAC3A5-AA30-0140-ACA0-23B73C5BF466}">
-  <dimension ref="A1:M58"/>
+  <dimension ref="A1:M60"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.6640625" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="14.5" customWidth="1"/>
+    <col min="2" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" customWidth="1"/>
+    <col min="4" max="4" width="17.5" customWidth="1"/>
     <col min="6" max="6" width="22.1640625" customWidth="1"/>
     <col min="9" max="9" width="44.83203125" customWidth="1"/>
     <col min="11" max="11" width="10.83203125" customWidth="1"/>
@@ -841,17 +855,17 @@
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
       <c r="D1" s="23" t="s">
-        <v>14</v>
+        <v>82</v>
       </c>
       <c r="E1" s="23"/>
       <c r="F1" s="23"/>
       <c r="G1" s="18"/>
       <c r="H1" s="23" t="s">
-        <v>15</v>
+        <v>83</v>
       </c>
       <c r="I1" s="23"/>
       <c r="K1" s="23" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="L1" s="23"/>
     </row>
@@ -860,7 +874,7 @@
         <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D3" s="8">
         <v>1</v>
@@ -871,17 +885,17 @@
       <c r="F3" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="G3" t="s">
-        <v>73</v>
+      <c r="G3" s="1" t="s">
+        <v>81</v>
       </c>
       <c r="K3" s="16">
         <v>1</v>
       </c>
       <c r="L3" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="M3" t="s">
-        <v>73</v>
+        <v>42</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.2">
@@ -893,8 +907,8 @@
       <c r="F4" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="G4" t="s">
-        <v>73</v>
+      <c r="G4" s="1" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
@@ -906,8 +920,8 @@
       <c r="F5" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G5" t="s">
-        <v>73</v>
+      <c r="G5" s="1" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
@@ -919,8 +933,8 @@
       <c r="F6" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="G6" t="s">
-        <v>73</v>
+      <c r="G6" s="1" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
@@ -932,8 +946,8 @@
       <c r="F7" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="G7" t="s">
-        <v>73</v>
+      <c r="G7" s="1" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
@@ -945,16 +959,16 @@
       <c r="F8" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="G8" t="s">
-        <v>73</v>
+      <c r="G8" s="1" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C10" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D10" s="8">
         <v>2</v>
@@ -965,17 +979,17 @@
       <c r="F10" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="G10" t="s">
-        <v>73</v>
+      <c r="G10" s="1" t="s">
+        <v>81</v>
       </c>
       <c r="H10" s="8">
         <v>1</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="J10" t="s">
-        <v>73</v>
+        <v>29</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
@@ -985,17 +999,17 @@
         <v>2</v>
       </c>
       <c r="F11" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="G11" t="s">
-        <v>73</v>
+        <v>25</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>81</v>
       </c>
       <c r="H11" s="11"/>
       <c r="I11" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="J11" t="s">
-        <v>73</v>
+        <v>30</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
@@ -1005,17 +1019,17 @@
         <v>4</v>
       </c>
       <c r="F12" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="G12" t="s">
-        <v>73</v>
+        <v>26</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>81</v>
       </c>
       <c r="H12" s="11"/>
       <c r="I12" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="J12" t="s">
-        <v>73</v>
+      <c r="J12" s="1" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
@@ -1025,17 +1039,17 @@
         <v>6</v>
       </c>
       <c r="F13" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="G13" t="s">
-        <v>73</v>
+        <v>27</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>81</v>
       </c>
       <c r="H13" s="13"/>
       <c r="I13" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="J13" t="s">
-        <v>73</v>
+        <v>31</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
@@ -1045,21 +1059,18 @@
         <v>8</v>
       </c>
       <c r="F14" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="G14" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="E15" s="1"/>
+        <v>28</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A16" s="4" t="s">
-        <v>34</v>
+      <c r="A16" s="6" t="s">
+        <v>37</v>
       </c>
       <c r="C16" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D16" s="8">
         <v>3</v>
@@ -1068,402 +1079,453 @@
         <v>0</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="G16" t="s">
-        <v>73</v>
-      </c>
-      <c r="H16" s="8">
-        <v>2</v>
-      </c>
-      <c r="I16" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="J16" t="s">
-        <v>73</v>
+        <v>38</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>81</v>
       </c>
       <c r="K16" s="16">
         <v>2</v>
       </c>
       <c r="L16" s="17" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A17" s="4"/>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A17" s="6"/>
       <c r="D17" s="11"/>
       <c r="E17" s="1" t="s">
         <v>2</v>
       </c>
       <c r="F17" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="G17" t="s">
-        <v>73</v>
-      </c>
-      <c r="H17" s="13"/>
-      <c r="I17" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="J17" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A18" s="4"/>
+        <v>40</v>
+      </c>
+      <c r="G17" s="24" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A18" s="6"/>
       <c r="D18" s="11"/>
       <c r="E18" s="1" t="s">
         <v>4</v>
       </c>
       <c r="F18" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="G18" t="s">
-        <v>73</v>
-      </c>
-      <c r="H18" s="1"/>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A19" s="4"/>
+        <v>39</v>
+      </c>
+      <c r="G18" s="24" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A19" s="6"/>
       <c r="D19" s="13"/>
       <c r="E19" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="F19" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="H19" s="8">
+      <c r="F19" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="G19" s="24" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="E20" s="1"/>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A21" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C21" t="s">
+        <v>74</v>
+      </c>
+      <c r="D21" s="8">
+        <v>4</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="F21" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="H21" s="8">
+        <v>2</v>
+      </c>
+      <c r="I21" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="J21" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="K21" s="16">
         <v>3</v>
       </c>
-      <c r="I19" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="J19" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A20" s="4"/>
-      <c r="E20" s="1"/>
-      <c r="H20" s="13"/>
-      <c r="I20" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="J20" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A22" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C22" t="s">
-        <v>77</v>
-      </c>
-      <c r="D22" s="8">
-        <v>4</v>
-      </c>
-      <c r="E22" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="F22" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="K22" s="16">
-        <v>3</v>
-      </c>
-      <c r="L22" s="17" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A23" s="6"/>
+      <c r="L21" s="17" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A22" s="4"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F22" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="H22" s="13"/>
+      <c r="I22" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A23" s="4"/>
       <c r="D23" s="11"/>
       <c r="E23" s="1" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F23" s="12" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A24" s="6"/>
-      <c r="D24" s="11"/>
-      <c r="E24" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F24" s="12" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A25" s="6"/>
-      <c r="D25" s="13"/>
-      <c r="E25" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="H23" s="1"/>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A24" s="4"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="F25" s="22" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A27" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="C27" t="s">
-        <v>78</v>
-      </c>
-      <c r="D27" s="8">
-        <v>5</v>
-      </c>
-      <c r="E27" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="F27" s="10" t="s">
-        <v>1</v>
-      </c>
+      <c r="F24" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="G24" t="s">
+        <v>71</v>
+      </c>
+      <c r="H24" s="8">
+        <v>3</v>
+      </c>
+      <c r="I24" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A25" s="4"/>
+      <c r="E25" s="1"/>
+      <c r="H25" s="13"/>
+      <c r="I25" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="J25" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="H26" s="1"/>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="H27" s="8">
         <v>4</v>
       </c>
-      <c r="I27" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="K27" s="16">
+      <c r="I27" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="J27" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="H28" s="13"/>
+      <c r="I28" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A30" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="C30" t="s">
+        <v>77</v>
+      </c>
+      <c r="D30" s="8">
+        <v>5</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="F30" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="H30" s="8">
+        <v>5</v>
+      </c>
+      <c r="I30" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="K30" s="16">
         <v>4</v>
       </c>
-      <c r="L27" s="17" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A28" s="5"/>
-      <c r="D28" s="11"/>
-      <c r="E28" s="1" t="s">
+      <c r="L30" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="M30" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A31" s="7"/>
+      <c r="D31" s="11"/>
+      <c r="E31" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F28" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="H28" s="11"/>
-      <c r="I28" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="K28" s="1"/>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A29" s="5"/>
-      <c r="D29" s="11"/>
-      <c r="E29" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F29" s="12" t="s">
-        <v>47</v>
-      </c>
-      <c r="H29" s="11"/>
-      <c r="I29" s="20" t="s">
-        <v>49</v>
-      </c>
-      <c r="K29" s="16">
-        <v>5</v>
-      </c>
-      <c r="L29" s="17" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A30" s="5"/>
-      <c r="D30" s="11"/>
-      <c r="E30" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F30" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="H30" s="11"/>
-      <c r="I30" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="K30" s="1"/>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A31" s="5"/>
-      <c r="D31" s="13"/>
-      <c r="E31" s="14" t="s">
-        <v>8</v>
-      </c>
-      <c r="F31" s="15" t="s">
-        <v>48</v>
+      <c r="F31" s="12" t="s">
+        <v>55</v>
       </c>
       <c r="H31" s="13"/>
       <c r="I31" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="K31" s="1"/>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A32" s="7"/>
+      <c r="D32" s="11"/>
+      <c r="E32" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F32" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="K32" s="16">
+        <v>5</v>
+      </c>
+      <c r="L32" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="M32" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A33" s="7"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="F33" s="15" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A35" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C35" t="s">
+        <v>76</v>
+      </c>
+      <c r="D35" s="8">
+        <v>6</v>
+      </c>
+      <c r="E35" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="F35" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="H35" s="8">
+        <v>6</v>
+      </c>
+      <c r="I35" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="K35" s="16">
+        <v>6</v>
+      </c>
+      <c r="L35" s="17" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A33" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="C33" t="s">
-        <v>79</v>
-      </c>
-      <c r="D33" s="8">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A36" s="5"/>
+      <c r="D36" s="11"/>
+      <c r="E36" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F36" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="H36" s="11"/>
+      <c r="I36" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="K36" s="1"/>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A37" s="5"/>
+      <c r="D37" s="11"/>
+      <c r="E37" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F37" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="H37" s="11"/>
+      <c r="I37" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="K37" s="16">
+        <v>7</v>
+      </c>
+      <c r="L37" s="17" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A38" s="5"/>
+      <c r="D38" s="11"/>
+      <c r="E38" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E33" s="9" t="s">
-        <v>0</v>
-      </c>
-      <c r="F33" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="H33" s="16">
-        <v>5</v>
-      </c>
-      <c r="I33" s="17" t="s">
-        <v>60</v>
-      </c>
-      <c r="K33" s="16">
-        <v>6</v>
-      </c>
-      <c r="L33" s="17" t="s">
+      <c r="F38" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="H38" s="11"/>
+      <c r="I38" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="K38" s="1"/>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A39" s="5"/>
+      <c r="D39" s="13"/>
+      <c r="E39" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="F39" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="H39" s="13"/>
+      <c r="I39" s="15" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" ht="21" x14ac:dyDescent="0.25">
+      <c r="A42" s="18" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A34" s="7"/>
-      <c r="D34" s="11"/>
-      <c r="E34" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="F34" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="K34" s="1"/>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A35" s="7"/>
-      <c r="D35" s="11"/>
-      <c r="E35" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F35" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="K35" s="16">
-        <v>7</v>
-      </c>
-      <c r="L35" s="17" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A36" s="7"/>
-      <c r="D36" s="13"/>
-      <c r="E36" s="14" t="s">
-        <v>6</v>
-      </c>
-      <c r="F36" s="15" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="40" spans="1:12" ht="21" x14ac:dyDescent="0.25">
-      <c r="A40" s="18" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A42" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="B43" t="s">
-        <v>17</v>
-      </c>
-      <c r="G43" t="s">
-        <v>64</v>
-      </c>
-    </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="B44" t="s">
-        <v>18</v>
+      <c r="A44" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B45" t="s">
-        <v>19</v>
+        <v>15</v>
+      </c>
+      <c r="G45" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B46" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B47" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="B48" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B49" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A50" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G50" t="s">
+        <v>63</v>
+      </c>
+      <c r="H50" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A51" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="G51" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A52" s="1"/>
+      <c r="B52" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B53" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B54" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B55" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A57" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A48" s="1" t="s">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B58" t="s">
         <v>22</v>
       </c>
-      <c r="G48" t="s">
-        <v>65</v>
-      </c>
-      <c r="H48" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A49" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="G49" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A50" s="1"/>
-      <c r="B50" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B51" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B52" t="s">
+      <c r="G58" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B59" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B60" t="s">
         <v>70</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B53" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A55" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B56" t="s">
-        <v>24</v>
-      </c>
-      <c r="G56" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B57" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B58" t="s">
-        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added updated summary file etc
</commit_message>
<xml_diff>
--- a/SUMMARY.xlsx
+++ b/SUMMARY.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amartyn/MPIPZ/amartyn/CSSP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{182BF844-AFFE-E947-881C-D945D524F1F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBFB175F-F177-EF4D-8393-F7115C37C98B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14380" yWindow="540" windowWidth="23120" windowHeight="19640" activeTab="1" xr2:uid="{3CB25A69-F844-9241-B587-A0F2F035342F}"/>
+    <workbookView xWindow="11860" yWindow="500" windowWidth="23120" windowHeight="19640" activeTab="1" xr2:uid="{3CB25A69-F844-9241-B587-A0F2F035342F}"/>
   </bookViews>
   <sheets>
     <sheet name="summary" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="203">
   <si>
     <t>A</t>
   </si>
@@ -446,18 +446,12 @@
     <t>check whether ANOVA is used everywhere; or think of potentially other method</t>
   </si>
   <si>
-    <t>Anna version RA: R version 4.5.0 (2025-04-11)</t>
-  </si>
-  <si>
     <t>7_DA_analysis</t>
   </si>
   <si>
     <t>combined</t>
   </si>
   <si>
-    <t>Anna couldn't run</t>
-  </si>
-  <si>
     <t>8_final_figures</t>
   </si>
   <si>
@@ -503,9 +497,6 @@
     <t>(contains pca, volcano plots, bubble plot, highlighted metabolite barplots)</t>
   </si>
   <si>
-    <t>&gt;&gt;&gt; Anna re-rean and got different number of metabolites (slightly)</t>
-  </si>
-  <si>
     <t>&gt;&gt; in DA Lotus overall list (in Annas new one, all the same apart from one feature 1582 which is not in DA list anymore): DA Hordeum are the same</t>
   </si>
   <si>
@@ -522,13 +513,145 @@
   </si>
   <si>
     <t>MISSING</t>
+  </si>
+  <si>
+    <t>Anna version R: R version 4.5.0 (2025-04-11)</t>
+  </si>
+  <si>
+    <t>6_prediction</t>
+  </si>
+  <si>
+    <t>Flowchart</t>
+  </si>
+  <si>
+    <t>Nested Model</t>
+  </si>
+  <si>
+    <t>Fig. 3</t>
+  </si>
+  <si>
+    <t>final_figures</t>
+  </si>
+  <si>
+    <t>suppl_tables</t>
+  </si>
+  <si>
+    <t>&gt;&gt; Anna couldn't run script (error messages)</t>
+  </si>
+  <si>
+    <t>Check in text</t>
+  </si>
+  <si>
+    <t>all orders written in italic</t>
+  </si>
+  <si>
+    <t>Questions</t>
+  </si>
+  <si>
+    <t>previosuly &lt;25% asvs shared among soils, now recalculating it is up to 40%?</t>
+  </si>
+  <si>
+    <t>Ib &gt; check prediction table &gt; results section needs to match this (I previously e.g. said that Burkholderiales, Streptomycetales, and Pseudomonadales where influential ASVs for prediction in Lotus, but according to the figure (stacked bp) it isnt Streptomycetales but Rhizobiales (which are however not found in table of ratios?)</t>
+  </si>
+  <si>
+    <t>add to M&amp;M where raw data, as well as output feature tables etc can be found</t>
+  </si>
+  <si>
+    <t>wrong spelling of abscisic acid in Figure 5D</t>
+  </si>
+  <si>
+    <t>check chao1 CSSP (supplementary figure 3B &gt; NPK rhizo WT and nsp2 both c?</t>
+  </si>
+  <si>
+    <t>&gt;&gt; check comments</t>
+  </si>
+  <si>
+    <t>&gt;&gt; missing: table info indicator ASVs (incl. taxonomy, RA in WT rhizopshere and root in different soils)</t>
+  </si>
+  <si>
+    <t>&gt;&gt;&gt; Anna re-ran and got different number of metabolites (slightly)</t>
+  </si>
+  <si>
+    <t>3_syncoms</t>
+  </si>
+  <si>
+    <t>1_Lotus</t>
+  </si>
+  <si>
+    <t>2_shoot_fw</t>
+  </si>
+  <si>
+    <t>3_nodule_cts</t>
+  </si>
+  <si>
+    <t>4_rarefication</t>
+  </si>
+  <si>
+    <t>for SynCom figures &gt; chao1, stacked bp etc &gt; do we use only matched ASVs or all ASVs (inclduing contaminants" for display?)</t>
+  </si>
+  <si>
+    <t>done for matched ASVs only, as well as all ASVs separately</t>
+  </si>
+  <si>
+    <t>5_chao1</t>
+  </si>
+  <si>
+    <t>1_scripts</t>
+  </si>
+  <si>
+    <t>allASVs</t>
+  </si>
+  <si>
+    <t>matchedASVsonly</t>
+  </si>
+  <si>
+    <t>2_figures</t>
+  </si>
+  <si>
+    <t>6_cpcoa_pcoa</t>
+  </si>
+  <si>
+    <t>cpcoa</t>
+  </si>
+  <si>
+    <t>7_stackedbp_barplots</t>
+  </si>
+  <si>
+    <t>8_DA_maaslin2</t>
+  </si>
+  <si>
+    <t>9_symbionts</t>
+  </si>
+  <si>
+    <t>2_Hordeum</t>
+  </si>
+  <si>
+    <t>later: adjust M&amp;M section to included all packages used</t>
+  </si>
+  <si>
+    <t>in root exudates Lotus data, we also had samples with R7A treatment in there in raw data &gt; we now just deleted those samples from the metadata file and hence only did the downstream analysis with our uninoculated samples &gt;&gt; sufficient?</t>
+  </si>
+  <si>
+    <t>3_rarefication</t>
+  </si>
+  <si>
+    <t>6_stackedbp_barplots</t>
+  </si>
+  <si>
+    <t>7_DA_maaslin2</t>
+  </si>
+  <si>
+    <t>Fig. 6</t>
+  </si>
+  <si>
+    <t>Suppl. Fig. 6</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -558,6 +681,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="11">
@@ -740,7 +869,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -764,13 +893,14 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1104,20 +1234,20 @@
       </c>
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
-      <c r="D1" s="23" t="s">
+      <c r="D1" s="26" t="s">
         <v>82</v>
       </c>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
       <c r="G1" s="18"/>
-      <c r="H1" s="23" t="s">
+      <c r="H1" s="26" t="s">
         <v>83</v>
       </c>
-      <c r="I1" s="23"/>
-      <c r="K1" s="23" t="s">
+      <c r="I1" s="26"/>
+      <c r="K1" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="L1" s="23"/>
+      <c r="L1" s="26"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
@@ -1802,16 +1932,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05F214DF-3300-D745-A4ED-6415291CCBF0}">
-  <dimension ref="A2:M73"/>
+  <dimension ref="A2:M117"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="18.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="19.83203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>136</v>
+        <v>159</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
@@ -1828,7 +1959,7 @@
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="C5" s="26" t="s">
+      <c r="C5" s="25" t="s">
         <v>86</v>
       </c>
       <c r="M5" t="s">
@@ -1836,10 +1967,10 @@
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="D6" s="26" t="s">
+      <c r="D6" s="25" t="s">
         <v>87</v>
       </c>
-      <c r="E6" s="26" t="s">
+      <c r="E6" s="25" t="s">
         <v>89</v>
       </c>
       <c r="M6" t="s">
@@ -1847,147 +1978,181 @@
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="D7" s="26" t="s">
+      <c r="D7" s="25" t="s">
         <v>88</v>
       </c>
-      <c r="E7" s="26" t="s">
-        <v>89</v>
+      <c r="E7" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="M7" s="27" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="C8" s="26" t="s">
+      <c r="C8" s="25" t="s">
         <v>90</v>
       </c>
+      <c r="M8" s="27" t="s">
+        <v>174</v>
+      </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="D9" s="26" t="s">
+      <c r="D9" s="25" t="s">
         <v>87</v>
       </c>
-      <c r="E9" s="26" t="s">
-        <v>89</v>
-      </c>
+      <c r="E9" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="M9" s="1"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="D10" s="26" t="s">
+      <c r="D10" s="25" t="s">
         <v>88</v>
       </c>
-      <c r="E10" s="26" t="s">
-        <v>89</v>
+      <c r="E10" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="C11" s="26" t="s">
+      <c r="C11" s="25" t="s">
         <v>91</v>
       </c>
+      <c r="M11" t="s">
+        <v>168</v>
+      </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="D12" s="26" t="s">
+      <c r="D12" s="25" t="s">
         <v>87</v>
       </c>
+      <c r="M12" s="27" t="s">
+        <v>171</v>
+      </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="E13" s="26" t="s">
+      <c r="E13" s="25" t="s">
         <v>92</v>
       </c>
-      <c r="F13" s="26" t="s">
-        <v>89</v>
-      </c>
-      <c r="G13" s="24" t="s">
+      <c r="F13" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="G13" s="23" t="s">
         <v>93</v>
       </c>
+      <c r="M13" s="27" t="s">
+        <v>172</v>
+      </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="E14" s="26" t="s">
+      <c r="E14" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="F14" s="26" t="s">
-        <v>89</v>
+      <c r="F14" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="M14" s="28" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="D15" s="26" t="s">
+      <c r="D15" s="25" t="s">
         <v>88</v>
       </c>
-      <c r="E15" s="26" t="s">
+      <c r="E15" s="25" t="s">
         <v>92</v>
       </c>
-      <c r="F15" s="26" t="s">
-        <v>89</v>
-      </c>
-      <c r="G15" s="24" t="s">
+      <c r="F15" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="G15" s="23" t="s">
         <v>94</v>
       </c>
+      <c r="M15" s="1"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="E16" s="26" t="s">
+      <c r="E16" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="F16" s="26" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="17" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="F16" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="M16" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="17" spans="3:13" x14ac:dyDescent="0.2">
       <c r="C17" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="18" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="D18" s="26" t="s">
+      <c r="M17" s="27" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="18" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="D18" s="25" t="s">
         <v>96</v>
       </c>
-      <c r="E18" s="26" t="s">
-        <v>89</v>
-      </c>
-      <c r="G18" s="25" t="s">
+      <c r="E18" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="G18" s="24" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="19" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="D19" s="26" t="s">
+      <c r="M18" s="27" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="19" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="D19" s="25" t="s">
         <v>98</v>
       </c>
-      <c r="E19" s="26" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="20" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="E19" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="M19" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="20" spans="3:13" x14ac:dyDescent="0.2">
       <c r="D20" t="s">
         <v>101</v>
       </c>
-      <c r="E20" s="27"/>
-    </row>
-    <row r="21" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="E21" s="26" t="s">
+    </row>
+    <row r="21" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="E21" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="F21" s="26" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="22" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="E22" s="27" t="s">
+      <c r="F21" s="25" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="22" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="E22" t="s">
         <v>102</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="G22" s="25" t="s">
+      <c r="G22" s="24" t="s">
         <v>97</v>
       </c>
       <c r="H22" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="23" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="D23" s="26" t="s">
+    <row r="23" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="D23" s="25" t="s">
         <v>104</v>
       </c>
-      <c r="E23" s="26"/>
-      <c r="F23" s="26" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="24" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="E23" s="25"/>
+      <c r="F23" s="25" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="24" spans="3:13" x14ac:dyDescent="0.2">
       <c r="D24" t="s">
         <v>105</v>
       </c>
@@ -2001,80 +2166,80 @@
         <v>106</v>
       </c>
     </row>
-    <row r="25" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="D25" s="26" t="s">
+    <row r="25" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="D25" s="25" t="s">
         <v>108</v>
       </c>
-      <c r="E25" s="26"/>
-      <c r="F25" s="26" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="26" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="E25" s="25"/>
+      <c r="F25" s="25" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="26" spans="3:13" x14ac:dyDescent="0.2">
       <c r="H26" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="27" spans="3:8" x14ac:dyDescent="0.2">
+    <row r="27" spans="3:13" x14ac:dyDescent="0.2">
       <c r="C27" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="28" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="D28" s="26" t="s">
+    <row r="28" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="D28" s="25" t="s">
         <v>110</v>
       </c>
-      <c r="E28" s="26" t="s">
-        <v>89</v>
-      </c>
-      <c r="G28" s="25" t="s">
+      <c r="E28" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="G28" s="24" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="29" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="D29" s="26" t="s">
+    <row r="29" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="D29" s="25" t="s">
         <v>111</v>
       </c>
-      <c r="E29" s="26" t="s">
-        <v>89</v>
-      </c>
-      <c r="G29" s="25" t="s">
+      <c r="E29" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="G29" s="24" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="30" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="D30" s="26" t="s">
+    <row r="30" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="D30" s="25" t="s">
         <v>112</v>
       </c>
-      <c r="E30" s="26"/>
-    </row>
-    <row r="31" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="E31" s="26" t="s">
+      <c r="E30" s="25"/>
+    </row>
+    <row r="31" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="E31" s="25" t="s">
         <v>87</v>
       </c>
-      <c r="F31" s="26" t="s">
-        <v>89</v>
-      </c>
-      <c r="G31" s="25" t="s">
+      <c r="F31" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="G31" s="24" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="32" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="E32" s="26" t="s">
+    <row r="32" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="E32" s="25" t="s">
         <v>88</v>
       </c>
-      <c r="F32" s="26" t="s">
-        <v>89</v>
-      </c>
-      <c r="G32" s="25" t="s">
+      <c r="F32" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="G32" s="24" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="33" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="D33" s="26" t="s">
+      <c r="D33" s="25" t="s">
         <v>113</v>
       </c>
-      <c r="E33" s="26" t="s">
+      <c r="E33" s="25" t="s">
         <v>89</v>
       </c>
     </row>
@@ -2085,7 +2250,7 @@
       <c r="E34" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="G34" s="25" t="s">
+      <c r="G34" s="24" t="s">
         <v>115</v>
       </c>
       <c r="H34" t="s">
@@ -2093,10 +2258,10 @@
       </c>
     </row>
     <row r="35" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="D35" s="26" t="s">
+      <c r="D35" s="25" t="s">
         <v>117</v>
       </c>
-      <c r="E35" s="26" t="s">
+      <c r="E35" s="25" t="s">
         <v>89</v>
       </c>
     </row>
@@ -2133,104 +2298,104 @@
       </c>
     </row>
     <row r="41" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="D41" s="26" t="s">
+      <c r="D41" s="25" t="s">
         <v>110</v>
       </c>
-      <c r="E41" s="26" t="s">
-        <v>89</v>
-      </c>
-      <c r="G41" s="25" t="s">
+      <c r="E41" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="G41" s="24" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="42" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="D42" s="26" t="s">
+      <c r="D42" s="25" t="s">
         <v>125</v>
       </c>
-      <c r="E42" s="26" t="s">
-        <v>89</v>
-      </c>
-      <c r="G42" s="25" t="s">
+      <c r="E42" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="G42" s="24" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="43" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="D43" s="26" t="s">
+      <c r="D43" s="25" t="s">
         <v>126</v>
       </c>
-      <c r="E43" s="26" t="s">
+      <c r="E43" s="25" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="44" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="D44" s="26" t="s">
+      <c r="D44" s="25" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="45" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="E45" s="26" t="s">
+      <c r="E45" s="25" t="s">
         <v>87</v>
       </c>
-      <c r="F45" s="26" t="s">
-        <v>89</v>
-      </c>
-      <c r="G45" s="25" t="s">
+      <c r="F45" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="G45" s="24" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="46" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="E46" s="26" t="s">
+      <c r="E46" s="25" t="s">
         <v>88</v>
       </c>
-      <c r="F46" s="26" t="s">
-        <v>89</v>
-      </c>
-      <c r="G46" s="25" t="s">
+      <c r="F46" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="G46" s="24" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="47" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="D47" s="26" t="s">
+      <c r="D47" s="25" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="48" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="E48" s="26" t="s">
+      <c r="E48" s="25" t="s">
         <v>87</v>
       </c>
-      <c r="F48" s="26" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="49" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="E49" s="26" t="s">
+      <c r="F48" s="25" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="49" spans="4:12" x14ac:dyDescent="0.2">
+      <c r="E49" s="25" t="s">
         <v>88</v>
       </c>
-      <c r="F49" s="26" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="50" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="F49" s="25" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="50" spans="4:12" x14ac:dyDescent="0.2">
       <c r="D50" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="51" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="E51" s="26" t="s">
+    <row r="51" spans="4:12" x14ac:dyDescent="0.2">
+      <c r="E51" s="25" t="s">
         <v>130</v>
       </c>
-      <c r="F51" s="26" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="52" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="E52" s="26" t="s">
+      <c r="F51" s="25" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="52" spans="4:12" x14ac:dyDescent="0.2">
+      <c r="E52" s="25" t="s">
         <v>131</v>
       </c>
       <c r="F52" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="G52" s="25" t="s">
+      <c r="G52" s="24" t="s">
         <v>132</v>
       </c>
       <c r="H52" t="s">
@@ -2240,40 +2405,42 @@
         <v>134</v>
       </c>
     </row>
-    <row r="53" spans="2:12" x14ac:dyDescent="0.2">
+    <row r="53" spans="4:12" x14ac:dyDescent="0.2">
       <c r="D53" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="54" spans="4:12" x14ac:dyDescent="0.2">
+      <c r="E54" t="s">
+        <v>87</v>
+      </c>
+      <c r="F54" s="2"/>
+      <c r="H54" s="11"/>
+    </row>
+    <row r="55" spans="4:12" x14ac:dyDescent="0.2">
+      <c r="E55" t="s">
+        <v>88</v>
+      </c>
+      <c r="F55" s="2"/>
+      <c r="H55" s="11" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="56" spans="4:12" x14ac:dyDescent="0.2">
+      <c r="E56" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="54" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="C54" t="s">
+      <c r="F56" s="2"/>
+      <c r="H56" s="11"/>
+    </row>
+    <row r="57" spans="4:12" x14ac:dyDescent="0.2">
+      <c r="D57" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="58" spans="4:12" x14ac:dyDescent="0.2">
+      <c r="E58" t="s">
         <v>139</v>
-      </c>
-      <c r="E54" s="27" t="s">
-        <v>87</v>
-      </c>
-      <c r="F54" s="2"/>
-    </row>
-    <row r="55" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="E55" s="27" t="s">
-        <v>88</v>
-      </c>
-      <c r="F55" s="2"/>
-    </row>
-    <row r="56" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="E56" s="27" t="s">
-        <v>138</v>
-      </c>
-      <c r="F56" s="2"/>
-    </row>
-    <row r="57" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="D57" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="58" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="E58" t="s">
-        <v>141</v>
       </c>
       <c r="F58" s="2" t="s">
         <v>89</v>
@@ -2282,123 +2449,398 @@
         <v>122</v>
       </c>
     </row>
-    <row r="59" spans="2:12" x14ac:dyDescent="0.2">
+    <row r="59" spans="4:12" x14ac:dyDescent="0.2">
       <c r="E59" t="s">
+        <v>140</v>
+      </c>
+      <c r="F59" s="25" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="60" spans="4:12" x14ac:dyDescent="0.2">
+      <c r="E60" t="s">
         <v>142</v>
       </c>
-      <c r="F59" s="26" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="60" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="E60" t="s">
+      <c r="F60" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="H60" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="61" spans="4:12" x14ac:dyDescent="0.2">
+      <c r="E61" t="s">
+        <v>141</v>
+      </c>
+      <c r="F61" s="25" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="62" spans="4:12" x14ac:dyDescent="0.2">
+      <c r="D62" t="s">
         <v>144</v>
-      </c>
-      <c r="F60" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="H60" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="61" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="E61" t="s">
-        <v>143</v>
-      </c>
-      <c r="F61" s="26" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="62" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="D62" t="s">
-        <v>146</v>
       </c>
       <c r="E62" s="2"/>
       <c r="H62" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="65" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="C65" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="66" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="D66" t="s">
+        <v>161</v>
+      </c>
+      <c r="F66" s="25" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="67" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="D67" t="s">
+        <v>162</v>
+      </c>
+      <c r="F67" s="2"/>
+      <c r="H67" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="68" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="D68" t="s">
+        <v>164</v>
+      </c>
+      <c r="E68" t="s">
+        <v>163</v>
+      </c>
+      <c r="F68" s="2"/>
+      <c r="H68" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="69" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="D69" t="s">
+        <v>165</v>
+      </c>
+      <c r="F69" s="2"/>
+      <c r="H69" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="71" spans="2:10" ht="21" x14ac:dyDescent="0.25">
+      <c r="B71" s="18" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="72" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="C72" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="64" spans="2:12" ht="21" x14ac:dyDescent="0.25">
-      <c r="B64" s="18" t="s">
+    <row r="73" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="D73" t="s">
+        <v>87</v>
+      </c>
+      <c r="E73" s="2"/>
+      <c r="F73" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="65" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C65" s="27" t="s">
+    <row r="74" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="D74" s="25" t="s">
+        <v>88</v>
+      </c>
+      <c r="E74" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="J74" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="75" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="C75" t="s">
+        <v>90</v>
+      </c>
+      <c r="D75" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="J75" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="76" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="C76" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="66" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="D66" t="s">
+      <c r="D76" t="s">
+        <v>152</v>
+      </c>
+      <c r="J76" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="77" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="C77" t="s">
+        <v>150</v>
+      </c>
+      <c r="J77" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="78" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="D78" s="25" t="s">
+        <v>156</v>
+      </c>
+      <c r="E78" s="25" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="79" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="D79" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="E79" s="2" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="80" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="C80" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="81" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="D81" s="25" t="s">
         <v>87</v>
       </c>
-      <c r="F66" t="s">
+      <c r="E81" s="25" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="82" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="D82" s="25" t="s">
+        <v>88</v>
+      </c>
+      <c r="E82" s="25" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="84" spans="2:7" ht="21" x14ac:dyDescent="0.25">
+      <c r="B84" s="18" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="85" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="C85" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="86" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="D86" s="25" t="s">
+        <v>86</v>
+      </c>
+      <c r="E86" s="25" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="87" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="D87" s="25" t="s">
+        <v>90</v>
+      </c>
+      <c r="E87" s="25" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="88" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="D88" s="25" t="s">
+        <v>180</v>
+      </c>
+      <c r="E88" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="G88" s="24" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="89" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="D89" s="25" t="s">
+        <v>181</v>
+      </c>
+      <c r="E89" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="G89" s="24" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="90" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="D90" s="25" t="s">
+        <v>182</v>
+      </c>
+      <c r="E90" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="G90" s="23" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="91" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="D91" s="25" t="s">
+        <v>185</v>
+      </c>
+      <c r="G91" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="92" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="E92" s="25" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="93" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="F93" s="25" t="s">
+        <v>187</v>
+      </c>
+      <c r="G93" s="25" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="94" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="F94" s="25" t="s">
+        <v>188</v>
+      </c>
+      <c r="G94" s="25" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="95" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="E95" s="25" t="s">
+        <v>189</v>
+      </c>
+      <c r="F95" s="25" t="s">
+        <v>89</v>
+      </c>
+      <c r="G95" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="96" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="D96" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="97" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="E97" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="98" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="E98" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="99" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D99" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="100" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D100" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="101" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D101" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="102" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C102" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="103" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D103" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="104" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D104" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="105" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D105" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="106" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D106" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="107" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D107" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="108" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D108" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="109" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D109" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="110" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D110" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="111" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C111" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="67" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="D67" t="s">
+    <row r="112" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D112" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="113" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D113" t="s">
+        <v>202</v>
+      </c>
+      <c r="E113" s="2" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="114" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="E114" s="2" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="115" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C115" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="116" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D116" t="s">
+        <v>87</v>
+      </c>
+      <c r="E116" s="2" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="117" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D117" t="s">
         <v>88</v>
       </c>
-      <c r="E67" s="26" t="s">
-        <v>89</v>
-      </c>
-      <c r="J67" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="68" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C68" t="s">
-        <v>90</v>
-      </c>
-      <c r="D68" s="26" t="s">
-        <v>89</v>
-      </c>
-      <c r="J68" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="69" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C69" t="s">
-        <v>151</v>
-      </c>
-      <c r="D69" t="s">
-        <v>154</v>
-      </c>
-      <c r="J69" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="70" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C70" t="s">
-        <v>152</v>
-      </c>
-      <c r="J70" t="s">
+      <c r="E117" s="2" t="s">
         <v>158</v>
-      </c>
-    </row>
-    <row r="71" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="D71" t="s">
-        <v>159</v>
-      </c>
-      <c r="E71" s="26" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="72" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="D72" t="s">
-        <v>160</v>
-      </c>
-      <c r="E72" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="73" spans="3:10" x14ac:dyDescent="0.2">
-      <c r="C73" t="s">
-        <v>153</v>
-      </c>
-      <c r="D73" s="26" t="s">
-        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added updated summary file and draft 5 and 6
</commit_message>
<xml_diff>
--- a/SUMMARY.xlsx
+++ b/SUMMARY.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amartyn/MPIPZ/amartyn/CSSP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBFB175F-F177-EF4D-8393-F7115C37C98B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59E04058-9A8E-6247-9A4A-C80EB066849F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11860" yWindow="500" windowWidth="23120" windowHeight="19640" activeTab="1" xr2:uid="{3CB25A69-F844-9241-B587-A0F2F035342F}"/>
+    <workbookView xWindow="0" yWindow="720" windowWidth="29400" windowHeight="18400" activeTab="1" xr2:uid="{3CB25A69-F844-9241-B587-A0F2F035342F}"/>
   </bookViews>
   <sheets>
     <sheet name="summary" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="216">
   <si>
     <t>A</t>
   </si>
@@ -645,6 +645,45 @@
   </si>
   <si>
     <t>Suppl. Fig. 6</t>
+  </si>
+  <si>
+    <t>ANNA (to do 03.02.)</t>
+  </si>
+  <si>
+    <t>finish bibliography</t>
+  </si>
+  <si>
+    <t>work on comments in draft6</t>
+  </si>
+  <si>
+    <t>bulk figure &gt; remove txt from workflow in panel A</t>
+  </si>
+  <si>
+    <t>WT figure &gt; adjust workflow in panel A (remove text)</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> adjust figure quality in all figures (if necessary)</t>
+  </si>
+  <si>
+    <t>root exudate figure &gt; add y axis to boxplots</t>
+  </si>
+  <si>
+    <t>work on SynCom figure &gt; also remove nodule section from bubbleplot &amp; move figure incl. nodule plot to Suppl.</t>
+  </si>
+  <si>
+    <t>write letter to editor</t>
+  </si>
+  <si>
+    <t>set up online PNAS submission</t>
+  </si>
+  <si>
+    <t>OVERALL PRIORITY</t>
+  </si>
+  <si>
+    <t>&gt; get text and figures done to send out to co-authors</t>
+  </si>
+  <si>
+    <t>figure captions</t>
   </si>
 </sst>
 </file>
@@ -869,7 +908,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -894,12 +933,13 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1234,20 +1274,20 @@
       </c>
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
-      <c r="D1" s="26" t="s">
+      <c r="D1" s="28" t="s">
         <v>82</v>
       </c>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
       <c r="G1" s="18"/>
-      <c r="H1" s="26" t="s">
+      <c r="H1" s="28" t="s">
         <v>83</v>
       </c>
-      <c r="I1" s="26"/>
-      <c r="K1" s="26" t="s">
+      <c r="I1" s="28"/>
+      <c r="K1" s="28" t="s">
         <v>41</v>
       </c>
-      <c r="L1" s="26"/>
+      <c r="L1" s="28"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
@@ -1959,7 +1999,7 @@
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="C5" s="25" t="s">
+      <c r="C5" s="24" t="s">
         <v>86</v>
       </c>
       <c r="M5" t="s">
@@ -1967,10 +2007,10 @@
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="D6" s="25" t="s">
+      <c r="D6" s="24" t="s">
         <v>87</v>
       </c>
-      <c r="E6" s="25" t="s">
+      <c r="E6" s="24" t="s">
         <v>89</v>
       </c>
       <c r="M6" t="s">
@@ -1978,165 +2018,171 @@
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="D7" s="25" t="s">
+      <c r="D7" s="24" t="s">
         <v>88</v>
       </c>
-      <c r="E7" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="M7" s="27" t="s">
+      <c r="E7" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="M7" s="25" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="C8" s="25" t="s">
+      <c r="C8" s="24" t="s">
         <v>90</v>
       </c>
-      <c r="M8" s="27" t="s">
+      <c r="M8" s="25" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="D9" s="25" t="s">
+      <c r="D9" s="24" t="s">
         <v>87</v>
       </c>
-      <c r="E9" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="M9" s="1"/>
+      <c r="E9" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="M9" s="29" t="s">
+        <v>208</v>
+      </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="D10" s="25" t="s">
+      <c r="D10" s="24" t="s">
         <v>88</v>
       </c>
-      <c r="E10" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="M10" s="1" t="s">
-        <v>167</v>
+      <c r="E10" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="M10" s="29" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="C11" s="25" t="s">
+      <c r="C11" s="24" t="s">
         <v>91</v>
       </c>
-      <c r="M11" t="s">
-        <v>168</v>
+      <c r="M11" s="25" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="D12" s="25" t="s">
+      <c r="D12" s="24" t="s">
         <v>87</v>
       </c>
-      <c r="M12" s="27" t="s">
-        <v>171</v>
-      </c>
+      <c r="M12" s="1"/>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="E13" s="25" t="s">
+      <c r="E13" s="24" t="s">
         <v>92</v>
       </c>
-      <c r="F13" s="25" t="s">
+      <c r="F13" s="24" t="s">
         <v>89</v>
       </c>
       <c r="G13" s="23" t="s">
         <v>93</v>
       </c>
-      <c r="M13" s="27" t="s">
-        <v>172</v>
+      <c r="M13" s="1" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="E14" s="25" t="s">
+      <c r="E14" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="F14" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="M14" s="28" t="s">
-        <v>196</v>
+      <c r="F14" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="M14" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="D15" s="25" t="s">
+      <c r="D15" s="24" t="s">
         <v>88</v>
       </c>
-      <c r="E15" s="25" t="s">
+      <c r="E15" s="24" t="s">
         <v>92</v>
       </c>
-      <c r="F15" s="25" t="s">
+      <c r="F15" s="24" t="s">
         <v>89</v>
       </c>
       <c r="G15" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="M15" s="1"/>
+      <c r="M15" s="25" t="s">
+        <v>172</v>
+      </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="E16" s="25" t="s">
+      <c r="E16" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="F16" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="M16" s="1" t="s">
-        <v>169</v>
+      <c r="F16" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="M16" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="17" spans="3:13" x14ac:dyDescent="0.2">
       <c r="C17" t="s">
         <v>95</v>
       </c>
-      <c r="M17" s="27" t="s">
+      <c r="M17" s="1"/>
+    </row>
+    <row r="18" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="D18" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="E18" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="G18" s="27" t="s">
+        <v>97</v>
+      </c>
+      <c r="M18" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="19" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="D19" s="26" t="s">
+        <v>98</v>
+      </c>
+      <c r="E19" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="M19" s="25" t="s">
         <v>170</v>
-      </c>
-    </row>
-    <row r="18" spans="3:13" x14ac:dyDescent="0.2">
-      <c r="D18" s="25" t="s">
-        <v>96</v>
-      </c>
-      <c r="E18" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="G18" s="24" t="s">
-        <v>97</v>
-      </c>
-      <c r="M18" s="27" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="19" spans="3:13" x14ac:dyDescent="0.2">
-      <c r="D19" s="25" t="s">
-        <v>98</v>
-      </c>
-      <c r="E19" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="M19" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="20" spans="3:13" x14ac:dyDescent="0.2">
       <c r="D20" t="s">
         <v>101</v>
       </c>
+      <c r="M20" s="25" t="s">
+        <v>183</v>
+      </c>
     </row>
     <row r="21" spans="3:13" x14ac:dyDescent="0.2">
-      <c r="E21" s="25" t="s">
+      <c r="E21" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="F21" s="25" t="s">
-        <v>89</v>
+      <c r="F21" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="M21" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="22" spans="3:13" x14ac:dyDescent="0.2">
-      <c r="E22" t="s">
+      <c r="E22" s="1" t="s">
         <v>102</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="G22" s="24" t="s">
+      <c r="G22" s="27" t="s">
         <v>97</v>
       </c>
       <c r="H22" t="s">
@@ -2144,11 +2190,11 @@
       </c>
     </row>
     <row r="23" spans="3:13" x14ac:dyDescent="0.2">
-      <c r="D23" s="25" t="s">
+      <c r="D23" s="24" t="s">
         <v>104</v>
       </c>
-      <c r="E23" s="25"/>
-      <c r="F23" s="25" t="s">
+      <c r="E23" s="24"/>
+      <c r="F23" s="24" t="s">
         <v>89</v>
       </c>
     </row>
@@ -2167,11 +2213,11 @@
       </c>
     </row>
     <row r="25" spans="3:13" x14ac:dyDescent="0.2">
-      <c r="D25" s="25" t="s">
+      <c r="D25" s="24" t="s">
         <v>108</v>
       </c>
-      <c r="E25" s="25"/>
-      <c r="F25" s="25" t="s">
+      <c r="E25" s="24"/>
+      <c r="F25" s="24" t="s">
         <v>89</v>
       </c>
     </row>
@@ -2186,91 +2232,130 @@
       </c>
     </row>
     <row r="28" spans="3:13" x14ac:dyDescent="0.2">
-      <c r="D28" s="25" t="s">
+      <c r="D28" s="24" t="s">
         <v>110</v>
       </c>
-      <c r="E28" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="G28" s="24" t="s">
+      <c r="E28" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="G28" s="27" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="29" spans="3:13" x14ac:dyDescent="0.2">
-      <c r="D29" s="25" t="s">
+      <c r="D29" s="24" t="s">
         <v>111</v>
       </c>
-      <c r="E29" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="G29" s="24" t="s">
+      <c r="E29" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="G29" s="27" t="s">
         <v>97</v>
       </c>
+      <c r="M29" s="1" t="s">
+        <v>203</v>
+      </c>
     </row>
     <row r="30" spans="3:13" x14ac:dyDescent="0.2">
-      <c r="D30" s="25" t="s">
+      <c r="D30" s="24" t="s">
         <v>112</v>
       </c>
-      <c r="E30" s="25"/>
+      <c r="E30" s="24"/>
+      <c r="L30" t="s">
+        <v>71</v>
+      </c>
+      <c r="M30" t="s">
+        <v>204</v>
+      </c>
     </row>
     <row r="31" spans="3:13" x14ac:dyDescent="0.2">
-      <c r="E31" s="25" t="s">
+      <c r="E31" s="24" t="s">
         <v>87</v>
       </c>
-      <c r="F31" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="G31" s="24" t="s">
+      <c r="F31" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="G31" s="27" t="s">
         <v>97</v>
       </c>
+      <c r="L31" t="s">
+        <v>71</v>
+      </c>
+      <c r="M31" t="s">
+        <v>205</v>
+      </c>
     </row>
     <row r="32" spans="3:13" x14ac:dyDescent="0.2">
-      <c r="E32" s="25" t="s">
+      <c r="E32" s="24" t="s">
         <v>88</v>
       </c>
-      <c r="F32" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="G32" s="24" t="s">
+      <c r="F32" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="G32" s="27" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="33" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="D33" s="25" t="s">
+      <c r="L32" t="s">
+        <v>71</v>
+      </c>
+      <c r="M32" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="33" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="D33" s="26" t="s">
         <v>113</v>
       </c>
-      <c r="E33" s="25" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="34" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="D34" t="s">
+      <c r="E33" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="L33" t="s">
+        <v>71</v>
+      </c>
+      <c r="M33" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="34" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="D34" s="1" t="s">
         <v>114</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="G34" s="24" t="s">
+      <c r="G34" s="27" t="s">
         <v>115</v>
       </c>
       <c r="H34" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="35" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="D35" s="25" t="s">
+      <c r="L34" t="s">
+        <v>71</v>
+      </c>
+      <c r="M34" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="35" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="D35" s="24" t="s">
         <v>117</v>
       </c>
-      <c r="E35" s="25" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="36" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="E35" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="M35" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="36" spans="3:13" x14ac:dyDescent="0.2">
       <c r="D36" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="37" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="M36" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="37" spans="3:13" x14ac:dyDescent="0.2">
       <c r="E37" t="s">
         <v>119</v>
       </c>
@@ -2280,8 +2365,11 @@
       <c r="H37" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="38" spans="3:8" x14ac:dyDescent="0.2">
+      <c r="M37" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="38" spans="3:13" x14ac:dyDescent="0.2">
       <c r="E38" t="s">
         <v>121</v>
       </c>
@@ -2292,86 +2380,94 @@
         <v>123</v>
       </c>
     </row>
-    <row r="40" spans="3:8" x14ac:dyDescent="0.2">
+    <row r="39" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="M39" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="40" spans="3:13" x14ac:dyDescent="0.2">
       <c r="C40" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="41" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="D41" s="25" t="s">
+      <c r="M40" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="41" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="D41" s="24" t="s">
         <v>110</v>
       </c>
-      <c r="E41" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="G41" s="24" t="s">
+      <c r="E41" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="G41" s="27" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="42" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="D42" s="25" t="s">
+    <row r="42" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="D42" s="24" t="s">
         <v>125</v>
       </c>
-      <c r="E42" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="G42" s="24" t="s">
+      <c r="E42" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="G42" s="27" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="43" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="D43" s="25" t="s">
+    <row r="43" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="D43" s="24" t="s">
         <v>126</v>
       </c>
-      <c r="E43" s="25" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="44" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="D44" s="25" t="s">
+      <c r="E43" s="24" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="44" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="D44" s="24" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="45" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="E45" s="25" t="s">
+    <row r="45" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="E45" s="24" t="s">
         <v>87</v>
       </c>
-      <c r="F45" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="G45" s="24" t="s">
+      <c r="F45" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="G45" s="27" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="46" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="E46" s="25" t="s">
+    <row r="46" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="E46" s="24" t="s">
         <v>88</v>
       </c>
-      <c r="F46" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="G46" s="24" t="s">
+      <c r="F46" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="G46" s="27" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="47" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="D47" s="25" t="s">
+    <row r="47" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="D47" s="26" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="48" spans="3:8" x14ac:dyDescent="0.2">
-      <c r="E48" s="25" t="s">
+    <row r="48" spans="3:13" x14ac:dyDescent="0.2">
+      <c r="E48" s="24" t="s">
         <v>87</v>
       </c>
-      <c r="F48" s="25" t="s">
+      <c r="F48" s="24" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="49" spans="4:12" x14ac:dyDescent="0.2">
-      <c r="E49" s="25" t="s">
+      <c r="E49" s="24" t="s">
         <v>88</v>
       </c>
-      <c r="F49" s="25" t="s">
+      <c r="F49" s="24" t="s">
         <v>89</v>
       </c>
     </row>
@@ -2381,21 +2477,21 @@
       </c>
     </row>
     <row r="51" spans="4:12" x14ac:dyDescent="0.2">
-      <c r="E51" s="25" t="s">
+      <c r="E51" s="26" t="s">
         <v>130</v>
       </c>
-      <c r="F51" s="25" t="s">
+      <c r="F51" s="24" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="52" spans="4:12" x14ac:dyDescent="0.2">
-      <c r="E52" s="25" t="s">
+      <c r="E52" s="24" t="s">
         <v>131</v>
       </c>
       <c r="F52" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="G52" s="24" t="s">
+      <c r="G52" s="27" t="s">
         <v>132</v>
       </c>
       <c r="H52" t="s">
@@ -2453,7 +2549,7 @@
       <c r="E59" t="s">
         <v>140</v>
       </c>
-      <c r="F59" s="25" t="s">
+      <c r="F59" s="24" t="s">
         <v>89</v>
       </c>
     </row>
@@ -2472,7 +2568,7 @@
       <c r="E61" t="s">
         <v>141</v>
       </c>
-      <c r="F61" s="25" t="s">
+      <c r="F61" s="24" t="s">
         <v>89</v>
       </c>
     </row>
@@ -2494,7 +2590,7 @@
       <c r="D66" t="s">
         <v>161</v>
       </c>
-      <c r="F66" s="25" t="s">
+      <c r="F66" s="24" t="s">
         <v>89</v>
       </c>
     </row>
@@ -2548,10 +2644,10 @@
       </c>
     </row>
     <row r="74" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="D74" s="25" t="s">
+      <c r="D74" s="24" t="s">
         <v>88</v>
       </c>
-      <c r="E74" s="25" t="s">
+      <c r="E74" s="24" t="s">
         <v>89</v>
       </c>
       <c r="J74" t="s">
@@ -2562,7 +2658,7 @@
       <c r="C75" t="s">
         <v>90</v>
       </c>
-      <c r="D75" s="25" t="s">
+      <c r="D75" s="24" t="s">
         <v>89</v>
       </c>
       <c r="J75" t="s">
@@ -2589,10 +2685,10 @@
       </c>
     </row>
     <row r="78" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="D78" s="25" t="s">
+      <c r="D78" s="24" t="s">
         <v>156</v>
       </c>
-      <c r="E78" s="25" t="s">
+      <c r="E78" s="24" t="s">
         <v>89</v>
       </c>
     </row>
@@ -2609,123 +2705,126 @@
         <v>151</v>
       </c>
     </row>
-    <row r="81" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="D81" s="25" t="s">
+    <row r="81" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="D81" s="24" t="s">
         <v>87</v>
       </c>
-      <c r="E81" s="25" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="82" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="D82" s="25" t="s">
+      <c r="E81" s="24" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="82" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="D82" s="24" t="s">
         <v>88</v>
       </c>
-      <c r="E82" s="25" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="84" spans="2:7" ht="21" x14ac:dyDescent="0.25">
+      <c r="E82" s="24" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="84" spans="2:12" ht="21" x14ac:dyDescent="0.25">
       <c r="B84" s="18" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="85" spans="2:7" x14ac:dyDescent="0.2">
+    <row r="85" spans="2:12" x14ac:dyDescent="0.2">
       <c r="C85" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="86" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="D86" s="25" t="s">
+    <row r="86" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="D86" s="24" t="s">
         <v>86</v>
       </c>
-      <c r="E86" s="25" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="87" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="D87" s="25" t="s">
+      <c r="E86" s="24" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="87" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="D87" s="24" t="s">
         <v>90</v>
       </c>
-      <c r="E87" s="25" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="88" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="D88" s="25" t="s">
+      <c r="E87" s="24" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="88" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="D88" s="24" t="s">
         <v>180</v>
       </c>
-      <c r="E88" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="G88" s="24" t="s">
+      <c r="E88" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="G88" s="27" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="89" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="D89" s="25" t="s">
+    <row r="89" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="D89" s="24" t="s">
         <v>181</v>
       </c>
-      <c r="E89" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="G89" s="24" t="s">
+      <c r="E89" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="G89" s="27" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="90" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="D90" s="25" t="s">
+    <row r="90" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="D90" s="24" t="s">
         <v>182</v>
       </c>
-      <c r="E90" s="25" t="s">
+      <c r="E90" s="24" t="s">
         <v>89</v>
       </c>
       <c r="G90" s="23" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="91" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="D91" s="25" t="s">
+    <row r="91" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="D91" s="24" t="s">
         <v>185</v>
       </c>
       <c r="G91" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="92" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="E92" s="25" t="s">
+    <row r="92" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="E92" s="24" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="93" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="F93" s="25" t="s">
+    <row r="93" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="F93" s="24" t="s">
         <v>187</v>
       </c>
-      <c r="G93" s="25" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="94" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="F94" s="25" t="s">
+      <c r="G93" s="24" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="94" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="F94" s="24" t="s">
         <v>188</v>
       </c>
-      <c r="G94" s="25" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="95" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="E95" s="25" t="s">
+      <c r="G94" s="24" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="95" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="E95" s="24" t="s">
         <v>189</v>
       </c>
-      <c r="F95" s="25" t="s">
+      <c r="F95" s="24" t="s">
         <v>89</v>
       </c>
       <c r="G95" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="96" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="D96" t="s">
+      <c r="L95" s="27" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="96" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="D96" s="1" t="s">
         <v>190</v>
       </c>
     </row>
@@ -2740,7 +2839,7 @@
       </c>
     </row>
     <row r="99" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="D99" t="s">
+      <c r="D99" s="1" t="s">
         <v>192</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added updated draft and summary file
</commit_message>
<xml_diff>
--- a/SUMMARY.xlsx
+++ b/SUMMARY.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amartyn/MPIPZ/amartyn/CSSP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59E04058-9A8E-6247-9A4A-C80EB066849F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F430F791-484F-5943-85BD-79EA2E13CDD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="720" windowWidth="29400" windowHeight="18400" activeTab="1" xr2:uid="{3CB25A69-F844-9241-B587-A0F2F035342F}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="17240" activeTab="1" xr2:uid="{3CB25A69-F844-9241-B587-A0F2F035342F}"/>
   </bookViews>
   <sheets>
     <sheet name="summary" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="213">
   <si>
     <t>A</t>
   </si>
@@ -497,9 +497,6 @@
     <t>(contains pca, volcano plots, bubble plot, highlighted metabolite barplots)</t>
   </si>
   <si>
-    <t>&gt;&gt; in DA Lotus overall list (in Annas new one, all the same apart from one feature 1582 which is not in DA list anymore): DA Hordeum are the same</t>
-  </si>
-  <si>
     <t>&gt;&gt; if time: Ib add slighlty more comments to explain procedure</t>
   </si>
   <si>
@@ -521,12 +518,6 @@
     <t>6_prediction</t>
   </si>
   <si>
-    <t>Flowchart</t>
-  </si>
-  <si>
-    <t>Nested Model</t>
-  </si>
-  <si>
     <t>Fig. 3</t>
   </si>
   <si>
@@ -551,9 +542,6 @@
     <t>previosuly &lt;25% asvs shared among soils, now recalculating it is up to 40%?</t>
   </si>
   <si>
-    <t>Ib &gt; check prediction table &gt; results section needs to match this (I previously e.g. said that Burkholderiales, Streptomycetales, and Pseudomonadales where influential ASVs for prediction in Lotus, but according to the figure (stacked bp) it isnt Streptomycetales but Rhizobiales (which are however not found in table of ratios?)</t>
-  </si>
-  <si>
     <t>add to M&amp;M where raw data, as well as output feature tables etc can be found</t>
   </si>
   <si>
@@ -653,9 +641,6 @@
     <t>finish bibliography</t>
   </si>
   <si>
-    <t>work on comments in draft6</t>
-  </si>
-  <si>
     <t>bulk figure &gt; remove txt from workflow in panel A</t>
   </si>
   <si>
@@ -684,6 +669,12 @@
   </si>
   <si>
     <t>figure captions</t>
+  </si>
+  <si>
+    <t>Analysis</t>
+  </si>
+  <si>
+    <t>&gt;&gt; in DI Lotus overall list (in Annas new one, all the same apart from one feature 1582 which is not in DA list anymore): DA Hordeum are the same</t>
   </si>
 </sst>
 </file>
@@ -728,7 +719,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -786,6 +777,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -908,7 +905,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -940,7 +937,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1972,7 +1970,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05F214DF-3300-D745-A4ED-6415291CCBF0}">
-  <dimension ref="A2:M117"/>
+  <dimension ref="A2:W117"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="18.6640625" bestFit="1" customWidth="1"/>
@@ -1980,17 +1978,17 @@
     <col min="6" max="6" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="M3" s="1" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="21" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" ht="21" x14ac:dyDescent="0.25">
       <c r="B4" s="18" t="s">
         <v>84</v>
       </c>
@@ -1998,7 +1996,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="C5" s="24" t="s">
         <v>86</v>
       </c>
@@ -2006,7 +2004,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="D6" s="24" t="s">
         <v>87</v>
       </c>
@@ -2017,37 +2015,40 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="D7" s="24" t="s">
         <v>88</v>
       </c>
       <c r="E7" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="M7" s="25" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="M7" s="30" t="s">
+        <v>169</v>
+      </c>
+      <c r="N7" s="29"/>
+      <c r="O7" s="29"/>
+      <c r="P7" s="29"/>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="C8" s="24" t="s">
         <v>90</v>
       </c>
       <c r="M8" s="25" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="D9" s="24" t="s">
         <v>87</v>
       </c>
       <c r="E9" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="M9" s="29" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="M9" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="D10" s="24" t="s">
         <v>88</v>
       </c>
@@ -2055,24 +2056,25 @@
         <v>89</v>
       </c>
       <c r="M10" s="29" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+        <v>204</v>
+      </c>
+      <c r="N10" s="29"/>
+      <c r="O10" s="29"/>
+      <c r="P10" s="29"/>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="C11" s="24" t="s">
         <v>91</v>
       </c>
-      <c r="M11" s="25" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="M11" s="25"/>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="D12" s="24" t="s">
         <v>87</v>
       </c>
       <c r="M12" s="1"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="E13" s="24" t="s">
         <v>92</v>
       </c>
@@ -2083,10 +2085,10 @@
         <v>93</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="E14" s="24" t="s">
         <v>3</v>
       </c>
@@ -2094,10 +2096,10 @@
         <v>89</v>
       </c>
       <c r="M14" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="D15" s="24" t="s">
         <v>88</v>
       </c>
@@ -2111,10 +2113,10 @@
         <v>94</v>
       </c>
       <c r="M15" s="25" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
       <c r="E16" s="24" t="s">
         <v>3</v>
       </c>
@@ -2122,14 +2124,13 @@
         <v>89</v>
       </c>
       <c r="M16" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
     </row>
     <row r="17" spans="3:13" x14ac:dyDescent="0.2">
       <c r="C17" t="s">
         <v>95</v>
       </c>
-      <c r="M17" s="1"/>
     </row>
     <row r="18" spans="3:13" x14ac:dyDescent="0.2">
       <c r="D18" s="24" t="s">
@@ -2141,9 +2142,7 @@
       <c r="G18" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="M18" s="1" t="s">
-        <v>169</v>
-      </c>
+      <c r="M18" s="1"/>
     </row>
     <row r="19" spans="3:13" x14ac:dyDescent="0.2">
       <c r="D19" s="26" t="s">
@@ -2152,8 +2151,8 @@
       <c r="E19" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="M19" s="25" t="s">
-        <v>170</v>
+      <c r="M19" s="1" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="20" spans="3:13" x14ac:dyDescent="0.2">
@@ -2161,7 +2160,7 @@
         <v>101</v>
       </c>
       <c r="M20" s="25" t="s">
-        <v>183</v>
+        <v>167</v>
       </c>
     </row>
     <row r="21" spans="3:13" x14ac:dyDescent="0.2">
@@ -2171,8 +2170,8 @@
       <c r="F21" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="M21" t="s">
-        <v>197</v>
+      <c r="M21" s="25" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="22" spans="3:13" x14ac:dyDescent="0.2">
@@ -2188,6 +2187,9 @@
       <c r="H22" t="s">
         <v>103</v>
       </c>
+      <c r="M22" t="s">
+        <v>193</v>
+      </c>
     </row>
     <row r="23" spans="3:13" x14ac:dyDescent="0.2">
       <c r="D23" s="24" t="s">
@@ -2253,7 +2255,7 @@
         <v>97</v>
       </c>
       <c r="M29" s="1" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
     </row>
     <row r="30" spans="3:13" x14ac:dyDescent="0.2">
@@ -2265,7 +2267,7 @@
         <v>71</v>
       </c>
       <c r="M30" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
     </row>
     <row r="31" spans="3:13" x14ac:dyDescent="0.2">
@@ -2299,7 +2301,7 @@
         <v>71</v>
       </c>
       <c r="M32" t="s">
-        <v>210</v>
+        <v>201</v>
       </c>
     </row>
     <row r="33" spans="3:13" x14ac:dyDescent="0.2">
@@ -2313,7 +2315,7 @@
         <v>71</v>
       </c>
       <c r="M33" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
     </row>
     <row r="34" spans="3:13" x14ac:dyDescent="0.2">
@@ -2333,7 +2335,7 @@
         <v>71</v>
       </c>
       <c r="M34" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="35" spans="3:13" x14ac:dyDescent="0.2">
@@ -2344,7 +2346,7 @@
         <v>89</v>
       </c>
       <c r="M35" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
     </row>
     <row r="36" spans="3:13" x14ac:dyDescent="0.2">
@@ -2352,7 +2354,7 @@
         <v>118</v>
       </c>
       <c r="M36" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="37" spans="3:13" x14ac:dyDescent="0.2">
@@ -2365,9 +2367,6 @@
       <c r="H37" t="s">
         <v>122</v>
       </c>
-      <c r="M37" t="s">
-        <v>215</v>
-      </c>
     </row>
     <row r="38" spans="3:13" x14ac:dyDescent="0.2">
       <c r="E38" t="s">
@@ -2382,7 +2381,7 @@
     </row>
     <row r="39" spans="3:13" x14ac:dyDescent="0.2">
       <c r="M39" s="1" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
     </row>
     <row r="40" spans="3:13" x14ac:dyDescent="0.2">
@@ -2390,7 +2389,7 @@
         <v>124</v>
       </c>
       <c r="M40" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
     </row>
     <row r="41" spans="3:13" x14ac:dyDescent="0.2">
@@ -2519,7 +2518,7 @@
       </c>
       <c r="F55" s="2"/>
       <c r="H55" s="11" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="56" spans="4:12" x14ac:dyDescent="0.2">
@@ -2581,60 +2580,56 @@
         <v>145</v>
       </c>
     </row>
-    <row r="65" spans="2:10" x14ac:dyDescent="0.2">
+    <row r="65" spans="2:23" x14ac:dyDescent="0.2">
       <c r="C65" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="66" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="D66" t="s">
+        <v>211</v>
+      </c>
+      <c r="F66" s="24" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="67" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="D67" t="s">
+        <v>161</v>
+      </c>
+      <c r="E67" t="s">
         <v>160</v>
-      </c>
-    </row>
-    <row r="66" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="D66" t="s">
-        <v>161</v>
-      </c>
-      <c r="F66" s="24" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="67" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="D67" t="s">
-        <v>162</v>
       </c>
       <c r="F67" s="2"/>
       <c r="H67" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="68" spans="2:10" x14ac:dyDescent="0.2">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="68" spans="2:23" x14ac:dyDescent="0.2">
       <c r="D68" t="s">
-        <v>164</v>
-      </c>
-      <c r="E68" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F68" s="2"/>
       <c r="H68" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="69" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="D69" t="s">
-        <v>165</v>
-      </c>
-      <c r="F69" s="2"/>
+        <v>171</v>
+      </c>
+    </row>
+    <row r="69" spans="2:23" x14ac:dyDescent="0.2">
       <c r="H69" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="71" spans="2:10" ht="21" x14ac:dyDescent="0.25">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="71" spans="2:23" ht="21" x14ac:dyDescent="0.25">
       <c r="B71" s="18" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="72" spans="2:10" x14ac:dyDescent="0.2">
+    <row r="72" spans="2:23" x14ac:dyDescent="0.2">
       <c r="C72" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="73" spans="2:10" x14ac:dyDescent="0.2">
+    <row r="73" spans="2:23" x14ac:dyDescent="0.2">
       <c r="D73" t="s">
         <v>87</v>
       </c>
@@ -2643,64 +2638,103 @@
         <v>148</v>
       </c>
     </row>
-    <row r="74" spans="2:10" x14ac:dyDescent="0.2">
+    <row r="74" spans="2:23" x14ac:dyDescent="0.2">
       <c r="D74" s="24" t="s">
         <v>88</v>
       </c>
       <c r="E74" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="J74" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="75" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="J74" s="29" t="s">
+        <v>173</v>
+      </c>
+      <c r="K74" s="29"/>
+      <c r="L74" s="29"/>
+      <c r="M74" s="29"/>
+      <c r="N74" s="29"/>
+      <c r="O74" s="29"/>
+      <c r="P74" s="29"/>
+      <c r="Q74" s="29"/>
+      <c r="R74" s="29"/>
+      <c r="S74" s="29"/>
+      <c r="T74" s="29"/>
+      <c r="U74" s="29"/>
+    </row>
+    <row r="75" spans="2:23" x14ac:dyDescent="0.2">
       <c r="C75" t="s">
         <v>90</v>
       </c>
       <c r="D75" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="J75" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="76" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="J75" s="29" t="s">
+        <v>212</v>
+      </c>
+      <c r="K75" s="29"/>
+      <c r="L75" s="29"/>
+      <c r="M75" s="29"/>
+      <c r="N75" s="29"/>
+      <c r="O75" s="29"/>
+      <c r="P75" s="29"/>
+      <c r="Q75" s="29"/>
+      <c r="R75" s="29"/>
+      <c r="S75" s="29"/>
+      <c r="T75" s="29"/>
+      <c r="U75" s="29"/>
+    </row>
+    <row r="76" spans="2:23" x14ac:dyDescent="0.2">
       <c r="C76" t="s">
         <v>149</v>
       </c>
       <c r="D76" t="s">
         <v>152</v>
       </c>
-      <c r="J76" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="77" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="J76" s="29" t="s">
+        <v>153</v>
+      </c>
+      <c r="K76" s="29"/>
+      <c r="L76" s="29"/>
+      <c r="M76" s="29"/>
+      <c r="N76" s="29"/>
+    </row>
+    <row r="77" spans="2:23" x14ac:dyDescent="0.2">
       <c r="C77" t="s">
         <v>150</v>
       </c>
-      <c r="J77" t="s">
+      <c r="J77" s="29" t="s">
+        <v>154</v>
+      </c>
+      <c r="K77" s="29"/>
+      <c r="L77" s="29"/>
+      <c r="M77" s="29"/>
+      <c r="N77" s="29"/>
+      <c r="O77" s="29"/>
+      <c r="P77" s="29"/>
+      <c r="Q77" s="29"/>
+      <c r="R77" s="29"/>
+      <c r="S77" s="29"/>
+      <c r="T77" s="29"/>
+      <c r="U77" s="29"/>
+      <c r="V77" s="29"/>
+      <c r="W77" s="29"/>
+    </row>
+    <row r="78" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="D78" s="24" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="78" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="D78" s="24" t="s">
+      <c r="E78" s="24" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="79" spans="2:23" x14ac:dyDescent="0.2">
+      <c r="D79" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="E78" s="24" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="79" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="D79" s="2" t="s">
+      <c r="E79" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="E79" s="2" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="80" spans="2:10" x14ac:dyDescent="0.2">
+    </row>
+    <row r="80" spans="2:23" x14ac:dyDescent="0.2">
       <c r="C80" t="s">
         <v>151</v>
       </c>
@@ -2723,12 +2757,12 @@
     </row>
     <row r="84" spans="2:12" ht="21" x14ac:dyDescent="0.25">
       <c r="B84" s="18" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
     </row>
     <row r="85" spans="2:12" x14ac:dyDescent="0.2">
       <c r="C85" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
     </row>
     <row r="86" spans="2:12" x14ac:dyDescent="0.2">
@@ -2749,7 +2783,7 @@
     </row>
     <row r="88" spans="2:12" x14ac:dyDescent="0.2">
       <c r="D88" s="24" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="E88" s="24" t="s">
         <v>89</v>
@@ -2760,7 +2794,7 @@
     </row>
     <row r="89" spans="2:12" x14ac:dyDescent="0.2">
       <c r="D89" s="24" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="E89" s="24" t="s">
         <v>89</v>
@@ -2771,7 +2805,7 @@
     </row>
     <row r="90" spans="2:12" x14ac:dyDescent="0.2">
       <c r="D90" s="24" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="E90" s="24" t="s">
         <v>89</v>
@@ -2782,20 +2816,20 @@
     </row>
     <row r="91" spans="2:12" x14ac:dyDescent="0.2">
       <c r="D91" s="24" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="G91" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
     </row>
     <row r="92" spans="2:12" x14ac:dyDescent="0.2">
       <c r="E92" s="24" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
     </row>
     <row r="93" spans="2:12" x14ac:dyDescent="0.2">
       <c r="F93" s="24" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="G93" s="24" t="s">
         <v>89</v>
@@ -2803,7 +2837,7 @@
     </row>
     <row r="94" spans="2:12" x14ac:dyDescent="0.2">
       <c r="F94" s="24" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="G94" s="24" t="s">
         <v>89</v>
@@ -2811,13 +2845,13 @@
     </row>
     <row r="95" spans="2:12" x14ac:dyDescent="0.2">
       <c r="E95" s="24" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="F95" s="24" t="s">
         <v>89</v>
       </c>
       <c r="G95" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="L95" s="27" t="s">
         <v>97</v>
@@ -2825,12 +2859,12 @@
     </row>
     <row r="96" spans="2:12" x14ac:dyDescent="0.2">
       <c r="D96" s="1" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
     </row>
     <row r="97" spans="3:5" x14ac:dyDescent="0.2">
       <c r="E97" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="98" spans="3:5" x14ac:dyDescent="0.2">
@@ -2840,22 +2874,22 @@
     </row>
     <row r="99" spans="3:5" x14ac:dyDescent="0.2">
       <c r="D99" s="1" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
     </row>
     <row r="100" spans="3:5" x14ac:dyDescent="0.2">
       <c r="D100" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
     </row>
     <row r="101" spans="3:5" x14ac:dyDescent="0.2">
       <c r="D101" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
     </row>
     <row r="102" spans="3:5" x14ac:dyDescent="0.2">
       <c r="C102" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
     </row>
     <row r="103" spans="3:5" x14ac:dyDescent="0.2">
@@ -2870,12 +2904,12 @@
     </row>
     <row r="105" spans="3:5" x14ac:dyDescent="0.2">
       <c r="D105" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
     </row>
     <row r="106" spans="3:5" x14ac:dyDescent="0.2">
       <c r="D106" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="107" spans="3:5" x14ac:dyDescent="0.2">
@@ -2890,12 +2924,12 @@
     </row>
     <row r="109" spans="3:5" x14ac:dyDescent="0.2">
       <c r="D109" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
     </row>
     <row r="110" spans="3:5" x14ac:dyDescent="0.2">
       <c r="D110" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
     </row>
     <row r="111" spans="3:5" x14ac:dyDescent="0.2">
@@ -2905,20 +2939,20 @@
     </row>
     <row r="112" spans="3:5" x14ac:dyDescent="0.2">
       <c r="D112" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
     </row>
     <row r="113" spans="3:5" x14ac:dyDescent="0.2">
       <c r="D113" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="E113" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="114" spans="3:5" x14ac:dyDescent="0.2">
       <c r="E114" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="115" spans="3:5" x14ac:dyDescent="0.2">
@@ -2931,7 +2965,7 @@
         <v>87</v>
       </c>
       <c r="E116" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="117" spans="3:5" x14ac:dyDescent="0.2">
@@ -2939,7 +2973,7 @@
         <v>88</v>
       </c>
       <c r="E117" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added updated summary and draft 6
</commit_message>
<xml_diff>
--- a/SUMMARY.xlsx
+++ b/SUMMARY.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amartyn/MPIPZ/amartyn/CSSP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC609FEA-0CCE-F549-8984-DD5F590A3FF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4037C75-AE02-E24C-AC7A-D6D4CB112AC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13780" yWindow="1820" windowWidth="23340" windowHeight="17240" activeTab="2" xr2:uid="{3CB25A69-F844-9241-B587-A0F2F035342F}"/>
+    <workbookView xWindow="0" yWindow="720" windowWidth="29400" windowHeight="18400" activeTab="2" xr2:uid="{3CB25A69-F844-9241-B587-A0F2F035342F}"/>
   </bookViews>
   <sheets>
     <sheet name="summary" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="278">
   <si>
     <t>A</t>
   </si>
@@ -471,9 +471,6 @@
     <t>9_suppl_tables</t>
   </si>
   <si>
-    <t>&gt;&gt; supplementary table missing  (DA isolates incl. taxonomy, abundance in genotype-compartment-soil combinations for Lotus and Hordeum separately)</t>
-  </si>
-  <si>
     <t>2_root_exudates</t>
   </si>
   <si>
@@ -793,13 +790,127 @@
   </si>
   <si>
     <t>&gt; literature added properly</t>
+  </si>
+  <si>
+    <t>Supplementary Table 8</t>
+  </si>
+  <si>
+    <t>Supplementary Table 9</t>
+  </si>
+  <si>
+    <t>&gt; change A</t>
+  </si>
+  <si>
+    <t>&gt; make figure sharp</t>
+  </si>
+  <si>
+    <t>&gt; remove text in A</t>
+  </si>
+  <si>
+    <t>&gt;&gt; supplementary table MODIFY  (DA isolates incl. taxonomy, abundance in genotype-compartment-soil combinations for Lotus and Hordeum separately)</t>
+  </si>
+  <si>
+    <t>&gt;&gt; combine in one Excel file (DA Lotus and DA Hordeum outputs &gt; overview and detailed tables)</t>
+  </si>
+  <si>
+    <t>&gt; modify Excel sheets (spread info among columns)</t>
+  </si>
+  <si>
+    <t>&gt; DA number off by one in Lotus</t>
+  </si>
+  <si>
+    <t>&gt; change "Abscisic acid"</t>
+  </si>
+  <si>
+    <t>&gt; y axis</t>
+  </si>
+  <si>
+    <t>&gt; Ib add updated files if needed</t>
+  </si>
+  <si>
+    <t>(&gt; Ib add updated files if needed)</t>
+  </si>
+  <si>
+    <t>Supplementary Figure 7</t>
+  </si>
+  <si>
+    <t>&gt; ANNA check</t>
+  </si>
+  <si>
+    <t>&gt; ANNA make Fig. (bubble plot with all compartments)</t>
+  </si>
+  <si>
+    <t>&gt; update workflow and rem. nodule part</t>
+  </si>
+  <si>
+    <t>ANNA</t>
+  </si>
+  <si>
+    <t>IB</t>
+  </si>
+  <si>
+    <t>Anna make caption for rest</t>
+  </si>
+  <si>
+    <r>
+      <t>ASVs not matching any member of the SynCom reference set were removed prior to downstream analysis.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t> </t>
+    </r>
+  </si>
+  <si>
+    <t>additional comments:</t>
+  </si>
+  <si>
+    <t>SynCom:</t>
+  </si>
+  <si>
+    <t>Root exudates:</t>
+  </si>
+  <si>
+    <r>
+      <t>The results of these tests were displayed in a volcano plot, with metabolites with a log-fold effect size with magnitude greater than 30 omitted for visual purposes. A bubble plot summarises the results by ClassyFire class, where only classes with at least two metabolites are differentially exudated in at least one mutant compared to WT</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+  </si>
+  <si>
+    <t>Ib: Figure 3 (prediction), Suppl. Table 2 (Indicator ASVs), Fig. 5 (root ex), Suppl. Fig. 5, Suppl. Tables 4,5</t>
+  </si>
+  <si>
+    <t>&gt; change significance testing (use WT as reference), adjust text in draft 6 (see comment)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -836,8 +947,29 @@
       <name val="Helvetica"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -907,6 +1039,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1029,7 +1167,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -1067,6 +1205,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="12" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2079,7 +2223,7 @@
         <v>8</v>
       </c>
       <c r="L58" s="34" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.2">
@@ -2090,7 +2234,7 @@
         <v>9</v>
       </c>
       <c r="L59" s="34" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.2">
@@ -2120,7 +2264,7 @@
   <sheetData>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
@@ -2163,7 +2307,7 @@
         <v>89</v>
       </c>
       <c r="M7" s="29" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="N7" s="28"/>
       <c r="O7" s="28"/>
@@ -2174,7 +2318,7 @@
         <v>90</v>
       </c>
       <c r="M8" s="25" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.2">
@@ -2185,7 +2329,7 @@
         <v>89</v>
       </c>
       <c r="M9" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.2">
@@ -2196,7 +2340,7 @@
         <v>89</v>
       </c>
       <c r="M10" s="28" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="N10" s="28"/>
       <c r="O10" s="28"/>
@@ -2225,7 +2369,7 @@
         <v>93</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
@@ -2236,7 +2380,7 @@
         <v>89</v>
       </c>
       <c r="M14" s="25" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
@@ -2253,7 +2397,7 @@
         <v>94</v>
       </c>
       <c r="M15" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.2">
@@ -2269,7 +2413,7 @@
         <v>95</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="18" spans="3:13" x14ac:dyDescent="0.2">
@@ -2283,7 +2427,7 @@
         <v>97</v>
       </c>
       <c r="M18" s="25" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="19" spans="3:13" x14ac:dyDescent="0.2">
@@ -2294,7 +2438,7 @@
         <v>89</v>
       </c>
       <c r="M19" s="25" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="20" spans="3:13" x14ac:dyDescent="0.2">
@@ -2302,7 +2446,7 @@
         <v>101</v>
       </c>
       <c r="M20" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="21" spans="3:13" x14ac:dyDescent="0.2">
@@ -2336,7 +2480,7 @@
         <v>89</v>
       </c>
       <c r="H23" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="24" spans="3:13" x14ac:dyDescent="0.2">
@@ -2350,7 +2494,7 @@
         <v>89</v>
       </c>
       <c r="H24" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="25" spans="3:13" x14ac:dyDescent="0.2">
@@ -2394,7 +2538,7 @@
         <v>97</v>
       </c>
       <c r="M29" s="1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="30" spans="3:13" x14ac:dyDescent="0.2">
@@ -2406,7 +2550,7 @@
         <v>71</v>
       </c>
       <c r="M30" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="31" spans="3:13" x14ac:dyDescent="0.2">
@@ -2423,7 +2567,7 @@
         <v>71</v>
       </c>
       <c r="M31" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="32" spans="3:13" x14ac:dyDescent="0.2">
@@ -2440,7 +2584,7 @@
         <v>71</v>
       </c>
       <c r="M32" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="33" spans="3:13" x14ac:dyDescent="0.2">
@@ -2454,7 +2598,7 @@
         <v>71</v>
       </c>
       <c r="M33" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="34" spans="3:13" x14ac:dyDescent="0.2">
@@ -2471,7 +2615,7 @@
         <v>115</v>
       </c>
       <c r="M34" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="35" spans="3:13" x14ac:dyDescent="0.2">
@@ -2482,7 +2626,7 @@
         <v>89</v>
       </c>
       <c r="M35" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="36" spans="3:13" x14ac:dyDescent="0.2">
@@ -2514,7 +2658,7 @@
     </row>
     <row r="39" spans="3:13" x14ac:dyDescent="0.2">
       <c r="M39" s="1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="40" spans="3:13" x14ac:dyDescent="0.2">
@@ -2522,7 +2666,7 @@
         <v>123</v>
       </c>
       <c r="M40" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="41" spans="3:13" x14ac:dyDescent="0.2">
@@ -2651,7 +2795,7 @@
       </c>
       <c r="F55" s="2"/>
       <c r="H55" s="11" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="56" spans="4:12" x14ac:dyDescent="0.2">
@@ -2710,17 +2854,22 @@
       </c>
       <c r="E62" s="2"/>
       <c r="H62" t="s">
-        <v>144</v>
+        <v>256</v>
+      </c>
+    </row>
+    <row r="63" spans="4:12" x14ac:dyDescent="0.2">
+      <c r="H63" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="65" spans="2:23" x14ac:dyDescent="0.2">
       <c r="C65" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="66" spans="2:23" x14ac:dyDescent="0.2">
       <c r="D66" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F66" s="24" t="s">
         <v>89</v>
@@ -2728,38 +2877,38 @@
     </row>
     <row r="67" spans="2:23" x14ac:dyDescent="0.2">
       <c r="D67" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E67" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F67" s="2"/>
       <c r="H67" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="68" spans="2:23" x14ac:dyDescent="0.2">
       <c r="D68" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F68" s="2"/>
       <c r="H68" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="69" spans="2:23" x14ac:dyDescent="0.2">
       <c r="H69" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="71" spans="2:23" ht="21" x14ac:dyDescent="0.25">
       <c r="B71" s="18" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="72" spans="2:23" x14ac:dyDescent="0.2">
       <c r="C72" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="73" spans="2:23" x14ac:dyDescent="0.2">
@@ -2768,7 +2917,7 @@
       </c>
       <c r="E73" s="2"/>
       <c r="F73" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="74" spans="2:23" x14ac:dyDescent="0.2">
@@ -2779,7 +2928,7 @@
         <v>89</v>
       </c>
       <c r="J74" s="28" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="K74" s="28"/>
       <c r="L74" s="28"/>
@@ -2801,7 +2950,7 @@
         <v>89</v>
       </c>
       <c r="J75" s="28" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="K75" s="28"/>
       <c r="L75" s="28"/>
@@ -2817,13 +2966,13 @@
     </row>
     <row r="76" spans="2:23" x14ac:dyDescent="0.2">
       <c r="C76" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D76" t="s">
+        <v>150</v>
+      </c>
+      <c r="J76" s="28" t="s">
         <v>151</v>
-      </c>
-      <c r="J76" s="28" t="s">
-        <v>152</v>
       </c>
       <c r="K76" s="28"/>
       <c r="L76" s="28"/>
@@ -2832,10 +2981,10 @@
     </row>
     <row r="77" spans="2:23" x14ac:dyDescent="0.2">
       <c r="C77" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J77" s="28" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="K77" s="28"/>
       <c r="L77" s="28"/>
@@ -2853,7 +3002,7 @@
     </row>
     <row r="78" spans="2:23" x14ac:dyDescent="0.2">
       <c r="D78" s="24" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E78" s="24" t="s">
         <v>89</v>
@@ -2861,15 +3010,15 @@
     </row>
     <row r="79" spans="2:23" x14ac:dyDescent="0.2">
       <c r="D79" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="E79" s="2" t="s">
         <v>155</v>
-      </c>
-      <c r="E79" s="2" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="80" spans="2:23" x14ac:dyDescent="0.2">
       <c r="C80" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="81" spans="2:12" x14ac:dyDescent="0.2">
@@ -2890,12 +3039,12 @@
     </row>
     <row r="84" spans="2:12" ht="21" x14ac:dyDescent="0.25">
       <c r="B84" s="18" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="85" spans="2:12" x14ac:dyDescent="0.2">
       <c r="C85" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="86" spans="2:12" x14ac:dyDescent="0.2">
@@ -2916,7 +3065,7 @@
     </row>
     <row r="88" spans="2:12" x14ac:dyDescent="0.2">
       <c r="D88" s="24" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E88" s="24" t="s">
         <v>89</v>
@@ -2927,7 +3076,7 @@
     </row>
     <row r="89" spans="2:12" x14ac:dyDescent="0.2">
       <c r="D89" s="24" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E89" s="24" t="s">
         <v>89</v>
@@ -2938,7 +3087,7 @@
     </row>
     <row r="90" spans="2:12" x14ac:dyDescent="0.2">
       <c r="D90" s="24" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E90" s="24" t="s">
         <v>89</v>
@@ -2949,20 +3098,20 @@
     </row>
     <row r="91" spans="2:12" x14ac:dyDescent="0.2">
       <c r="D91" s="24" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G91" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="92" spans="2:12" x14ac:dyDescent="0.2">
       <c r="E92" s="24" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="93" spans="2:12" x14ac:dyDescent="0.2">
       <c r="F93" s="24" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="G93" s="24" t="s">
         <v>89</v>
@@ -2970,7 +3119,7 @@
     </row>
     <row r="94" spans="2:12" x14ac:dyDescent="0.2">
       <c r="F94" s="24" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="G94" s="24" t="s">
         <v>89</v>
@@ -2978,13 +3127,13 @@
     </row>
     <row r="95" spans="2:12" x14ac:dyDescent="0.2">
       <c r="E95" s="24" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F95" s="24" t="s">
         <v>89</v>
       </c>
       <c r="G95" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="L95" s="27" t="s">
         <v>97</v>
@@ -2992,12 +3141,12 @@
     </row>
     <row r="96" spans="2:12" x14ac:dyDescent="0.2">
       <c r="D96" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="97" spans="3:5" x14ac:dyDescent="0.2">
       <c r="E97" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="98" spans="3:5" x14ac:dyDescent="0.2">
@@ -3007,22 +3156,22 @@
     </row>
     <row r="99" spans="3:5" x14ac:dyDescent="0.2">
       <c r="D99" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="100" spans="3:5" x14ac:dyDescent="0.2">
       <c r="D100" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="101" spans="3:5" x14ac:dyDescent="0.2">
       <c r="D101" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="102" spans="3:5" x14ac:dyDescent="0.2">
       <c r="C102" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="103" spans="3:5" x14ac:dyDescent="0.2">
@@ -3037,12 +3186,12 @@
     </row>
     <row r="105" spans="3:5" x14ac:dyDescent="0.2">
       <c r="D105" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="106" spans="3:5" x14ac:dyDescent="0.2">
       <c r="D106" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="107" spans="3:5" x14ac:dyDescent="0.2">
@@ -3057,40 +3206,40 @@
     </row>
     <row r="109" spans="3:5" x14ac:dyDescent="0.2">
       <c r="D109" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="110" spans="3:5" x14ac:dyDescent="0.2">
       <c r="D110" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="111" spans="3:5" x14ac:dyDescent="0.2">
       <c r="C111" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="112" spans="3:5" x14ac:dyDescent="0.2">
       <c r="D112" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="113" spans="3:5" x14ac:dyDescent="0.2">
       <c r="D113" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="E113" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="114" spans="3:5" x14ac:dyDescent="0.2">
       <c r="E114" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="115" spans="3:5" x14ac:dyDescent="0.2">
       <c r="C115" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="116" spans="3:5" x14ac:dyDescent="0.2">
@@ -3098,7 +3247,7 @@
         <v>87</v>
       </c>
       <c r="E116" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="117" spans="3:5" x14ac:dyDescent="0.2">
@@ -3106,7 +3255,7 @@
         <v>88</v>
       </c>
       <c r="E117" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -3116,169 +3265,272 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAEB7DF4-A933-4345-8067-1627111DF6E1}">
-  <dimension ref="B3:H22"/>
+  <dimension ref="B3:I34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35.1640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="20.83203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="76.1640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="20.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="19.5" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="4" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B4" s="31" t="s">
         <v>214</v>
       </c>
-    </row>
-    <row r="4" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B4" t="s">
+      <c r="C4" s="31" t="s">
+        <v>217</v>
+      </c>
+      <c r="G4" s="31" t="s">
+        <v>226</v>
+      </c>
+      <c r="H4" s="31" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="5" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B5" s="35" t="s">
         <v>215</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C5" s="35" t="s">
         <v>218</v>
       </c>
-      <c r="G4" t="s">
-        <v>227</v>
-      </c>
-      <c r="H4" t="s">
+      <c r="D5" s="35" t="s">
+        <v>253</v>
+      </c>
+      <c r="E5" s="31" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="5" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B5" t="s">
+    <row r="6" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B6" s="31" t="s">
         <v>216</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C6" s="31" t="s">
+        <v>221</v>
+      </c>
+      <c r="G6" s="31" t="s">
+        <v>229</v>
+      </c>
+      <c r="H6" s="31" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B7" s="35" t="s">
+        <v>220</v>
+      </c>
+      <c r="C7" s="35" t="s">
         <v>219</v>
       </c>
-      <c r="E5" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B6" t="s">
-        <v>217</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="D7" s="35" t="s">
+        <v>254</v>
+      </c>
+      <c r="E7" s="31" t="s">
+        <v>231</v>
+      </c>
+      <c r="G7" s="35" t="s">
+        <v>235</v>
+      </c>
+      <c r="H7" s="35" t="s">
+        <v>234</v>
+      </c>
+      <c r="I7" s="35" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B8" s="35"/>
+      <c r="C8" s="35"/>
+      <c r="D8" s="35" t="s">
+        <v>255</v>
+      </c>
+      <c r="E8" s="31" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="E9" s="31" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="10" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B10" s="6" t="s">
         <v>222</v>
       </c>
-      <c r="G6" t="s">
-        <v>230</v>
-      </c>
-      <c r="H6" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="7" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B7" t="s">
-        <v>221</v>
-      </c>
-      <c r="C7" t="s">
-        <v>220</v>
-      </c>
-      <c r="E7" t="s">
-        <v>232</v>
-      </c>
-      <c r="G7" t="s">
+      <c r="C10" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="E10" s="6" t="s">
         <v>236</v>
       </c>
-      <c r="H7" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="8" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="E8" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="E9" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B10" t="s">
+      <c r="F10" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="12" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="13" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B13" s="35" t="s">
         <v>223</v>
       </c>
-      <c r="C10" t="s">
-        <v>226</v>
-      </c>
-      <c r="E10" t="s">
-        <v>237</v>
-      </c>
-      <c r="G10" t="s">
+      <c r="C13" s="35" t="s">
+        <v>224</v>
+      </c>
+      <c r="D13" s="35" t="s">
+        <v>267</v>
+      </c>
+      <c r="E13" s="35" t="s">
         <v>242</v>
       </c>
-      <c r="H10" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="G11" t="s">
+      <c r="F13" s="35" t="s">
+        <v>265</v>
+      </c>
+      <c r="G13" s="35" t="s">
         <v>240</v>
       </c>
-      <c r="H11" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B12" t="s">
-        <v>224</v>
-      </c>
-      <c r="C12" t="s">
-        <v>225</v>
-      </c>
-      <c r="E12" t="s">
+      <c r="H13" s="35" t="s">
         <v>243</v>
       </c>
-      <c r="G12" t="s">
-        <v>241</v>
-      </c>
-      <c r="H12" t="s">
+    </row>
+    <row r="14" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B14" s="35"/>
+      <c r="C14" s="35"/>
+      <c r="D14" s="35"/>
+      <c r="E14" s="35" t="s">
+        <v>264</v>
+      </c>
+      <c r="F14" s="35" t="s">
+        <v>266</v>
+      </c>
+      <c r="G14" s="35" t="s">
+        <v>245</v>
+      </c>
+      <c r="H14" s="35" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="G13" t="s">
+    <row r="16" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="G16" s="31" t="s">
+        <v>251</v>
+      </c>
+      <c r="H16" s="31" t="s">
         <v>246</v>
       </c>
-      <c r="H13" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="15" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="G15" s="31" t="s">
-        <v>246</v>
-      </c>
-      <c r="H15" s="31" t="s">
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="G17" s="31" t="s">
+        <v>252</v>
+      </c>
+      <c r="H17" s="31" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="16" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="G16" s="31" t="s">
-        <v>246</v>
-      </c>
-      <c r="H16" s="31" t="s">
+    <row r="20" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B20" t="s">
         <v>248</v>
       </c>
-    </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B20" t="s">
+      <c r="D20" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="D21" s="35" t="s">
+        <v>270</v>
+      </c>
+      <c r="G21" s="36"/>
+      <c r="H21" s="36"/>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="G22" s="36"/>
+    </row>
+    <row r="23" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="D23" s="38" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="24" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="D24" t="s">
+        <v>273</v>
+      </c>
+      <c r="E24" s="36" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="25" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="D25" t="s">
+        <v>274</v>
+      </c>
+      <c r="E25" s="36" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="28" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B28" s="35" t="s">
         <v>249</v>
       </c>
-    </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B21" t="s">
+      <c r="F28" s="36"/>
+    </row>
+    <row r="29" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B29" s="35" t="s">
         <v>250</v>
       </c>
-    </row>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B22" t="s">
-        <v>251</v>
+      <c r="F29" s="37"/>
+    </row>
+    <row r="33" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B33" s="35" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="34" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="B34" s="6" t="s">
+        <v>269</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added updated summary file and draft 6 with captions
</commit_message>
<xml_diff>
--- a/SUMMARY.xlsx
+++ b/SUMMARY.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amartyn/MPIPZ/amartyn/CSSP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50B9C76C-C443-EC48-80EB-6DAFF5E2C5E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0BFB6C0-8E6D-094A-9BF2-5EA168A1521A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8480" yWindow="740" windowWidth="20920" windowHeight="17160" activeTab="2" xr2:uid="{3CB25A69-F844-9241-B587-A0F2F035342F}"/>
+    <workbookView xWindow="14280" yWindow="860" windowWidth="15100" windowHeight="17160" activeTab="2" xr2:uid="{3CB25A69-F844-9241-B587-A0F2F035342F}"/>
   </bookViews>
   <sheets>
     <sheet name="summary" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="458" uniqueCount="278">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="267">
   <si>
     <t>A</t>
   </si>
@@ -802,21 +802,6 @@
   </si>
   <si>
     <t>&gt;&gt; combine in one Excel file (DA Lotus and DA Hordeum outputs &gt; overview and detailed tables)</t>
-  </si>
-  <si>
-    <t>&gt; DA number off by one in Lotus</t>
-  </si>
-  <si>
-    <t>&gt; change "Abscisic acid"</t>
-  </si>
-  <si>
-    <t>&gt; y axis</t>
-  </si>
-  <si>
-    <t>&gt; Ib add updated files if needed</t>
-  </si>
-  <si>
-    <t>(&gt; Ib add updated files if needed)</t>
   </si>
   <si>
     <t>Supplementary Figure 7</t>
@@ -861,49 +846,10 @@
     <t>SynCom:</t>
   </si>
   <si>
-    <t>Root exudates:</t>
-  </si>
-  <si>
-    <r>
-      <t>The results of these tests were displayed in a volcano plot, with metabolites with a log-fold effect size with magnitude greater than 30 omitted for visual purposes. A bubble plot summarises the results by ClassyFire class, where only classes with at least two metabolites are differentially exudated in at least one mutant compared to WT</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-  </si>
-  <si>
     <t>Ib: Figure 3 (prediction), Suppl. Table 2 (Indicator ASVs), Fig. 5 (root ex), Suppl. Fig. 5, Suppl. Tables 4,5</t>
   </si>
   <si>
-    <t>&gt; change significance testing (use WT as reference), adjust text in draft 6 (see comment)</t>
-  </si>
-  <si>
     <t>&gt; quality problem, but cannot fix atm so will keep as is</t>
-  </si>
-  <si>
-    <t>ALSO: add info whether NPC classifier or Classyfire used (in main figure Classyfire and in suppl. NPC)</t>
-  </si>
-  <si>
-    <t>ALSO: change Abs. acid molecule header to: Abscisic acid; and make headers with mutant names italic</t>
-  </si>
-  <si>
-    <t>Ib check whether all highlighted compounds in suppl. Table (except for last metabolite &gt; supposed to be in plot)</t>
   </si>
 </sst>
 </file>
@@ -1173,7 +1119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -1204,7 +1150,6 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="12" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
@@ -1213,11 +1158,16 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2226,10 +2176,10 @@
       <c r="G58" t="s">
         <v>63</v>
       </c>
-      <c r="K58" s="31">
+      <c r="K58" s="30">
         <v>8</v>
       </c>
-      <c r="L58" s="32" t="s">
+      <c r="L58" s="31" t="s">
         <v>211</v>
       </c>
     </row>
@@ -2237,10 +2187,10 @@
       <c r="B59" t="s">
         <v>23</v>
       </c>
-      <c r="K59" s="31">
+      <c r="K59" s="30">
         <v>9</v>
       </c>
-      <c r="L59" s="32" t="s">
+      <c r="L59" s="31" t="s">
         <v>212</v>
       </c>
     </row>
@@ -3271,277 +3221,292 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAEB7DF4-A933-4345-8067-1627111DF6E1}">
-  <dimension ref="B3:I34"/>
+  <dimension ref="A3:J34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="47.33203125" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="76.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="20.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8" style="38" customWidth="1"/>
+    <col min="6" max="6" width="20.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="76.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.1640625" style="38" customWidth="1"/>
+    <col min="9" max="9" width="20.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B4" s="39" t="s">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A4" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="B4" s="36" t="s">
         <v>214</v>
       </c>
-      <c r="C4" s="39" t="s">
+      <c r="C4" s="36" t="s">
         <v>217</v>
       </c>
       <c r="D4" t="s">
-        <v>274</v>
-      </c>
-      <c r="G4" s="39" t="s">
+        <v>266</v>
+      </c>
+      <c r="H4" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="I4" s="36" t="s">
         <v>226</v>
       </c>
-      <c r="H4" s="39" t="s">
+      <c r="J4" s="36" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B5" s="39" t="s">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A5" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="B5" s="36" t="s">
         <v>215</v>
       </c>
-      <c r="C5" s="39" t="s">
+      <c r="C5" s="36" t="s">
         <v>218</v>
       </c>
       <c r="D5" t="s">
-        <v>274</v>
-      </c>
-      <c r="E5" s="39" t="s">
+        <v>266</v>
+      </c>
+      <c r="E5" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="F5" s="36" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="6" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B6" s="39" t="s">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="B6" s="36" t="s">
         <v>216</v>
       </c>
-      <c r="C6" s="39" t="s">
+      <c r="C6" s="36" t="s">
         <v>221</v>
       </c>
-      <c r="G6" s="39" t="s">
+      <c r="H6" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="I6" s="36" t="s">
         <v>229</v>
       </c>
-      <c r="H6" s="39" t="s">
+      <c r="J6" s="36" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B7" s="39" t="s">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="B7" s="36" t="s">
         <v>220</v>
       </c>
-      <c r="C7" s="39" t="s">
+      <c r="C7" s="36" t="s">
         <v>219</v>
       </c>
       <c r="D7" t="s">
-        <v>274</v>
-      </c>
-      <c r="E7" s="39" t="s">
+        <v>266</v>
+      </c>
+      <c r="E7" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="F7" s="36" t="s">
         <v>231</v>
       </c>
-      <c r="G7" s="39" t="s">
+      <c r="H7" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="I7" s="36" t="s">
         <v>235</v>
       </c>
-      <c r="H7" s="39" t="s">
+      <c r="J7" s="36" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="E8" s="39" t="s">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E8" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="F8" s="36" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="E9" s="39" t="s">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E9" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="F9" s="36" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B10" s="6" t="s">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A10" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="B10" s="36" t="s">
         <v>222</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="36" t="s">
         <v>225</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="E10" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="F10" s="36" t="s">
+        <v>236</v>
+      </c>
+      <c r="H10" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="I10" s="36" t="s">
+        <v>241</v>
+      </c>
+      <c r="J10" s="36" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H11" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="I11" s="36" t="s">
+        <v>239</v>
+      </c>
+      <c r="J11" s="36" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B13" s="32" t="s">
+        <v>223</v>
+      </c>
+      <c r="C13" s="32" t="s">
+        <v>224</v>
+      </c>
+      <c r="D13" s="32" t="s">
+        <v>258</v>
+      </c>
+      <c r="F13" s="32" t="s">
+        <v>242</v>
+      </c>
+      <c r="G13" s="32" t="s">
+        <v>256</v>
+      </c>
+      <c r="I13" s="32" t="s">
+        <v>240</v>
+      </c>
+      <c r="J13" s="32" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B14" s="32"/>
+      <c r="C14" s="32"/>
+      <c r="D14" s="32"/>
+      <c r="F14" s="32" t="s">
         <v>255</v>
       </c>
-      <c r="E10" s="6" t="s">
-        <v>236</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>273</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>241</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>237</v>
-      </c>
-      <c r="I10" s="6" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6" t="s">
-        <v>256</v>
-      </c>
-      <c r="G11" s="6" t="s">
-        <v>239</v>
-      </c>
-      <c r="H11" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="I11" s="6" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6" t="s">
+      <c r="G14" s="32" t="s">
         <v>257</v>
       </c>
-    </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B13" s="33" t="s">
-        <v>223</v>
-      </c>
-      <c r="C13" s="33" t="s">
-        <v>224</v>
-      </c>
-      <c r="D13" s="33" t="s">
-        <v>263</v>
-      </c>
-      <c r="E13" s="33" t="s">
-        <v>242</v>
-      </c>
-      <c r="F13" s="33" t="s">
-        <v>261</v>
-      </c>
-      <c r="G13" s="33" t="s">
-        <v>240</v>
-      </c>
-      <c r="H13" s="33" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="14" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B14" s="33"/>
-      <c r="C14" s="33"/>
-      <c r="D14" s="33"/>
-      <c r="E14" s="33" t="s">
-        <v>260</v>
-      </c>
-      <c r="F14" s="33" t="s">
-        <v>262</v>
-      </c>
-      <c r="G14" s="33" t="s">
+      <c r="I14" s="32" t="s">
         <v>245</v>
       </c>
-      <c r="H14" s="33" t="s">
+      <c r="J14" s="32" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="16" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="G16" s="30" t="s">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H16" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="I16" s="36" t="s">
         <v>251</v>
       </c>
-      <c r="H16" s="30" t="s">
+      <c r="J16" s="36" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="G17" s="30" t="s">
+    <row r="17" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="H17" s="36" t="s">
+        <v>71</v>
+      </c>
+      <c r="I17" s="36" t="s">
         <v>252</v>
       </c>
-      <c r="H17" s="30" t="s">
+      <c r="J17" s="36" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B20" t="s">
         <v>248</v>
       </c>
-      <c r="D20" s="6" t="s">
-        <v>272</v>
-      </c>
-      <c r="E20" s="6"/>
-      <c r="F20" s="6"/>
-    </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="D21" s="33" t="s">
-        <v>266</v>
-      </c>
-      <c r="G21" s="34"/>
-      <c r="H21" s="34"/>
-    </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="G22" s="34"/>
-    </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="D23" s="36" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="D20" s="36" t="s">
+        <v>265</v>
+      </c>
+      <c r="E20" s="36"/>
+      <c r="F20" s="36"/>
+      <c r="G20" s="36"/>
+    </row>
+    <row r="21" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="D21" s="32" t="s">
+        <v>261</v>
+      </c>
+      <c r="I21" s="33"/>
+      <c r="J21" s="33"/>
+    </row>
+    <row r="22" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="I22" s="33"/>
+    </row>
+    <row r="23" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="D23" s="35" t="s">
+        <v>263</v>
+      </c>
+      <c r="E23" s="41"/>
+    </row>
+    <row r="24" spans="2:10" x14ac:dyDescent="0.2">
       <c r="D24" t="s">
-        <v>269</v>
-      </c>
-      <c r="E24" s="34" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="D25" t="s">
-        <v>270</v>
-      </c>
-      <c r="E25" s="34" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="26" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="E26" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="27" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="E27" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="28" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B28" s="38" t="s">
+        <v>264</v>
+      </c>
+      <c r="F24" s="33" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="25" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="F25" s="33"/>
+    </row>
+    <row r="28" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B28" t="s">
         <v>249</v>
       </c>
-      <c r="E28" t="s">
-        <v>277</v>
-      </c>
-      <c r="F28" s="34"/>
-    </row>
-    <row r="29" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B29" s="39" t="s">
+      <c r="G28" s="33"/>
+      <c r="H28" s="39"/>
+    </row>
+    <row r="29" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B29" s="36" t="s">
         <v>250</v>
       </c>
-      <c r="C29" s="30"/>
-      <c r="F29" s="35"/>
+      <c r="C29" s="36"/>
+      <c r="G29" s="34"/>
+      <c r="H29" s="40"/>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B33" s="33" t="s">
-        <v>264</v>
+      <c r="B33" s="32" t="s">
+        <v>259</v>
       </c>
     </row>
     <row r="34" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B34" s="6" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
SynCom part incl figures and suppl figures and tables
</commit_message>
<xml_diff>
--- a/SUMMARY.xlsx
+++ b/SUMMARY.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amartyn/MPIPZ/amartyn/CSSP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0BFB6C0-8E6D-094A-9BF2-5EA168A1521A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5B3B8A1-1F97-DF41-9D51-D18C25349BDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14280" yWindow="860" windowWidth="15100" windowHeight="17160" activeTab="2" xr2:uid="{3CB25A69-F844-9241-B587-A0F2F035342F}"/>
+    <workbookView minimized="1" xWindow="16620" yWindow="860" windowWidth="19600" windowHeight="18760" activeTab="1" xr2:uid="{3CB25A69-F844-9241-B587-A0F2F035342F}"/>
   </bookViews>
   <sheets>
     <sheet name="summary" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="269">
   <si>
     <t>A</t>
   </si>
@@ -850,6 +850,12 @@
   </si>
   <si>
     <t>&gt; quality problem, but cannot fix atm so will keep as is</t>
+  </si>
+  <si>
+    <t>one sample &lt;1000 &gt; was removed (ccamk rhizo)</t>
+  </si>
+  <si>
+    <t>&gt; for final figure I used Ibs script outputs, but in a separate file I did I calculate cpcoa and pcoa, and my outputs slighlty differ to Ibs &gt;  we need to check this soon!</t>
   </si>
 </sst>
 </file>
@@ -1119,7 +1125,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -1162,12 +1168,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3096,86 +3096,134 @@
       </c>
     </row>
     <row r="96" spans="2:12" x14ac:dyDescent="0.2">
-      <c r="D96" s="1" t="s">
+      <c r="D96" s="26" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="97" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="E97" t="s">
+      <c r="E96" s="24"/>
+    </row>
+    <row r="97" spans="3:7" x14ac:dyDescent="0.2">
+      <c r="D97" s="24"/>
+      <c r="E97" s="24" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="98" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="E98" t="s">
+      <c r="F97" s="24" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="98" spans="3:7" x14ac:dyDescent="0.2">
+      <c r="D98" s="24"/>
+      <c r="E98" s="24" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="99" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="D99" s="1" t="s">
+      <c r="F98" s="24" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="99" spans="3:7" x14ac:dyDescent="0.2">
+      <c r="D99" s="26" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="100" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="D100" t="s">
+      <c r="E99" s="24" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="100" spans="3:7" x14ac:dyDescent="0.2">
+      <c r="D100" s="24" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="101" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="D101" t="s">
+      <c r="E100" s="24" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="101" spans="3:7" x14ac:dyDescent="0.2">
+      <c r="D101" s="24" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="102" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="E101" s="24" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="102" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C102" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="103" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="D103" t="s">
+    <row r="103" spans="3:7" x14ac:dyDescent="0.2">
+      <c r="D103" s="24" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="104" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="D104" t="s">
+      <c r="E103" s="24" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="104" spans="3:7" x14ac:dyDescent="0.2">
+      <c r="D104" s="24" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="105" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="D105" t="s">
+      <c r="E104" s="24" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="105" spans="3:7" x14ac:dyDescent="0.2">
+      <c r="D105" s="24" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="106" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="D106" t="s">
+      <c r="E105" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="G105" s="27" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="106" spans="3:7" x14ac:dyDescent="0.2">
+      <c r="D106" s="24" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="107" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="D107" t="s">
+      <c r="E106" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="G106" s="23" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="107" spans="3:7" x14ac:dyDescent="0.2">
+      <c r="D107" s="24" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="108" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="D108" t="s">
+      <c r="E107" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="G107" s="27" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="108" spans="3:7" x14ac:dyDescent="0.2">
+      <c r="D108" s="26" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="109" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="D109" t="s">
+      <c r="E108" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="G108" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="109" spans="3:7" x14ac:dyDescent="0.2">
+      <c r="D109" s="1" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="110" spans="3:5" x14ac:dyDescent="0.2">
+    <row r="110" spans="3:7" x14ac:dyDescent="0.2">
       <c r="D110" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="111" spans="3:5" x14ac:dyDescent="0.2">
+    <row r="111" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C111" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="112" spans="3:5" x14ac:dyDescent="0.2">
+    <row r="112" spans="3:7" x14ac:dyDescent="0.2">
       <c r="D112" t="s">
         <v>194</v>
       </c>
@@ -3226,10 +3274,10 @@
   <cols>
     <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="47.33203125" customWidth="1"/>
-    <col min="5" max="5" width="8" style="38" customWidth="1"/>
+    <col min="5" max="5" width="8" customWidth="1"/>
     <col min="6" max="6" width="20.83203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="76.1640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.1640625" style="38" customWidth="1"/>
+    <col min="8" max="8" width="8.1640625" customWidth="1"/>
     <col min="9" max="9" width="20.1640625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="21.5" bestFit="1" customWidth="1"/>
   </cols>
@@ -3471,7 +3519,7 @@
       <c r="D23" s="35" t="s">
         <v>263</v>
       </c>
-      <c r="E23" s="41"/>
+      <c r="E23" s="35"/>
     </row>
     <row r="24" spans="2:10" x14ac:dyDescent="0.2">
       <c r="D24" t="s">
@@ -3489,7 +3537,7 @@
         <v>249</v>
       </c>
       <c r="G28" s="33"/>
-      <c r="H28" s="39"/>
+      <c r="H28" s="33"/>
     </row>
     <row r="29" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B29" s="36" t="s">
@@ -3497,7 +3545,7 @@
       </c>
       <c r="C29" s="36"/>
       <c r="G29" s="34"/>
-      <c r="H29" s="40"/>
+      <c r="H29" s="34"/>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B33" s="32" t="s">

</xml_diff>

<commit_message>
added summary file also
</commit_message>
<xml_diff>
--- a/SUMMARY.xlsx
+++ b/SUMMARY.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amartyn/MPIPZ/amartyn/CSSP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5B3B8A1-1F97-DF41-9D51-D18C25349BDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5579AB0-90AA-914C-9844-97B628E8F471}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="16620" yWindow="860" windowWidth="19600" windowHeight="18760" activeTab="1" xr2:uid="{3CB25A69-F844-9241-B587-A0F2F035342F}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" activeTab="2" xr2:uid="{3CB25A69-F844-9241-B587-A0F2F035342F}"/>
   </bookViews>
   <sheets>
     <sheet name="summary" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="270">
   <si>
     <t>A</t>
   </si>
@@ -805,15 +805,6 @@
   </si>
   <si>
     <t>Supplementary Figure 7</t>
-  </si>
-  <si>
-    <t>&gt; ANNA check</t>
-  </si>
-  <si>
-    <t>&gt; ANNA make Fig. (bubble plot with all compartments)</t>
-  </si>
-  <si>
-    <t>&gt; update workflow and rem. nodule part</t>
   </si>
   <si>
     <t>ANNA</t>
@@ -856,6 +847,18 @@
   </si>
   <si>
     <t>&gt; for final figure I used Ibs script outputs, but in a separate file I did I calculate cpcoa and pcoa, and my outputs slighlty differ to Ibs &gt;  we need to check this soon!</t>
+  </si>
+  <si>
+    <t>ALSO! In the DA plots for the SynComs we used MaAsLin2 for sign. Analysis of orders! No where else!</t>
+  </si>
+  <si>
+    <t>MAASLIN2</t>
+  </si>
+  <si>
+    <t>DA plot Lotus with nodule compartment</t>
+  </si>
+  <si>
+    <t>&gt; can be made prettier but ok for now</t>
   </si>
 </sst>
 </file>
@@ -1125,7 +1128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -1168,6 +1171,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2031,6 +2035,7 @@
       <c r="F36" s="12" t="s">
         <v>25</v>
       </c>
+      <c r="G36" s="1"/>
       <c r="H36" s="11"/>
       <c r="I36" s="12" t="s">
         <v>27</v>
@@ -2046,6 +2051,7 @@
       <c r="F37" s="12" t="s">
         <v>45</v>
       </c>
+      <c r="G37" s="1"/>
       <c r="H37" s="11"/>
       <c r="I37" s="20" t="s">
         <v>47</v>
@@ -2066,6 +2072,7 @@
       <c r="F38" s="12" t="s">
         <v>9</v>
       </c>
+      <c r="G38" s="1"/>
       <c r="H38" s="11"/>
       <c r="I38" s="12" t="s">
         <v>48</v>
@@ -2081,15 +2088,26 @@
       <c r="F39" s="15" t="s">
         <v>46</v>
       </c>
+      <c r="G39" s="1"/>
       <c r="H39" s="13"/>
       <c r="I39" s="15" t="s">
         <v>49</v>
       </c>
     </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="H41" s="8">
+        <v>7</v>
+      </c>
+      <c r="I41" s="10" t="s">
+        <v>268</v>
+      </c>
+    </row>
     <row r="42" spans="1:12" ht="21" x14ac:dyDescent="0.25">
       <c r="A42" s="18" t="s">
         <v>61</v>
       </c>
+      <c r="H42" s="13"/>
+      <c r="I42" s="15"/>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
@@ -2211,7 +2229,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05F214DF-3300-D745-A4ED-6415291CCBF0}">
-  <dimension ref="A2:W117"/>
+  <dimension ref="A2:W120"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="18.6640625" bestFit="1" customWidth="1"/>
@@ -3126,6 +3144,9 @@
       <c r="E99" s="24" t="s">
         <v>89</v>
       </c>
+      <c r="G99" s="38" t="s">
+        <v>267</v>
+      </c>
     </row>
     <row r="100" spans="3:7" x14ac:dyDescent="0.2">
       <c r="D100" s="24" t="s">
@@ -3183,7 +3204,7 @@
         <v>89</v>
       </c>
       <c r="G106" s="23" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
     </row>
     <row r="107" spans="3:7" x14ac:dyDescent="0.2">
@@ -3205,17 +3226,26 @@
         <v>89</v>
       </c>
       <c r="G108" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
     </row>
     <row r="109" spans="3:7" x14ac:dyDescent="0.2">
-      <c r="D109" s="1" t="s">
+      <c r="D109" s="26" t="s">
         <v>192</v>
       </c>
+      <c r="E109" s="24" t="s">
+        <v>89</v>
+      </c>
+      <c r="G109" s="38" t="s">
+        <v>267</v>
+      </c>
     </row>
     <row r="110" spans="3:7" x14ac:dyDescent="0.2">
-      <c r="D110" t="s">
+      <c r="D110" s="24" t="s">
         <v>193</v>
+      </c>
+      <c r="E110" s="24" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="111" spans="3:7" x14ac:dyDescent="0.2">
@@ -3224,8 +3254,11 @@
       </c>
     </row>
     <row r="112" spans="3:7" x14ac:dyDescent="0.2">
-      <c r="D112" t="s">
+      <c r="D112" s="24" t="s">
         <v>194</v>
+      </c>
+      <c r="E112" s="24" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="113" spans="3:5" x14ac:dyDescent="0.2">
@@ -3260,6 +3293,11 @@
       </c>
       <c r="E117" s="2" t="s">
         <v>155</v>
+      </c>
+    </row>
+    <row r="120" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C120" s="1" t="s">
+        <v>266</v>
       </c>
     </row>
   </sheetData>
@@ -3298,7 +3336,7 @@
         <v>217</v>
       </c>
       <c r="D4" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="H4" s="36" t="s">
         <v>71</v>
@@ -3321,7 +3359,7 @@
         <v>218</v>
       </c>
       <c r="D5" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="E5" s="36" t="s">
         <v>71</v>
@@ -3361,7 +3399,7 @@
         <v>219</v>
       </c>
       <c r="D7" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="E7" s="36" t="s">
         <v>71</v>
@@ -3433,42 +3471,38 @@
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B13" s="32" t="s">
+      <c r="B13" s="36" t="s">
         <v>223</v>
       </c>
-      <c r="C13" s="32" t="s">
+      <c r="C13" s="36" t="s">
         <v>224</v>
       </c>
-      <c r="D13" s="32" t="s">
-        <v>258</v>
-      </c>
-      <c r="F13" s="32" t="s">
+      <c r="F13" s="36" t="s">
         <v>242</v>
       </c>
-      <c r="G13" s="32" t="s">
-        <v>256</v>
-      </c>
-      <c r="I13" s="32" t="s">
+      <c r="G13" s="36" t="s">
+        <v>269</v>
+      </c>
+      <c r="I13" s="36" t="s">
         <v>240</v>
       </c>
-      <c r="J13" s="32" t="s">
+      <c r="J13" s="36" t="s">
         <v>243</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B14" s="32"/>
-      <c r="C14" s="32"/>
-      <c r="D14" s="32"/>
-      <c r="F14" s="32" t="s">
+      <c r="B14" s="36"/>
+      <c r="C14" s="36"/>
+      <c r="F14" s="36" t="s">
         <v>255</v>
       </c>
-      <c r="G14" s="32" t="s">
-        <v>257</v>
-      </c>
-      <c r="I14" s="32" t="s">
+      <c r="G14" s="36" t="s">
+        <v>269</v>
+      </c>
+      <c r="I14" s="36" t="s">
         <v>245</v>
       </c>
-      <c r="J14" s="32" t="s">
+      <c r="J14" s="36" t="s">
         <v>244</v>
       </c>
     </row>
@@ -3499,7 +3533,7 @@
         <v>248</v>
       </c>
       <c r="D20" s="36" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="E20" s="36"/>
       <c r="F20" s="36"/>
@@ -3507,7 +3541,7 @@
     </row>
     <row r="21" spans="2:10" x14ac:dyDescent="0.2">
       <c r="D21" s="32" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="I21" s="33"/>
       <c r="J21" s="33"/>
@@ -3517,16 +3551,16 @@
     </row>
     <row r="23" spans="2:10" x14ac:dyDescent="0.2">
       <c r="D23" s="35" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="E23" s="35"/>
     </row>
     <row r="24" spans="2:10" x14ac:dyDescent="0.2">
       <c r="D24" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="F24" s="33" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
     </row>
     <row r="25" spans="2:10" x14ac:dyDescent="0.2">
@@ -3549,12 +3583,12 @@
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B33" s="32" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
     </row>
     <row r="34" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B34" s="6" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added updated summary file
</commit_message>
<xml_diff>
--- a/SUMMARY.xlsx
+++ b/SUMMARY.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amartyn/MPIPZ/amartyn/CSSP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5579AB0-90AA-914C-9844-97B628E8F471}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEBDE6F0-5696-A54C-B6BB-7461FC12381F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="21600" activeTab="2" xr2:uid="{3CB25A69-F844-9241-B587-A0F2F035342F}"/>
+    <workbookView xWindow="-20" yWindow="500" windowWidth="37200" windowHeight="19700" activeTab="3" xr2:uid="{3CB25A69-F844-9241-B587-A0F2F035342F}"/>
   </bookViews>
   <sheets>
     <sheet name="summary" sheetId="1" r:id="rId1"/>
     <sheet name="to do" sheetId="2" r:id="rId2"/>
     <sheet name="sending to co-authors2" sheetId="3" r:id="rId3"/>
+    <sheet name="TO DO v2" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="256">
   <si>
     <t>A</t>
   </si>
@@ -336,12 +337,6 @@
     <t>2_pcoa</t>
   </si>
   <si>
-    <t>check all cpcoa and pcoa script whether done the same way and properly (e.g. no constraining by biorep etc)</t>
-  </si>
-  <si>
-    <t>check that all stacked bp scripts are correct (when e.g. mean of one conditions is shown &gt; previously not done correctly always)</t>
-  </si>
-  <si>
     <t>3_barplots_orders</t>
   </si>
   <si>
@@ -441,9 +436,6 @@
     <t>&gt; Ib consider to change significance testing method?</t>
   </si>
   <si>
-    <t>check whether ANOVA is used everywhere; or think of potentially other method</t>
-  </si>
-  <si>
     <t>7_DA_analysis</t>
   </si>
   <si>
@@ -465,9 +457,6 @@
     <t>Suppl.Fig.3</t>
   </si>
   <si>
-    <t>&gt;&gt; change order in A to Rhizosphere, Root, Nodules; add grey bars behind Lotus/Hordeum title in C,D,E,F</t>
-  </si>
-  <si>
     <t>9_suppl_tables</t>
   </si>
   <si>
@@ -492,12 +481,6 @@
     <t>(contains pca, volcano plots, bubble plot, highlighted metabolite barplots)</t>
   </si>
   <si>
-    <t>&gt;&gt; if time: Ib add slighlty more comments to explain procedure</t>
-  </si>
-  <si>
-    <t>&gt;&gt; add scripts for missing supplementary figure (Suppl. Fig.5 &gt; stacked bp all features, with colours by pathway &amp; one with barplots diffewrences among genotypes per pathway (ANOVA)</t>
-  </si>
-  <si>
     <t>Fig. 5</t>
   </si>
   <si>
@@ -522,36 +505,6 @@
     <t>suppl_tables</t>
   </si>
   <si>
-    <t>&gt;&gt; Anna couldn't run script (error messages)</t>
-  </si>
-  <si>
-    <t>Check in text</t>
-  </si>
-  <si>
-    <t>Questions</t>
-  </si>
-  <si>
-    <t>previosuly &lt;25% asvs shared among soils, now recalculating it is up to 40%?</t>
-  </si>
-  <si>
-    <t>add to M&amp;M where raw data, as well as output feature tables etc can be found</t>
-  </si>
-  <si>
-    <t>wrong spelling of abscisic acid in Figure 5D</t>
-  </si>
-  <si>
-    <t>check chao1 CSSP (supplementary figure 3B &gt; NPK rhizo WT and nsp2 both c?</t>
-  </si>
-  <si>
-    <t>&gt;&gt; check comments</t>
-  </si>
-  <si>
-    <t>&gt;&gt; missing: table info indicator ASVs (incl. taxonomy, RA in WT rhizopshere and root in different soils)</t>
-  </si>
-  <si>
-    <t>&gt;&gt;&gt; Anna re-ran and got different number of metabolites (slightly)</t>
-  </si>
-  <si>
     <t>3_syncoms</t>
   </si>
   <si>
@@ -567,9 +520,6 @@
     <t>4_rarefication</t>
   </si>
   <si>
-    <t>for SynCom figures &gt; chao1, stacked bp etc &gt; do we use only matched ASVs or all ASVs (inclduing contaminants" for display?)</t>
-  </si>
-  <si>
     <t>done for matched ASVs only, as well as all ASVs separately</t>
   </si>
   <si>
@@ -606,12 +556,6 @@
     <t>2_Hordeum</t>
   </si>
   <si>
-    <t>later: adjust M&amp;M section to included all packages used</t>
-  </si>
-  <si>
-    <t>in root exudates Lotus data, we also had samples with R7A treatment in there in raw data &gt; we now just deleted those samples from the metadata file and hence only did the downstream analysis with our uninoculated samples &gt;&gt; sufficient?</t>
-  </si>
-  <si>
     <t>3_rarefication</t>
   </si>
   <si>
@@ -627,45 +571,9 @@
     <t>Suppl. Fig. 6</t>
   </si>
   <si>
-    <t>ANNA (to do 03.02.)</t>
-  </si>
-  <si>
-    <t>finish bibliography</t>
-  </si>
-  <si>
-    <t>WT figure &gt; adjust workflow in panel A (remove text)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> adjust figure quality in all figures (if necessary)</t>
-  </si>
-  <si>
-    <t>root exudate figure &gt; add y axis to boxplots</t>
-  </si>
-  <si>
-    <t>work on SynCom figure &gt; also remove nodule section from bubbleplot &amp; move figure incl. nodule plot to Suppl.</t>
-  </si>
-  <si>
-    <t>write letter to editor</t>
-  </si>
-  <si>
-    <t>set up online PNAS submission</t>
-  </si>
-  <si>
-    <t>OVERALL PRIORITY</t>
-  </si>
-  <si>
-    <t>&gt; get text and figures done to send out to co-authors</t>
-  </si>
-  <si>
-    <t>figure captions</t>
-  </si>
-  <si>
     <t>Analysis</t>
   </si>
   <si>
-    <t>&gt;&gt; in DI Lotus overall list (in Annas new one, all the same apart from one feature 1582 which is not in DA list anymore): DA Hordeum are the same</t>
-  </si>
-  <si>
     <t>&gt;&gt; sort quality problem of final figure with workflow</t>
   </si>
   <si>
@@ -783,15 +691,6 @@
     <t>Hordeum SynCom info</t>
   </si>
   <si>
-    <t>&gt; captions</t>
-  </si>
-  <si>
-    <t>&gt; go through comments in text</t>
-  </si>
-  <si>
-    <t>&gt; literature added properly</t>
-  </si>
-  <si>
     <t>Supplementary Table 8</t>
   </si>
   <si>
@@ -807,51 +706,12 @@
     <t>Supplementary Figure 7</t>
   </si>
   <si>
-    <t>ANNA</t>
-  </si>
-  <si>
-    <t>IB</t>
-  </si>
-  <si>
-    <t>Anna make caption for rest</t>
-  </si>
-  <si>
-    <r>
-      <t>ASVs not matching any member of the SynCom reference set were removed prior to downstream analysis.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="8"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t> </t>
-    </r>
-  </si>
-  <si>
-    <t>additional comments:</t>
-  </si>
-  <si>
-    <t>SynCom:</t>
-  </si>
-  <si>
-    <t>Ib: Figure 3 (prediction), Suppl. Table 2 (Indicator ASVs), Fig. 5 (root ex), Suppl. Fig. 5, Suppl. Tables 4,5</t>
-  </si>
-  <si>
     <t>&gt; quality problem, but cannot fix atm so will keep as is</t>
   </si>
   <si>
     <t>one sample &lt;1000 &gt; was removed (ccamk rhizo)</t>
   </si>
   <si>
-    <t>&gt; for final figure I used Ibs script outputs, but in a separate file I did I calculate cpcoa and pcoa, and my outputs slighlty differ to Ibs &gt;  we need to check this soon!</t>
-  </si>
-  <si>
-    <t>ALSO! In the DA plots for the SynComs we used MaAsLin2 for sign. Analysis of orders! No where else!</t>
-  </si>
-  <si>
     <t>MAASLIN2</t>
   </si>
   <si>
@@ -859,13 +719,100 @@
   </si>
   <si>
     <t>&gt; can be made prettier but ok for now</t>
+  </si>
+  <si>
+    <t>&gt; upload raw data (Askov Soil exp, SynCom exp, root exudate Lotus and Hordeum)</t>
+  </si>
+  <si>
+    <t>&gt; ANOVA + Tukey HSD used correctly everywhere?</t>
+  </si>
+  <si>
+    <t>&gt; check all cpcoa and pcoa script whether done the same way and properly (e.g. no constraining by biorep etc)</t>
+  </si>
+  <si>
+    <t>&gt; check that all stacked bp scripts are correct (when e.g. mean of one conditions is shown &gt; previously not done correctly always)</t>
+  </si>
+  <si>
+    <t>&gt; finish upload info PNAS website</t>
+  </si>
+  <si>
+    <t>&gt; adjust figure quality in all figures (if necessary)</t>
+  </si>
+  <si>
+    <t>&gt; add to draft info on where raw data, as well as output feature tables etc can be found</t>
+  </si>
+  <si>
+    <t>&gt; once all scripts done: in M&amp;M section list all packages (+ references if this is commonly done; ideally do not add as already many references)</t>
+  </si>
+  <si>
+    <t>&gt; in root exudates Lotus data, we also had samples with R7A treatment in there in raw data &gt; we now just deleted those samples from the metadata file and hence only did the downstream analysis with our uninoculated samples &gt;&gt; sufficient?</t>
+  </si>
+  <si>
+    <t>&gt; check whether letter positions fine everywhere? (Figures and Suppl. Figures ) &gt; Anna changed it in 1-2 plots manually in Inkscape, maybe we can adjust it in script though</t>
+  </si>
+  <si>
+    <t>&gt; check whether anywhere else in scripts significance method is used where it shouldn't/ use correct one</t>
+  </si>
+  <si>
+    <t>&gt; check SynCom caption whether explaines properly that MaAsLin2 used for comparing mutant to WT abundances in bacterial order barplots</t>
+  </si>
+  <si>
+    <t>&gt; why in DA tables Syncom (suppl. Tables 6,7) are some spaces empty where there should be 1, 0, -1???</t>
+  </si>
+  <si>
+    <t>&gt; letter to the editor</t>
+  </si>
+  <si>
+    <t>Camilla</t>
+  </si>
+  <si>
+    <t>&gt; batch file root ex Lotus</t>
+  </si>
+  <si>
+    <t>&gt; add which significance methods were overall used to M&amp;M?</t>
+  </si>
+  <si>
+    <t>&gt; soil WT heatmap &gt; so far Kruskal Wallis used &gt; change to ANOVA and check caption + check text in draft whether mentioned results still match</t>
+  </si>
+  <si>
+    <t>(esp. check SynCom part &gt; in cpcoa_pcoa folder; pcoas used for plot done by Ib, then separate script by Anna doing cpcoa and pcoa where cpcoa used for suppl. Figure. &gt; combine in one script for tidier structure and for not generating pcoa outputs twice in different locations)</t>
+  </si>
+  <si>
+    <t>&gt; overall check all scripts whether straight forward, commented well and no chat gpt comments present etc (in some of Anna's scripts).</t>
+  </si>
+  <si>
+    <t>Anna</t>
+  </si>
+  <si>
+    <t>Ib (for now)</t>
+  </si>
+  <si>
+    <t>&gt; check that colours for bacterial orders are consistent everywhere (change script to refer to one csv file in set location)</t>
+  </si>
+  <si>
+    <t>&gt; soil bulk fig: why Chloroflexales still shown? (all letter a)</t>
+  </si>
+  <si>
+    <t>&gt; soil bulk fig: make white space between pies smaller (Anna has done this in Inkscape, maybe we can adjust script also)</t>
+  </si>
+  <si>
+    <t>&gt; soil bulk fig: main figure:  in panel E we have two orders Bacillales and Subgroup_5 which are not in legend/plots of D and F &gt; technically these should be in legend or these orders shouldn’t be in the barplots?? &gt; CHECK (and if necessary adjust results section if we are referring to an order that is not displayed anymore)</t>
+  </si>
+  <si>
+    <t>Anna?</t>
+  </si>
+  <si>
+    <t>&gt; check soil CSSP chao1 (supplementary figure 3B &gt; NPK rhizo WT and nsp2 both c? they look very different though?)</t>
+  </si>
+  <si>
+    <t>&gt; suggest editors/reviewers??</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -915,16 +862,8 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <u/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="15">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -987,25 +926,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5"/>
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor theme="5" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1128,7 +1061,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -1157,21 +1090,20 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1505,20 +1437,20 @@
       </c>
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
-      <c r="D1" s="37" t="s">
+      <c r="D1" s="34" t="s">
         <v>82</v>
       </c>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
       <c r="G1" s="18"/>
-      <c r="H1" s="37" t="s">
+      <c r="H1" s="34" t="s">
         <v>83</v>
       </c>
-      <c r="I1" s="37"/>
-      <c r="K1" s="37" t="s">
+      <c r="I1" s="34"/>
+      <c r="K1" s="34" t="s">
         <v>41</v>
       </c>
-      <c r="L1" s="37"/>
+      <c r="L1" s="34"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
@@ -2099,7 +2031,7 @@
         <v>7</v>
       </c>
       <c r="I41" s="10" t="s">
-        <v>268</v>
+        <v>225</v>
       </c>
     </row>
     <row r="42" spans="1:12" ht="21" x14ac:dyDescent="0.25">
@@ -2194,22 +2126,22 @@
       <c r="G58" t="s">
         <v>63</v>
       </c>
-      <c r="K58" s="30">
+      <c r="K58" s="28">
         <v>8</v>
       </c>
-      <c r="L58" s="31" t="s">
-        <v>211</v>
+      <c r="L58" s="29" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B59" t="s">
         <v>23</v>
       </c>
-      <c r="K59" s="30">
+      <c r="K59" s="28">
         <v>9</v>
       </c>
-      <c r="L59" s="31" t="s">
-        <v>212</v>
+      <c r="L59" s="29" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.2">
@@ -2229,7 +2161,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{05F214DF-3300-D745-A4ED-6415291CCBF0}">
-  <dimension ref="A2:W120"/>
+  <dimension ref="A2:M120"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="18.6640625" bestFit="1" customWidth="1"/>
@@ -2237,103 +2169,77 @@
     <col min="6" max="6" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="M3" s="1" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="21" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" ht="21" x14ac:dyDescent="0.25">
       <c r="B4" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="M4" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="C5" s="24" t="s">
         <v>86</v>
       </c>
-      <c r="M5" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="D6" s="24" t="s">
         <v>87</v>
       </c>
       <c r="E6" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="M6" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="D7" s="24" t="s">
         <v>88</v>
       </c>
       <c r="E7" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="M7" s="29" t="s">
-        <v>166</v>
-      </c>
-      <c r="N7" s="28"/>
-      <c r="O7" s="28"/>
-      <c r="P7" s="28"/>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="C8" s="24" t="s">
         <v>90</v>
       </c>
-      <c r="M8" s="25" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="M8" s="25"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="D9" s="24" t="s">
         <v>87</v>
       </c>
       <c r="E9" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="M9" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="D10" s="24" t="s">
         <v>88</v>
       </c>
       <c r="E10" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="M10" s="28" t="s">
-        <v>200</v>
-      </c>
-      <c r="N10" s="28"/>
-      <c r="O10" s="28"/>
-      <c r="P10" s="28"/>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="C11" s="24" t="s">
         <v>91</v>
       </c>
       <c r="M11" s="25"/>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="D12" s="24" t="s">
         <v>87</v>
       </c>
       <c r="M12" s="1"/>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="E13" s="24" t="s">
         <v>92</v>
       </c>
@@ -2343,22 +2249,18 @@
       <c r="G13" s="23" t="s">
         <v>93</v>
       </c>
-      <c r="M13" s="1" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="M13" s="1"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="E14" s="24" t="s">
         <v>3</v>
       </c>
       <c r="F14" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="M14" s="25" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="M14" s="25"/>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="D15" s="24" t="s">
         <v>88</v>
       </c>
@@ -2371,11 +2273,8 @@
       <c r="G15" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="M15" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="E16" s="24" t="s">
         <v>3</v>
       </c>
@@ -2387,9 +2286,7 @@
       <c r="C17" t="s">
         <v>95</v>
       </c>
-      <c r="M17" s="1" t="s">
-        <v>163</v>
-      </c>
+      <c r="M17" s="1"/>
     </row>
     <row r="18" spans="3:13" x14ac:dyDescent="0.2">
       <c r="D18" s="24" t="s">
@@ -2401,9 +2298,7 @@
       <c r="G18" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="M18" s="25" t="s">
-        <v>164</v>
-      </c>
+      <c r="M18" s="25"/>
     </row>
     <row r="19" spans="3:13" x14ac:dyDescent="0.2">
       <c r="D19" s="26" t="s">
@@ -2412,16 +2307,11 @@
       <c r="E19" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="M19" s="25" t="s">
-        <v>176</v>
-      </c>
+      <c r="M19" s="25"/>
     </row>
     <row r="20" spans="3:13" x14ac:dyDescent="0.2">
       <c r="D20" t="s">
-        <v>101</v>
-      </c>
-      <c r="M20" t="s">
-        <v>190</v>
+        <v>99</v>
       </c>
     </row>
     <row r="21" spans="3:13" x14ac:dyDescent="0.2">
@@ -2434,7 +2324,7 @@
     </row>
     <row r="22" spans="3:13" x14ac:dyDescent="0.2">
       <c r="E22" s="1" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>89</v>
@@ -2443,37 +2333,37 @@
         <v>97</v>
       </c>
       <c r="H22" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="23" spans="3:13" x14ac:dyDescent="0.2">
       <c r="D23" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F23" s="2" t="s">
         <v>89</v>
       </c>
       <c r="H23" t="s">
-        <v>210</v>
+        <v>179</v>
       </c>
     </row>
     <row r="24" spans="3:13" x14ac:dyDescent="0.2">
       <c r="D24" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="E24" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>89</v>
       </c>
       <c r="H24" t="s">
-        <v>209</v>
+        <v>178</v>
       </c>
     </row>
     <row r="25" spans="3:13" x14ac:dyDescent="0.2">
       <c r="D25" s="24" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="E25" s="24"/>
       <c r="F25" s="24" t="s">
@@ -2482,17 +2372,17 @@
     </row>
     <row r="26" spans="3:13" x14ac:dyDescent="0.2">
       <c r="H26" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="27" spans="3:13" x14ac:dyDescent="0.2">
       <c r="C27" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="28" spans="3:13" x14ac:dyDescent="0.2">
       <c r="D28" s="24" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="E28" s="24" t="s">
         <v>89</v>
@@ -2503,7 +2393,7 @@
     </row>
     <row r="29" spans="3:13" x14ac:dyDescent="0.2">
       <c r="D29" s="24" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E29" s="24" t="s">
         <v>89</v>
@@ -2511,21 +2401,13 @@
       <c r="G29" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="M29" s="1" t="s">
-        <v>196</v>
-      </c>
+      <c r="M29" s="1"/>
     </row>
     <row r="30" spans="3:13" x14ac:dyDescent="0.2">
       <c r="D30" s="24" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="E30" s="24"/>
-      <c r="L30" t="s">
-        <v>71</v>
-      </c>
-      <c r="M30" t="s">
-        <v>197</v>
-      </c>
     </row>
     <row r="31" spans="3:13" x14ac:dyDescent="0.2">
       <c r="E31" s="24" t="s">
@@ -2537,12 +2419,6 @@
       <c r="G31" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="L31" t="s">
-        <v>71</v>
-      </c>
-      <c r="M31" t="s">
-        <v>201</v>
-      </c>
     </row>
     <row r="32" spans="3:13" x14ac:dyDescent="0.2">
       <c r="E32" s="24" t="s">
@@ -2554,98 +2430,75 @@
       <c r="G32" s="27" t="s">
         <v>97</v>
       </c>
-      <c r="L32" t="s">
-        <v>71</v>
-      </c>
-      <c r="M32" t="s">
-        <v>198</v>
-      </c>
     </row>
     <row r="33" spans="3:13" x14ac:dyDescent="0.2">
       <c r="D33" s="26" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E33" s="24" t="s">
         <v>89</v>
-      </c>
-      <c r="L33" t="s">
-        <v>71</v>
-      </c>
-      <c r="M33" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="34" spans="3:13" x14ac:dyDescent="0.2">
       <c r="D34" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="G34" s="27" t="s">
+        <v>112</v>
+      </c>
+      <c r="H34" t="s">
         <v>113</v>
-      </c>
-      <c r="E34" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="G34" s="27" t="s">
-        <v>114</v>
-      </c>
-      <c r="H34" t="s">
-        <v>115</v>
-      </c>
-      <c r="M34" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="35" spans="3:13" x14ac:dyDescent="0.2">
       <c r="D35" s="24" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E35" s="24" t="s">
         <v>89</v>
-      </c>
-      <c r="M35" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="36" spans="3:13" x14ac:dyDescent="0.2">
       <c r="D36" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="37" spans="3:13" x14ac:dyDescent="0.2">
       <c r="E37" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F37" s="2" t="s">
         <v>89</v>
       </c>
       <c r="H37" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="38" spans="3:13" x14ac:dyDescent="0.2">
       <c r="E38" t="s">
+        <v>118</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="H38" t="s">
         <v>120</v>
       </c>
-      <c r="F38" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="H38" t="s">
-        <v>122</v>
-      </c>
     </row>
     <row r="39" spans="3:13" x14ac:dyDescent="0.2">
-      <c r="M39" s="1" t="s">
-        <v>204</v>
-      </c>
+      <c r="M39" s="1"/>
     </row>
     <row r="40" spans="3:13" x14ac:dyDescent="0.2">
       <c r="C40" t="s">
-        <v>123</v>
-      </c>
-      <c r="M40" t="s">
-        <v>205</v>
+        <v>121</v>
       </c>
     </row>
     <row r="41" spans="3:13" x14ac:dyDescent="0.2">
       <c r="D41" s="24" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="E41" s="24" t="s">
         <v>89</v>
@@ -2656,7 +2509,7 @@
     </row>
     <row r="42" spans="3:13" x14ac:dyDescent="0.2">
       <c r="D42" s="24" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="E42" s="24" t="s">
         <v>89</v>
@@ -2667,7 +2520,7 @@
     </row>
     <row r="43" spans="3:13" x14ac:dyDescent="0.2">
       <c r="D43" s="24" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="E43" s="24" t="s">
         <v>89</v>
@@ -2675,7 +2528,7 @@
     </row>
     <row r="44" spans="3:13" x14ac:dyDescent="0.2">
       <c r="D44" s="24" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="45" spans="3:13" x14ac:dyDescent="0.2">
@@ -2702,7 +2555,7 @@
     </row>
     <row r="47" spans="3:13" x14ac:dyDescent="0.2">
       <c r="D47" s="26" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="48" spans="3:13" x14ac:dyDescent="0.2">
@@ -2723,12 +2576,12 @@
     </row>
     <row r="50" spans="4:12" x14ac:dyDescent="0.2">
       <c r="D50" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="51" spans="4:12" x14ac:dyDescent="0.2">
       <c r="E51" s="26" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="F51" s="24" t="s">
         <v>89</v>
@@ -2736,24 +2589,24 @@
     </row>
     <row r="52" spans="4:12" x14ac:dyDescent="0.2">
       <c r="E52" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="G52" s="27" t="s">
+        <v>129</v>
+      </c>
+      <c r="H52" t="s">
         <v>130</v>
       </c>
-      <c r="F52" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="G52" s="27" t="s">
+      <c r="L52" t="s">
         <v>131</v>
-      </c>
-      <c r="H52" t="s">
-        <v>132</v>
-      </c>
-      <c r="L52" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="53" spans="4:12" x14ac:dyDescent="0.2">
       <c r="D53" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="54" spans="4:12" x14ac:dyDescent="0.2">
@@ -2768,36 +2621,34 @@
         <v>88</v>
       </c>
       <c r="F55" s="2"/>
-      <c r="H55" s="11" t="s">
-        <v>161</v>
-      </c>
+      <c r="H55" s="11"/>
     </row>
     <row r="56" spans="4:12" x14ac:dyDescent="0.2">
       <c r="E56" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="F56" s="2"/>
       <c r="H56" s="11"/>
     </row>
     <row r="57" spans="4:12" x14ac:dyDescent="0.2">
       <c r="D57" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
     <row r="58" spans="4:12" x14ac:dyDescent="0.2">
       <c r="E58" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="F58" s="2" t="s">
         <v>89</v>
       </c>
       <c r="H58" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="59" spans="4:12" x14ac:dyDescent="0.2">
       <c r="E59" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="F59" s="24" t="s">
         <v>89</v>
@@ -2805,18 +2656,15 @@
     </row>
     <row r="60" spans="4:12" x14ac:dyDescent="0.2">
       <c r="E60" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="F60" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="H60" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="61" spans="4:12" x14ac:dyDescent="0.2">
       <c r="E61" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="F61" s="24" t="s">
         <v>89</v>
@@ -2824,175 +2672,113 @@
     </row>
     <row r="62" spans="4:12" x14ac:dyDescent="0.2">
       <c r="D62" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="E62" s="2"/>
       <c r="H62" t="s">
-        <v>253</v>
+        <v>219</v>
       </c>
     </row>
     <row r="63" spans="4:12" x14ac:dyDescent="0.2">
       <c r="H63" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="65" spans="2:23" x14ac:dyDescent="0.2">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="65" spans="2:6" x14ac:dyDescent="0.2">
       <c r="C65" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="66" spans="2:23" x14ac:dyDescent="0.2">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="66" spans="2:6" x14ac:dyDescent="0.2">
       <c r="D66" t="s">
-        <v>207</v>
+        <v>177</v>
       </c>
       <c r="F66" s="24" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="67" spans="2:23" x14ac:dyDescent="0.2">
+    <row r="67" spans="2:6" x14ac:dyDescent="0.2">
       <c r="D67" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="E67" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="F67" s="2"/>
-      <c r="H67" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="68" spans="2:23" x14ac:dyDescent="0.2">
+    </row>
+    <row r="68" spans="2:6" x14ac:dyDescent="0.2">
       <c r="D68" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="F68" s="2"/>
-      <c r="H68" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="69" spans="2:23" x14ac:dyDescent="0.2">
-      <c r="H69" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="71" spans="2:23" ht="21" x14ac:dyDescent="0.25">
+    </row>
+    <row r="71" spans="2:6" ht="21" x14ac:dyDescent="0.25">
       <c r="B71" s="18" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="72" spans="2:23" x14ac:dyDescent="0.2">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="72" spans="2:6" x14ac:dyDescent="0.2">
       <c r="C72" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="73" spans="2:23" x14ac:dyDescent="0.2">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="73" spans="2:6" x14ac:dyDescent="0.2">
       <c r="D73" t="s">
         <v>87</v>
       </c>
       <c r="E73" s="2"/>
       <c r="F73" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="74" spans="2:23" x14ac:dyDescent="0.2">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="74" spans="2:6" x14ac:dyDescent="0.2">
       <c r="D74" s="24" t="s">
         <v>88</v>
       </c>
       <c r="E74" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="J74" s="28" t="s">
-        <v>170</v>
-      </c>
-      <c r="K74" s="28"/>
-      <c r="L74" s="28"/>
-      <c r="M74" s="28"/>
-      <c r="N74" s="28"/>
-      <c r="O74" s="28"/>
-      <c r="P74" s="28"/>
-      <c r="Q74" s="28"/>
-      <c r="R74" s="28"/>
-      <c r="S74" s="28"/>
-      <c r="T74" s="28"/>
-      <c r="U74" s="28"/>
-    </row>
-    <row r="75" spans="2:23" x14ac:dyDescent="0.2">
+    </row>
+    <row r="75" spans="2:6" x14ac:dyDescent="0.2">
       <c r="C75" t="s">
         <v>90</v>
       </c>
       <c r="D75" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="J75" s="28" t="s">
-        <v>208</v>
-      </c>
-      <c r="K75" s="28"/>
-      <c r="L75" s="28"/>
-      <c r="M75" s="28"/>
-      <c r="N75" s="28"/>
-      <c r="O75" s="28"/>
-      <c r="P75" s="28"/>
-      <c r="Q75" s="28"/>
-      <c r="R75" s="28"/>
-      <c r="S75" s="28"/>
-      <c r="T75" s="28"/>
-      <c r="U75" s="28"/>
-    </row>
-    <row r="76" spans="2:23" x14ac:dyDescent="0.2">
+    </row>
+    <row r="76" spans="2:6" x14ac:dyDescent="0.2">
       <c r="C76" t="s">
+        <v>143</v>
+      </c>
+      <c r="D76" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="77" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="C77" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="78" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="D78" s="24" t="s">
         <v>147</v>
       </c>
-      <c r="D76" t="s">
-        <v>150</v>
-      </c>
-      <c r="J76" s="28" t="s">
-        <v>151</v>
-      </c>
-      <c r="K76" s="28"/>
-      <c r="L76" s="28"/>
-      <c r="M76" s="28"/>
-      <c r="N76" s="28"/>
-    </row>
-    <row r="77" spans="2:23" x14ac:dyDescent="0.2">
-      <c r="C77" t="s">
+      <c r="E78" s="24" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="79" spans="2:6" x14ac:dyDescent="0.2">
+      <c r="D79" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="J77" s="28" t="s">
-        <v>152</v>
-      </c>
-      <c r="K77" s="28"/>
-      <c r="L77" s="28"/>
-      <c r="M77" s="28"/>
-      <c r="N77" s="28"/>
-      <c r="O77" s="28"/>
-      <c r="P77" s="28"/>
-      <c r="Q77" s="28"/>
-      <c r="R77" s="28"/>
-      <c r="S77" s="28"/>
-      <c r="T77" s="28"/>
-      <c r="U77" s="28"/>
-      <c r="V77" s="28"/>
-      <c r="W77" s="28"/>
-    </row>
-    <row r="78" spans="2:23" x14ac:dyDescent="0.2">
-      <c r="D78" s="24" t="s">
-        <v>153</v>
-      </c>
-      <c r="E78" s="24" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="79" spans="2:23" x14ac:dyDescent="0.2">
-      <c r="D79" s="2" t="s">
-        <v>154</v>
-      </c>
       <c r="E79" s="2" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="80" spans="2:23" x14ac:dyDescent="0.2">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="80" spans="2:6" x14ac:dyDescent="0.2">
       <c r="C80" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
     </row>
     <row r="81" spans="2:12" x14ac:dyDescent="0.2">
@@ -3013,12 +2799,12 @@
     </row>
     <row r="84" spans="2:12" ht="21" x14ac:dyDescent="0.25">
       <c r="B84" s="18" t="s">
-        <v>171</v>
+        <v>155</v>
       </c>
     </row>
     <row r="85" spans="2:12" x14ac:dyDescent="0.2">
       <c r="C85" t="s">
-        <v>172</v>
+        <v>156</v>
       </c>
     </row>
     <row r="86" spans="2:12" x14ac:dyDescent="0.2">
@@ -3039,7 +2825,7 @@
     </row>
     <row r="88" spans="2:12" x14ac:dyDescent="0.2">
       <c r="D88" s="24" t="s">
-        <v>173</v>
+        <v>157</v>
       </c>
       <c r="E88" s="24" t="s">
         <v>89</v>
@@ -3050,7 +2836,7 @@
     </row>
     <row r="89" spans="2:12" x14ac:dyDescent="0.2">
       <c r="D89" s="24" t="s">
-        <v>174</v>
+        <v>158</v>
       </c>
       <c r="E89" s="24" t="s">
         <v>89</v>
@@ -3061,7 +2847,7 @@
     </row>
     <row r="90" spans="2:12" x14ac:dyDescent="0.2">
       <c r="D90" s="24" t="s">
-        <v>175</v>
+        <v>159</v>
       </c>
       <c r="E90" s="24" t="s">
         <v>89</v>
@@ -3072,20 +2858,20 @@
     </row>
     <row r="91" spans="2:12" x14ac:dyDescent="0.2">
       <c r="D91" s="24" t="s">
-        <v>178</v>
+        <v>161</v>
       </c>
       <c r="G91" t="s">
-        <v>177</v>
+        <v>160</v>
       </c>
     </row>
     <row r="92" spans="2:12" x14ac:dyDescent="0.2">
       <c r="E92" s="24" t="s">
-        <v>179</v>
+        <v>162</v>
       </c>
     </row>
     <row r="93" spans="2:12" x14ac:dyDescent="0.2">
       <c r="F93" s="24" t="s">
-        <v>180</v>
+        <v>163</v>
       </c>
       <c r="G93" s="24" t="s">
         <v>89</v>
@@ -3093,7 +2879,7 @@
     </row>
     <row r="94" spans="2:12" x14ac:dyDescent="0.2">
       <c r="F94" s="24" t="s">
-        <v>181</v>
+        <v>164</v>
       </c>
       <c r="G94" s="24" t="s">
         <v>89</v>
@@ -3101,13 +2887,13 @@
     </row>
     <row r="95" spans="2:12" x14ac:dyDescent="0.2">
       <c r="E95" s="24" t="s">
-        <v>182</v>
+        <v>165</v>
       </c>
       <c r="F95" s="24" t="s">
         <v>89</v>
       </c>
       <c r="G95" t="s">
-        <v>177</v>
+        <v>160</v>
       </c>
       <c r="L95" s="27" t="s">
         <v>97</v>
@@ -3115,14 +2901,14 @@
     </row>
     <row r="96" spans="2:12" x14ac:dyDescent="0.2">
       <c r="D96" s="26" t="s">
-        <v>183</v>
+        <v>166</v>
       </c>
       <c r="E96" s="24"/>
     </row>
     <row r="97" spans="3:7" x14ac:dyDescent="0.2">
       <c r="D97" s="24"/>
       <c r="E97" s="24" t="s">
-        <v>184</v>
+        <v>167</v>
       </c>
       <c r="F97" s="24" t="s">
         <v>89</v>
@@ -3139,18 +2925,18 @@
     </row>
     <row r="99" spans="3:7" x14ac:dyDescent="0.2">
       <c r="D99" s="26" t="s">
-        <v>185</v>
+        <v>168</v>
       </c>
       <c r="E99" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="G99" s="38" t="s">
-        <v>267</v>
+      <c r="G99" s="33" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="100" spans="3:7" x14ac:dyDescent="0.2">
       <c r="D100" s="24" t="s">
-        <v>186</v>
+        <v>169</v>
       </c>
       <c r="E100" s="24" t="s">
         <v>89</v>
@@ -3158,7 +2944,7 @@
     </row>
     <row r="101" spans="3:7" x14ac:dyDescent="0.2">
       <c r="D101" s="24" t="s">
-        <v>187</v>
+        <v>170</v>
       </c>
       <c r="E101" s="24" t="s">
         <v>89</v>
@@ -3166,7 +2952,7 @@
     </row>
     <row r="102" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C102" t="s">
-        <v>188</v>
+        <v>171</v>
       </c>
     </row>
     <row r="103" spans="3:7" x14ac:dyDescent="0.2">
@@ -3187,7 +2973,7 @@
     </row>
     <row r="105" spans="3:7" x14ac:dyDescent="0.2">
       <c r="D105" s="24" t="s">
-        <v>173</v>
+        <v>157</v>
       </c>
       <c r="E105" s="24" t="s">
         <v>89</v>
@@ -3198,18 +2984,18 @@
     </row>
     <row r="106" spans="3:7" x14ac:dyDescent="0.2">
       <c r="D106" s="24" t="s">
-        <v>191</v>
+        <v>172</v>
       </c>
       <c r="E106" s="24" t="s">
         <v>89</v>
       </c>
       <c r="G106" s="23" t="s">
-        <v>264</v>
+        <v>223</v>
       </c>
     </row>
     <row r="107" spans="3:7" x14ac:dyDescent="0.2">
       <c r="D107" s="24" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="E107" s="24" t="s">
         <v>89</v>
@@ -3220,29 +3006,26 @@
     </row>
     <row r="108" spans="3:7" x14ac:dyDescent="0.2">
       <c r="D108" s="26" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="E108" s="24" t="s">
         <v>89</v>
-      </c>
-      <c r="G108" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="109" spans="3:7" x14ac:dyDescent="0.2">
       <c r="D109" s="26" t="s">
-        <v>192</v>
+        <v>173</v>
       </c>
       <c r="E109" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="G109" s="38" t="s">
-        <v>267</v>
+      <c r="G109" s="33" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="110" spans="3:7" x14ac:dyDescent="0.2">
       <c r="D110" s="24" t="s">
-        <v>193</v>
+        <v>174</v>
       </c>
       <c r="E110" s="24" t="s">
         <v>89</v>
@@ -3250,12 +3033,12 @@
     </row>
     <row r="111" spans="3:7" x14ac:dyDescent="0.2">
       <c r="C111" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
     </row>
     <row r="112" spans="3:7" x14ac:dyDescent="0.2">
       <c r="D112" s="24" t="s">
-        <v>194</v>
+        <v>175</v>
       </c>
       <c r="E112" s="24" t="s">
         <v>89</v>
@@ -3263,20 +3046,20 @@
     </row>
     <row r="113" spans="3:5" x14ac:dyDescent="0.2">
       <c r="D113" t="s">
-        <v>195</v>
+        <v>176</v>
       </c>
       <c r="E113" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
     </row>
     <row r="114" spans="3:5" x14ac:dyDescent="0.2">
       <c r="E114" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
     </row>
     <row r="115" spans="3:5" x14ac:dyDescent="0.2">
       <c r="C115" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
     </row>
     <row r="116" spans="3:5" x14ac:dyDescent="0.2">
@@ -3284,7 +3067,7 @@
         <v>87</v>
       </c>
       <c r="E116" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
     </row>
     <row r="117" spans="3:5" x14ac:dyDescent="0.2">
@@ -3292,13 +3075,11 @@
         <v>88</v>
       </c>
       <c r="E117" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
     </row>
     <row r="120" spans="3:5" x14ac:dyDescent="0.2">
-      <c r="C120" s="1" t="s">
-        <v>266</v>
-      </c>
+      <c r="C120" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3307,7 +3088,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAEB7DF4-A933-4345-8067-1627111DF6E1}">
-  <dimension ref="A3:J34"/>
+  <dimension ref="A3:J29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
@@ -3322,277 +3103,372 @@
   <sheetData>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A4" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="B4" s="32" t="s">
+        <v>183</v>
+      </c>
+      <c r="C4" s="32" t="s">
+        <v>186</v>
+      </c>
+      <c r="D4" t="s">
+        <v>222</v>
+      </c>
+      <c r="H4" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="I4" s="32" t="s">
+        <v>195</v>
+      </c>
+      <c r="J4" s="32" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A5" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="B5" s="32" t="s">
+        <v>184</v>
+      </c>
+      <c r="C5" s="32" t="s">
+        <v>187</v>
+      </c>
+      <c r="D5" t="s">
+        <v>222</v>
+      </c>
+      <c r="E5" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="F5" s="32" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="B6" s="32" t="s">
+        <v>185</v>
+      </c>
+      <c r="C6" s="32" t="s">
+        <v>190</v>
+      </c>
+      <c r="H6" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="I6" s="32" t="s">
+        <v>198</v>
+      </c>
+      <c r="J6" s="32" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="B7" s="32" t="s">
+        <v>189</v>
+      </c>
+      <c r="C7" s="32" t="s">
+        <v>188</v>
+      </c>
+      <c r="D7" t="s">
+        <v>222</v>
+      </c>
+      <c r="E7" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="F7" s="32" t="s">
+        <v>200</v>
+      </c>
+      <c r="H7" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="I7" s="32" t="s">
+        <v>204</v>
+      </c>
+      <c r="J7" s="32" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E8" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="F8" s="32" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E9" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="F9" s="32" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A10" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="B10" s="32" t="s">
+        <v>191</v>
+      </c>
+      <c r="C10" s="32" t="s">
+        <v>194</v>
+      </c>
+      <c r="E10" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="F10" s="32" t="s">
+        <v>205</v>
+      </c>
+      <c r="H10" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="I10" s="32" t="s">
+        <v>210</v>
+      </c>
+      <c r="J10" s="32" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H11" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="I11" s="32" t="s">
+        <v>208</v>
+      </c>
+      <c r="J11" s="32" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B13" s="32" t="s">
+        <v>192</v>
+      </c>
+      <c r="C13" s="32" t="s">
+        <v>193</v>
+      </c>
+      <c r="D13" t="s">
+        <v>222</v>
+      </c>
+      <c r="F13" s="32" t="s">
+        <v>211</v>
+      </c>
+      <c r="G13" s="32" t="s">
+        <v>226</v>
+      </c>
+      <c r="I13" s="32" t="s">
+        <v>209</v>
+      </c>
+      <c r="J13" s="32" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B14" s="32"/>
+      <c r="C14" s="32"/>
+      <c r="F14" s="32" t="s">
+        <v>221</v>
+      </c>
+      <c r="G14" s="32" t="s">
+        <v>226</v>
+      </c>
+      <c r="I14" s="32" t="s">
+        <v>214</v>
+      </c>
+      <c r="J14" s="32" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A4" s="36" t="s">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H16" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="B4" s="36" t="s">
-        <v>214</v>
-      </c>
-      <c r="C4" s="36" t="s">
+      <c r="I16" s="32" t="s">
         <v>217</v>
       </c>
-      <c r="D4" t="s">
-        <v>263</v>
-      </c>
-      <c r="H4" s="36" t="s">
+      <c r="J16" s="32" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="17" spans="8:10" x14ac:dyDescent="0.2">
+      <c r="H17" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="I4" s="36" t="s">
-        <v>226</v>
-      </c>
-      <c r="J4" s="36" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A5" s="36" t="s">
-        <v>71</v>
-      </c>
-      <c r="B5" s="36" t="s">
-        <v>215</v>
-      </c>
-      <c r="C5" s="36" t="s">
+      <c r="I17" s="32" t="s">
         <v>218</v>
       </c>
-      <c r="D5" t="s">
-        <v>263</v>
-      </c>
-      <c r="E5" s="36" t="s">
-        <v>71</v>
-      </c>
-      <c r="F5" s="36" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A6" s="36" t="s">
-        <v>71</v>
-      </c>
-      <c r="B6" s="36" t="s">
+      <c r="J17" s="32" t="s">
         <v>216</v>
       </c>
-      <c r="C6" s="36" t="s">
-        <v>221</v>
-      </c>
-      <c r="H6" s="36" t="s">
-        <v>71</v>
-      </c>
-      <c r="I6" s="36" t="s">
-        <v>229</v>
-      </c>
-      <c r="J6" s="36" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A7" s="36" t="s">
-        <v>71</v>
-      </c>
-      <c r="B7" s="36" t="s">
-        <v>220</v>
-      </c>
-      <c r="C7" s="36" t="s">
-        <v>219</v>
-      </c>
-      <c r="D7" t="s">
-        <v>263</v>
-      </c>
-      <c r="E7" s="36" t="s">
-        <v>71</v>
-      </c>
-      <c r="F7" s="36" t="s">
-        <v>231</v>
-      </c>
-      <c r="H7" s="36" t="s">
-        <v>71</v>
-      </c>
-      <c r="I7" s="36" t="s">
-        <v>235</v>
-      </c>
-      <c r="J7" s="36" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="E8" s="36" t="s">
-        <v>71</v>
-      </c>
-      <c r="F8" s="36" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="E9" s="36" t="s">
-        <v>71</v>
-      </c>
-      <c r="F9" s="36" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A10" s="36" t="s">
-        <v>71</v>
-      </c>
-      <c r="B10" s="36" t="s">
-        <v>222</v>
-      </c>
-      <c r="C10" s="36" t="s">
-        <v>225</v>
-      </c>
-      <c r="E10" s="36" t="s">
-        <v>71</v>
-      </c>
-      <c r="F10" s="36" t="s">
-        <v>236</v>
-      </c>
-      <c r="H10" s="36" t="s">
-        <v>71</v>
-      </c>
-      <c r="I10" s="36" t="s">
-        <v>241</v>
-      </c>
-      <c r="J10" s="36" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="H11" s="36" t="s">
-        <v>71</v>
-      </c>
-      <c r="I11" s="36" t="s">
-        <v>239</v>
-      </c>
-      <c r="J11" s="36" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B13" s="36" t="s">
-        <v>223</v>
-      </c>
-      <c r="C13" s="36" t="s">
-        <v>224</v>
-      </c>
-      <c r="F13" s="36" t="s">
-        <v>242</v>
-      </c>
-      <c r="G13" s="36" t="s">
-        <v>269</v>
-      </c>
-      <c r="I13" s="36" t="s">
-        <v>240</v>
-      </c>
-      <c r="J13" s="36" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="B14" s="36"/>
-      <c r="C14" s="36"/>
-      <c r="F14" s="36" t="s">
-        <v>255</v>
-      </c>
-      <c r="G14" s="36" t="s">
-        <v>269</v>
-      </c>
-      <c r="I14" s="36" t="s">
-        <v>245</v>
-      </c>
-      <c r="J14" s="36" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="H16" s="36" t="s">
-        <v>71</v>
-      </c>
-      <c r="I16" s="36" t="s">
-        <v>251</v>
-      </c>
-      <c r="J16" s="36" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="17" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="H17" s="36" t="s">
-        <v>71</v>
-      </c>
-      <c r="I17" s="36" t="s">
-        <v>252</v>
-      </c>
-      <c r="J17" s="36" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="20" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B20" t="s">
-        <v>248</v>
-      </c>
-      <c r="D20" s="36" t="s">
-        <v>262</v>
-      </c>
-      <c r="E20" s="36"/>
-      <c r="F20" s="36"/>
-      <c r="G20" s="36"/>
-    </row>
-    <row r="21" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="D21" s="32" t="s">
-        <v>258</v>
-      </c>
-      <c r="I21" s="33"/>
-      <c r="J21" s="33"/>
-    </row>
-    <row r="22" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="I22" s="33"/>
-    </row>
-    <row r="23" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="D23" s="35" t="s">
-        <v>260</v>
-      </c>
-      <c r="E23" s="35"/>
-    </row>
-    <row r="24" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="D24" t="s">
-        <v>261</v>
-      </c>
-      <c r="F24" s="33" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="25" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="F25" s="33"/>
-    </row>
-    <row r="28" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B28" t="s">
-        <v>249</v>
-      </c>
-      <c r="G28" s="33"/>
-      <c r="H28" s="33"/>
-    </row>
-    <row r="29" spans="2:10" x14ac:dyDescent="0.2">
-      <c r="B29" s="36" t="s">
-        <v>250</v>
-      </c>
-      <c r="C29" s="36"/>
-      <c r="G29" s="34"/>
-      <c r="H29" s="34"/>
-    </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B33" s="32" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B34" s="6" t="s">
-        <v>257</v>
-      </c>
+    </row>
+    <row r="21" spans="8:10" x14ac:dyDescent="0.2">
+      <c r="I21" s="30"/>
+      <c r="J21" s="30"/>
+    </row>
+    <row r="22" spans="8:10" x14ac:dyDescent="0.2">
+      <c r="I22" s="30"/>
+    </row>
+    <row r="28" spans="8:10" x14ac:dyDescent="0.2">
+      <c r="H28" s="30"/>
+    </row>
+    <row r="29" spans="8:10" x14ac:dyDescent="0.2">
+      <c r="H29" s="31"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62FA262E-F179-974C-9831-3EFA13F1295F}">
+  <dimension ref="A2:D22"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="69.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="255.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" s="35" t="s">
+        <v>240</v>
+      </c>
+      <c r="B3" t="s">
+        <v>242</v>
+      </c>
+      <c r="D3" s="35" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" s="35" t="s">
+        <v>231</v>
+      </c>
+      <c r="D4" s="35" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>227</v>
+      </c>
+      <c r="D5" s="35" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>235</v>
+      </c>
+      <c r="D6" s="35" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>255</v>
+      </c>
+      <c r="D7" s="35" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D8" s="37" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D9" s="35" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D10" s="36" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D11" s="33" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D12" s="35" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D13" s="33" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D14" s="35" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D15" s="33" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D16" s="35" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="17" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="D17" s="35" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="18" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="D18" s="33" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="19" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="D19" s="33" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="20" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="D20" s="33" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="22" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C22" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="D22" s="33" t="s">
+        <v>232</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
added new summary file
</commit_message>
<xml_diff>
--- a/SUMMARY.xlsx
+++ b/SUMMARY.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/amartyn/MPIPZ/amartyn/CSSP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AEBDE6F0-5696-A54C-B6BB-7461FC12381F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5AB2C0F-BD67-2A40-AD7E-5A980F4D4F26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="500" windowWidth="37200" windowHeight="19700" activeTab="3" xr2:uid="{3CB25A69-F844-9241-B587-A0F2F035342F}"/>
+    <workbookView xWindow="5680" yWindow="1120" windowWidth="26820" windowHeight="16980" activeTab="3" xr2:uid="{3CB25A69-F844-9241-B587-A0F2F035342F}"/>
   </bookViews>
   <sheets>
     <sheet name="summary" sheetId="1" r:id="rId1"/>
     <sheet name="to do" sheetId="2" r:id="rId2"/>
     <sheet name="sending to co-authors2" sheetId="3" r:id="rId3"/>
     <sheet name="TO DO v2" sheetId="4" r:id="rId4"/>
+    <sheet name="colour info" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="293">
   <si>
     <t>A</t>
   </si>
@@ -806,6 +807,117 @@
   </si>
   <si>
     <t>&gt; suggest editors/reviewers??</t>
+  </si>
+  <si>
+    <t>check text where Suppl. 3B is mentioned (chao1 order was incorrect)</t>
+  </si>
+  <si>
+    <t>bulk soil figure &gt; svg file has old figure, add new one where chloroflexales Is gone and update + save</t>
+  </si>
+  <si>
+    <t>soil WT figure &gt; hetamap &gt; now ANOVA use correct figure (Hordeum Rhizosphere Burkholderiales a,b,c) &gt; add correct figure to svg file and check text</t>
+  </si>
+  <si>
+    <t>soil WT</t>
+  </si>
+  <si>
+    <t>barplots significant orders</t>
+  </si>
+  <si>
+    <t>pie charts</t>
+  </si>
+  <si>
+    <t>currently</t>
+  </si>
+  <si>
+    <t>top 20 for each soil separately &gt; all unique orders displayed</t>
+  </si>
+  <si>
+    <t>top 20 across soils used</t>
+  </si>
+  <si>
+    <t>wanted</t>
+  </si>
+  <si>
+    <t>top 20 for each soil separately &gt; all unique orders displayed (here only significant ones shown)</t>
+  </si>
+  <si>
+    <t>figure type</t>
+  </si>
+  <si>
+    <t>panel</t>
+  </si>
+  <si>
+    <t>figure</t>
+  </si>
+  <si>
+    <t>soil bulk</t>
+  </si>
+  <si>
+    <t>Suppl. Fig. 1</t>
+  </si>
+  <si>
+    <t>choose top 20 (with min. 1% RA), in Lotus rhizo and root COMBINED; as well as top20 (with min. 1%RA) in Hordeum rhizo and root COMBINED &gt;&gt; all those orders for Lotus and Hordeum combined (united not intersect)</t>
+  </si>
+  <si>
+    <t>all orders displayed</t>
+  </si>
+  <si>
+    <t>prediction</t>
+  </si>
+  <si>
+    <t>Suppl. Fig. 4</t>
+  </si>
+  <si>
+    <t>GO OVER WHOLE TEXT AND CAPTIONS +M&amp;M with new figures</t>
+  </si>
+  <si>
+    <t>top 20 Lotus (WT only, top 20 across all rhizosphere-root and soil combinations together); same for Hordeum &gt; and then lists combined (united not intersection) (NO 1% filtering)</t>
+  </si>
+  <si>
+    <t>FIGURE SIZES</t>
+  </si>
+  <si>
+    <t>small</t>
+  </si>
+  <si>
+    <t>medium</t>
+  </si>
+  <si>
+    <t>large</t>
+  </si>
+  <si>
+    <t>9x6cm</t>
+  </si>
+  <si>
+    <t>11x11cm</t>
+  </si>
+  <si>
+    <t>18x22cm</t>
+  </si>
+  <si>
+    <t>Suppl. Fig. 7</t>
+  </si>
+  <si>
+    <t>G</t>
+  </si>
+  <si>
+    <t>DA plot incl. nodule comp.</t>
+  </si>
+  <si>
+    <t>barplots sign orders</t>
+  </si>
+  <si>
+    <t>DA plot excl. nodule comp.</t>
+  </si>
+  <si>
+    <t>all orders</t>
+  </si>
+  <si>
+    <t>&gt; check whether in captions all significance methods named correctly + which orders chosen for display (top20 in what??)</t>
+  </si>
+  <si>
+    <t>ANNA</t>
   </si>
 </sst>
 </file>
@@ -1098,12 +1210,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1437,20 +1549,20 @@
       </c>
       <c r="B1" s="18"/>
       <c r="C1" s="18"/>
-      <c r="D1" s="34" t="s">
+      <c r="D1" s="37" t="s">
         <v>82</v>
       </c>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
       <c r="G1" s="18"/>
-      <c r="H1" s="34" t="s">
+      <c r="H1" s="37" t="s">
         <v>83</v>
       </c>
-      <c r="I1" s="34"/>
-      <c r="K1" s="34" t="s">
+      <c r="I1" s="37"/>
+      <c r="K1" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="L1" s="34"/>
+      <c r="L1" s="37"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
@@ -3333,7 +3445,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62FA262E-F179-974C-9831-3EFA13F1295F}">
-  <dimension ref="A2:D22"/>
+  <dimension ref="A2:D36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="69.6640625" bestFit="1" customWidth="1"/>
@@ -3353,21 +3465,21 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="35" t="s">
+      <c r="A3" s="34" t="s">
         <v>240</v>
       </c>
       <c r="B3" t="s">
         <v>242</v>
       </c>
-      <c r="D3" s="35" t="s">
+      <c r="D3" s="34" t="s">
         <v>228</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="35" t="s">
+      <c r="A4" s="34" t="s">
         <v>231</v>
       </c>
-      <c r="D4" s="35" t="s">
+      <c r="D4" s="34" t="s">
         <v>244</v>
       </c>
     </row>
@@ -3375,7 +3487,7 @@
       <c r="A5" t="s">
         <v>227</v>
       </c>
-      <c r="D5" s="35" t="s">
+      <c r="D5" s="34" t="s">
         <v>229</v>
       </c>
     </row>
@@ -3383,7 +3495,7 @@
       <c r="A6" t="s">
         <v>235</v>
       </c>
-      <c r="D6" s="35" t="s">
+      <c r="D6" s="34" t="s">
         <v>245</v>
       </c>
     </row>
@@ -3391,22 +3503,22 @@
       <c r="A7" t="s">
         <v>255</v>
       </c>
-      <c r="D7" s="35" t="s">
+      <c r="D7" s="34" t="s">
         <v>230</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="D8" s="37" t="s">
+      <c r="D8" s="36" t="s">
         <v>254</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="D9" s="35" t="s">
+      <c r="D9" s="34" t="s">
         <v>249</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="D10" s="36" t="s">
+      <c r="D10" s="35" t="s">
         <v>233</v>
       </c>
     </row>
@@ -3416,7 +3528,7 @@
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="D12" s="35" t="s">
+      <c r="D12" s="34" t="s">
         <v>250</v>
       </c>
     </row>
@@ -3426,7 +3538,7 @@
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="D14" s="35" t="s">
+      <c r="D14" s="34" t="s">
         <v>252</v>
       </c>
     </row>
@@ -3436,12 +3548,12 @@
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="D16" s="35" t="s">
+      <c r="D16" s="34" t="s">
         <v>237</v>
       </c>
     </row>
     <row r="17" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="D17" s="35" t="s">
+      <c r="D17" s="34" t="s">
         <v>239</v>
       </c>
     </row>
@@ -3466,6 +3578,324 @@
       </c>
       <c r="D22" s="33" t="s">
         <v>232</v>
+      </c>
+    </row>
+    <row r="25" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="D25" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="26" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="D26" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="27" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="D27" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="30" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="D30" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="31" spans="3:4" x14ac:dyDescent="0.2">
+      <c r="C31" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="D31" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="34" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="B34" t="s">
+        <v>278</v>
+      </c>
+      <c r="C34" t="s">
+        <v>279</v>
+      </c>
+      <c r="D34" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="35" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="C35" t="s">
+        <v>280</v>
+      </c>
+      <c r="D35" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="36" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="C36" t="s">
+        <v>281</v>
+      </c>
+      <c r="D36" t="s">
+        <v>284</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{49BFEA0E-6634-F449-A731-9A1898A29FC9}">
+  <dimension ref="D2:O24"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="5" max="5" width="13.33203125" customWidth="1"/>
+    <col min="7" max="7" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="50.83203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="4:15" x14ac:dyDescent="0.2">
+      <c r="E2" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="3" spans="4:15" x14ac:dyDescent="0.2">
+      <c r="D3" t="s">
+        <v>270</v>
+      </c>
+      <c r="E3" t="s">
+        <v>183</v>
+      </c>
+      <c r="F3" t="s">
+        <v>6</v>
+      </c>
+      <c r="G3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I3" s="34" t="s">
+        <v>264</v>
+      </c>
+      <c r="J3" s="34"/>
+      <c r="K3" s="34" t="s">
+        <v>263</v>
+      </c>
+      <c r="L3" s="34"/>
+      <c r="M3" s="34"/>
+      <c r="N3" s="34"/>
+      <c r="O3" s="34"/>
+    </row>
+    <row r="4" spans="4:15" x14ac:dyDescent="0.2">
+      <c r="F4" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" t="s">
+        <v>260</v>
+      </c>
+      <c r="I4" t="s">
+        <v>263</v>
+      </c>
+      <c r="K4" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="5" spans="4:15" x14ac:dyDescent="0.2">
+      <c r="F5" t="s">
+        <v>10</v>
+      </c>
+      <c r="G5" t="s">
+        <v>261</v>
+      </c>
+      <c r="I5" s="34" t="s">
+        <v>264</v>
+      </c>
+      <c r="J5" s="34"/>
+      <c r="K5" s="34" t="s">
+        <v>263</v>
+      </c>
+      <c r="L5" s="34"/>
+      <c r="M5" s="34"/>
+      <c r="N5" s="34"/>
+      <c r="O5" s="34"/>
+    </row>
+    <row r="7" spans="4:15" x14ac:dyDescent="0.2">
+      <c r="D7" t="s">
+        <v>259</v>
+      </c>
+      <c r="E7" t="s">
+        <v>184</v>
+      </c>
+      <c r="F7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G7" t="s">
+        <v>128</v>
+      </c>
+      <c r="I7" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="9" spans="4:15" x14ac:dyDescent="0.2">
+      <c r="E9" t="s">
+        <v>271</v>
+      </c>
+      <c r="F9" t="s">
+        <v>4</v>
+      </c>
+      <c r="G9" t="s">
+        <v>7</v>
+      </c>
+      <c r="I9" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="11" spans="4:15" x14ac:dyDescent="0.2">
+      <c r="D11" t="s">
+        <v>274</v>
+      </c>
+      <c r="E11" t="s">
+        <v>185</v>
+      </c>
+      <c r="F11" t="s">
+        <v>6</v>
+      </c>
+      <c r="G11" t="s">
+        <v>7</v>
+      </c>
+      <c r="I11" t="s">
+        <v>273</v>
+      </c>
+      <c r="K11" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="13" spans="4:15" x14ac:dyDescent="0.2">
+      <c r="D13" t="s">
+        <v>32</v>
+      </c>
+      <c r="E13" t="s">
+        <v>183</v>
+      </c>
+      <c r="F13" t="s">
+        <v>6</v>
+      </c>
+      <c r="G13" t="s">
+        <v>46</v>
+      </c>
+      <c r="I13" t="s">
+        <v>277</v>
+      </c>
+      <c r="K13" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="15" spans="4:15" x14ac:dyDescent="0.2">
+      <c r="E15" t="s">
+        <v>275</v>
+      </c>
+      <c r="F15" t="s">
+        <v>0</v>
+      </c>
+      <c r="G15" t="s">
+        <v>7</v>
+      </c>
+      <c r="I15" t="s">
+        <v>277</v>
+      </c>
+      <c r="K15" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="16" spans="4:15" x14ac:dyDescent="0.2">
+      <c r="F16" t="s">
+        <v>2</v>
+      </c>
+      <c r="G16" t="s">
+        <v>128</v>
+      </c>
+      <c r="I16" t="s">
+        <v>277</v>
+      </c>
+      <c r="K16" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="18" spans="4:11" x14ac:dyDescent="0.2">
+      <c r="D18" t="s">
+        <v>193</v>
+      </c>
+      <c r="E18" t="s">
+        <v>192</v>
+      </c>
+      <c r="F18" t="s">
+        <v>6</v>
+      </c>
+      <c r="G18" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="19" spans="4:11" x14ac:dyDescent="0.2">
+      <c r="F19" t="s">
+        <v>8</v>
+      </c>
+      <c r="G19" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="21" spans="4:11" x14ac:dyDescent="0.2">
+      <c r="E21" t="s">
+        <v>176</v>
+      </c>
+      <c r="F21" t="s">
+        <v>10</v>
+      </c>
+      <c r="G21" t="s">
+        <v>7</v>
+      </c>
+      <c r="I21" t="s">
+        <v>290</v>
+      </c>
+      <c r="K21" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="22" spans="4:11" x14ac:dyDescent="0.2">
+      <c r="F22" t="s">
+        <v>286</v>
+      </c>
+      <c r="G22" t="s">
+        <v>7</v>
+      </c>
+      <c r="I22" t="s">
+        <v>290</v>
+      </c>
+      <c r="K22" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="24" spans="4:11" x14ac:dyDescent="0.2">
+      <c r="E24" t="s">
+        <v>285</v>
+      </c>
+      <c r="F24" t="s">
+        <v>2</v>
+      </c>
+      <c r="G24" t="s">
+        <v>287</v>
+      </c>
+      <c r="I24" t="s">
+        <v>290</v>
+      </c>
+      <c r="K24" t="s">
+        <v>290</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Order colours all fixed.
</commit_message>
<xml_diff>
--- a/SUMMARY.xlsx
+++ b/SUMMARY.xlsx
@@ -1405,7 +1405,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M60"/>
-  <sheetFormatPr defaultColWidth="10.609375" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.6015625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="19.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
@@ -2157,7 +2157,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:M120"/>
-  <sheetFormatPr defaultColWidth="10.609375" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.6015625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.83"/>
@@ -3093,14 +3093,14 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A3:J29"/>
-  <sheetFormatPr defaultColWidth="10.609375" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.6015625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="47.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="8"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="20.83"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="76.16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="8.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="8.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="20.17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="21.5"/>
   </cols>
@@ -3346,7 +3346,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:D36"/>
-  <sheetFormatPr defaultColWidth="10.609375" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.6015625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="69.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="21.67"/>
@@ -3413,7 +3413,7 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D9" s="35" t="s">
+      <c r="D9" s="36" t="s">
         <v>242</v>
       </c>
     </row>
@@ -3438,7 +3438,7 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D14" s="35" t="s">
+      <c r="D14" s="36" t="s">
         <v>247</v>
       </c>
     </row>
@@ -3552,11 +3552,11 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="D2:O24"/>
-  <sheetFormatPr defaultColWidth="10.609375" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.6015625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="22.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="50.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="22.82"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="50.82"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Cleaned package information for all scripts
</commit_message>
<xml_diff>
--- a/SUMMARY.xlsx
+++ b/SUMMARY.xlsx
@@ -996,7 +996,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFE699"/>
-        <bgColor rgb="FFFFE994"/>
+        <bgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -1008,7 +1008,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF8FAADC"/>
-        <bgColor rgb="FFCC99FF"/>
+        <bgColor rgb="FFB4C7DC"/>
       </patternFill>
     </fill>
     <fill>
@@ -1044,7 +1044,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFBDD7EE"/>
-        <bgColor rgb="FFDBDBDB"/>
+        <bgColor rgb="FFB4C7DC"/>
       </patternFill>
     </fill>
     <fill>
@@ -1067,8 +1067,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFE994"/>
-        <bgColor rgb="FFFFE699"/>
+        <fgColor rgb="FFB4C7DC"/>
+        <bgColor rgb="FFBDD7EE"/>
       </patternFill>
     </fill>
   </fills>
@@ -1176,7 +1176,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="40">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1322,10 +1322,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="14" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1353,7 +1349,7 @@
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFFFE699"/>
+      <rgbColor rgb="FFC5E0B4"/>
       <rgbColor rgb="FFFF0000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
@@ -1366,7 +1362,7 @@
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFAFD095"/>
+      <rgbColor rgb="FFB4C7DC"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF8FAADC"/>
       <rgbColor rgb="FF993366"/>
@@ -1387,8 +1383,8 @@
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFDBDBDB"/>
       <rgbColor rgb="FFE2F0D9"/>
-      <rgbColor rgb="FFFFE994"/>
-      <rgbColor rgb="FFC5E0B4"/>
+      <rgbColor rgb="FFFFE699"/>
+      <rgbColor rgb="FFAFD095"/>
       <rgbColor rgb="FFF4B183"/>
       <rgbColor rgb="FFCC99FF"/>
       <rgbColor rgb="FFF8CBAD"/>
@@ -1419,7 +1415,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M60"/>
-  <sheetFormatPr defaultColWidth="10.57421875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.56640625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="19.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
@@ -2171,7 +2167,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:M120"/>
-  <sheetFormatPr defaultColWidth="10.57421875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.56640625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="19.83"/>
@@ -3107,7 +3103,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A3:J29"/>
-  <sheetFormatPr defaultColWidth="10.57421875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.56640625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="47.33"/>
@@ -3360,7 +3356,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A2:D36"/>
-  <sheetFormatPr defaultColWidth="10.57421875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.56640625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="69.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="21.67"/>
@@ -3422,10 +3418,10 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="37" t="s">
+      <c r="A8" s="27" t="s">
         <v>241</v>
       </c>
-      <c r="D8" s="38" t="s">
+      <c r="D8" s="37" t="s">
         <v>242</v>
       </c>
     </row>
@@ -3435,7 +3431,7 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D10" s="31" t="s">
+      <c r="D10" s="38" t="s">
         <v>244</v>
       </c>
     </row>
@@ -3455,7 +3451,7 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D14" s="31" t="s">
+      <c r="D14" s="36" t="s">
         <v>248</v>
       </c>
     </row>
@@ -3485,7 +3481,7 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D20" s="39" t="s">
+      <c r="D20" s="36" t="s">
         <v>254</v>
       </c>
     </row>
@@ -3570,7 +3566,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="D2:O24"/>
-  <sheetFormatPr defaultColWidth="10.57421875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.56640625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="13.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="22.81"/>
@@ -3611,14 +3607,14 @@
       <c r="I3" s="0" t="s">
         <v>276</v>
       </c>
-      <c r="J3" s="40"/>
+      <c r="J3" s="39"/>
       <c r="K3" s="0" t="s">
         <v>276</v>
       </c>
-      <c r="L3" s="40"/>
-      <c r="M3" s="40"/>
-      <c r="N3" s="40"/>
-      <c r="O3" s="40"/>
+      <c r="L3" s="39"/>
+      <c r="M3" s="39"/>
+      <c r="N3" s="39"/>
+      <c r="O3" s="39"/>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F4" s="0" t="s">
@@ -3644,14 +3640,14 @@
       <c r="I5" s="0" t="s">
         <v>276</v>
       </c>
-      <c r="J5" s="40"/>
+      <c r="J5" s="39"/>
       <c r="K5" s="0" t="s">
         <v>276</v>
       </c>
-      <c r="L5" s="40"/>
-      <c r="M5" s="40"/>
-      <c r="N5" s="40"/>
-      <c r="O5" s="40"/>
+      <c r="L5" s="39"/>
+      <c r="M5" s="39"/>
+      <c r="N5" s="39"/>
+      <c r="O5" s="39"/>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D7" s="0" t="s">

</xml_diff>